<commit_message>
Lines of code updated for the user_cat, others scenarios
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14410" windowHeight="3410" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14410" windowHeight="2780" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
@@ -12,12 +12,12 @@
     <sheet name="ADD_PET" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:D10"/>
+  <oleSize ref="A1:G7"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="991">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="1017">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -2962,41 +2962,118 @@
     <t>Nexra</t>
   </si>
   <si>
-    <t>Charlie24</t>
-  </si>
-  <si>
-    <t>Milo19</t>
-  </si>
-  <si>
-    <t>Taffy22</t>
-  </si>
-  <si>
-    <t>Cutie14</t>
-  </si>
-  <si>
-    <t>Cinder14</t>
-  </si>
-  <si>
-    <t>pony10</t>
-  </si>
-  <si>
-    <t>fury7</t>
-  </si>
-  <si>
-    <t>Ryder7</t>
-  </si>
-  <si>
-    <t>Rabbit14</t>
-  </si>
-  <si>
-    <t>Sheep13</t>
+    <t>MHYCCP</t>
+  </si>
+  <si>
+    <t>7MAH7R</t>
+  </si>
+  <si>
+    <t>ERYCCD</t>
+  </si>
+  <si>
+    <t>PE6DFR</t>
+  </si>
+  <si>
+    <t>HFKR7H</t>
+  </si>
+  <si>
+    <t>A4RJF7</t>
+  </si>
+  <si>
+    <t>GN6NE4</t>
+  </si>
+  <si>
+    <t>UNYATN</t>
+  </si>
+  <si>
+    <t>EFPAYP</t>
+  </si>
+  <si>
+    <t>PAUHPA</t>
+  </si>
+  <si>
+    <t>MUHDPU</t>
+  </si>
+  <si>
+    <t>TTHFYC</t>
+  </si>
+  <si>
+    <t>JR9TUK</t>
+  </si>
+  <si>
+    <t>PX6PDT</t>
+  </si>
+  <si>
+    <t>VT4KUK</t>
+  </si>
+  <si>
+    <t>VFJEVK</t>
+  </si>
+  <si>
+    <t>MCPKGM</t>
+  </si>
+  <si>
+    <t>KFV7JR</t>
+  </si>
+  <si>
+    <t>9E4R9F</t>
+  </si>
+  <si>
+    <t>UXXEVD</t>
+  </si>
+  <si>
+    <t>DE3VMP</t>
+  </si>
+  <si>
+    <t>YC7CHC</t>
+  </si>
+  <si>
+    <t>HF6RFG</t>
+  </si>
+  <si>
+    <t>NXMMAC</t>
+  </si>
+  <si>
+    <t>G6VTG7</t>
+  </si>
+  <si>
+    <t>JXEFFJ</t>
+  </si>
+  <si>
+    <t>9N77VR</t>
+  </si>
+  <si>
+    <t>FNGKYX</t>
+  </si>
+  <si>
+    <t>UGFMHH</t>
+  </si>
+  <si>
+    <t>VPDVEP</t>
+  </si>
+  <si>
+    <t>REKDKT</t>
+  </si>
+  <si>
+    <t>RARFM9</t>
+  </si>
+  <si>
+    <t>PFMYRN</t>
+  </si>
+  <si>
+    <t>XJUUXF</t>
+  </si>
+  <si>
+    <t>XRMGCJ</t>
+  </si>
+  <si>
+    <t>ER76DX</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3052,7 +3129,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="186">
+  <cellXfs count="265">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -3227,18 +3304,99 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3545,21 +3703,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="17.81640625"/>
-    <col min="2" max="2" customWidth="true" style="1" width="15.0"/>
-    <col min="3" max="3" customWidth="true" style="1" width="15.36328125"/>
-    <col min="4" max="4" customWidth="true" style="1" width="17.453125"/>
-    <col min="5" max="5" customWidth="true" style="1" width="16.6328125"/>
-    <col min="6" max="6" customWidth="true" style="1" width="18.0"/>
-    <col min="7" max="7" customWidth="true" style="1" width="17.26953125"/>
-    <col min="8" max="8" customWidth="true" style="1" width="18.1796875"/>
-    <col min="9" max="9" customWidth="true" style="1" width="18.36328125"/>
-    <col min="10" max="10" customWidth="true" style="1" width="17.453125"/>
-    <col min="11" max="11" customWidth="true" style="1" width="17.36328125"/>
-    <col min="12" max="16384" style="1" width="8.7265625"/>
+    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -3921,13 +4079,13 @@
       <c r="A21" s="97" t="s">
         <v>63</v>
       </c>
-      <c r="B21" s="176" t="s">
+      <c r="B21" s="175" t="s">
         <v>119</v>
       </c>
       <c r="C21" s="75" t="s">
         <v>169</v>
       </c>
-      <c r="D21" s="179" t="s">
+      <c r="D21" s="178" t="s">
         <v>219</v>
       </c>
       <c r="E21" s="24" t="s">
@@ -3938,13 +4096,13 @@
       <c r="A22" s="98" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="186" t="s">
         <v>120</v>
       </c>
       <c r="C22" s="76" t="s">
         <v>170</v>
       </c>
-      <c r="D22" s="180" t="s">
+      <c r="D22" s="179" t="s">
         <v>220</v>
       </c>
       <c r="E22" s="25" t="s">
@@ -3955,13 +4113,13 @@
       <c r="A23" s="107" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="197" t="s">
         <v>121</v>
       </c>
       <c r="C23" s="77" t="s">
         <v>171</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="189" t="s">
         <v>221</v>
       </c>
       <c r="E23" s="26" t="s">
@@ -3972,13 +4130,13 @@
       <c r="A24" s="109" t="s">
         <v>66</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="200" t="s">
         <v>122</v>
       </c>
       <c r="C24" s="78" t="s">
         <v>172</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="190" t="s">
         <v>222</v>
       </c>
       <c r="E24" s="27" t="s">
@@ -3989,13 +4147,13 @@
       <c r="A25" s="124" t="s">
         <v>67</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="203" t="s">
         <v>123</v>
       </c>
       <c r="C25" s="100" t="s">
         <v>173</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="209" t="s">
         <v>223</v>
       </c>
       <c r="E25" s="28" t="s">
@@ -4006,13 +4164,13 @@
       <c r="A26" s="126" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="206" t="s">
         <v>124</v>
       </c>
       <c r="C26" s="110" t="s">
         <v>174</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="210" t="s">
         <v>224</v>
       </c>
       <c r="E26" s="29" t="s">
@@ -4023,13 +4181,13 @@
       <c r="A27" s="127" t="s">
         <v>69</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="218" t="s">
         <v>125</v>
       </c>
       <c r="C27" s="130" t="s">
         <v>175</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="220" t="s">
         <v>225</v>
       </c>
       <c r="E27" s="82" t="s">
@@ -4040,13 +4198,13 @@
       <c r="A28" s="129" t="s">
         <v>70</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="222" t="s">
         <v>126</v>
       </c>
       <c r="C28" s="136" t="s">
         <v>176</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="225" t="s">
         <v>226</v>
       </c>
       <c r="E28" s="83" t="s">
@@ -4057,13 +4215,13 @@
       <c r="A29" s="133" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="231" t="s">
         <v>127</v>
       </c>
       <c r="C29" s="142" t="s">
         <v>177</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="226" t="s">
         <v>227</v>
       </c>
       <c r="E29" s="84" t="s">
@@ -4074,13 +4232,13 @@
       <c r="A30" s="135" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="234" t="s">
         <v>128</v>
       </c>
       <c r="C30" s="152" t="s">
         <v>178</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="237" t="s">
         <v>228</v>
       </c>
       <c r="E30" s="85" t="s">
@@ -4091,13 +4249,13 @@
       <c r="A31" s="139" t="s">
         <v>73</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="244" t="s">
         <v>129</v>
       </c>
       <c r="C31" s="162" t="s">
         <v>179</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D31" s="238" t="s">
         <v>229</v>
       </c>
       <c r="E31" s="86" t="s">
@@ -4108,13 +4266,13 @@
       <c r="A32" s="141" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="255" t="s">
         <v>130</v>
       </c>
-      <c r="C32" s="178" t="s">
+      <c r="C32" s="177" t="s">
         <v>180</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D32" s="247" t="s">
         <v>230</v>
       </c>
       <c r="E32" s="87" t="s">
@@ -4128,10 +4286,10 @@
       <c r="B33" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="188" t="s">
         <v>181</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" s="248" t="s">
         <v>231</v>
       </c>
       <c r="E33" s="88" t="s">
@@ -4145,10 +4303,10 @@
       <c r="B34" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="208" t="s">
         <v>182</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D34" s="258" t="s">
         <v>232</v>
       </c>
       <c r="E34" s="89" t="s">
@@ -4162,10 +4320,10 @@
       <c r="B35" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="224" t="s">
         <v>183</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="D35" s="259" t="s">
         <v>233</v>
       </c>
       <c r="E35" s="90" t="s">
@@ -4179,7 +4337,7 @@
       <c r="B36" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="236" t="s">
         <v>184</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -4196,7 +4354,7 @@
       <c r="B37" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="246" t="s">
         <v>185</v>
       </c>
       <c r="D37" s="1" t="s">
@@ -4207,13 +4365,13 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="175" t="s">
+      <c r="A38" s="174" t="s">
         <v>80</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="257" t="s">
         <v>186</v>
       </c>
       <c r="D38" s="1" t="s">
@@ -4224,7 +4382,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="177" t="s">
+      <c r="A39" s="176" t="s">
         <v>81</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -4241,7 +4399,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" s="1" t="s">
+      <c r="A40" s="185" t="s">
         <v>82</v>
       </c>
       <c r="B40" s="1" t="s">
@@ -4258,7 +4416,7 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" s="1" t="s">
+      <c r="A41" s="187" t="s">
         <v>83</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -4275,7 +4433,7 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="196" t="s">
         <v>84</v>
       </c>
       <c r="B42" s="1" t="s">
@@ -4292,7 +4450,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" s="1" t="s">
+      <c r="A43" s="198" t="s">
         <v>85</v>
       </c>
       <c r="B43" s="1" t="s">
@@ -4309,7 +4467,7 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" s="1" t="s">
+      <c r="A44" s="199" t="s">
         <v>86</v>
       </c>
       <c r="B44" s="1" t="s">
@@ -4326,7 +4484,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" s="1" t="s">
+      <c r="A45" s="201" t="s">
         <v>87</v>
       </c>
       <c r="B45" s="1" t="s">
@@ -4343,7 +4501,7 @@
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" s="1" t="s">
+      <c r="A46" s="202" t="s">
         <v>88</v>
       </c>
       <c r="B46" s="1" t="s">
@@ -4360,7 +4518,7 @@
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" s="1" t="s">
+      <c r="A47" s="204" t="s">
         <v>89</v>
       </c>
       <c r="B47" s="1" t="s">
@@ -4377,7 +4535,7 @@
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="1" t="s">
+      <c r="A48" s="205" t="s">
         <v>90</v>
       </c>
       <c r="B48" s="1" t="s">
@@ -4391,7 +4549,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="1" t="s">
+      <c r="A49" s="207" t="s">
         <v>91</v>
       </c>
       <c r="B49" s="1" t="s">
@@ -4405,7 +4563,7 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="1" t="s">
+      <c r="A50" s="216" t="s">
         <v>92</v>
       </c>
       <c r="B50" s="1" t="s">
@@ -4419,7 +4577,7 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="1" t="s">
+      <c r="A51" s="219" t="s">
         <v>93</v>
       </c>
       <c r="B51" s="1" t="s">
@@ -4433,7 +4591,7 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="1" t="s">
+      <c r="A52" s="221" t="s">
         <v>94</v>
       </c>
       <c r="E52" s="121" t="s">
@@ -4441,7 +4599,7 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" s="1" t="s">
+      <c r="A53" s="223" t="s">
         <v>95</v>
       </c>
       <c r="E53" s="122" t="s">
@@ -4449,7 +4607,7 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" s="1" t="s">
+      <c r="A54" s="230" t="s">
         <v>96</v>
       </c>
       <c r="E54" s="123" t="s">
@@ -4457,7 +4615,7 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A55" s="1" t="s">
+      <c r="A55" s="232" t="s">
         <v>97</v>
       </c>
       <c r="E55" s="145" t="s">
@@ -4465,7 +4623,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A56" s="1" t="s">
+      <c r="A56" s="233" t="s">
         <v>98</v>
       </c>
       <c r="E56" s="146" t="s">
@@ -4473,7 +4631,7 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A57" s="1" t="s">
+      <c r="A57" s="235" t="s">
         <v>99</v>
       </c>
       <c r="E57" s="155" t="s">
@@ -4481,98 +4639,260 @@
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" s="243" t="s">
+        <v>1007</v>
+      </c>
       <c r="E58" s="156" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" s="245" t="s">
+        <v>1008</v>
+      </c>
       <c r="E59" s="157" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" s="254" t="s">
+        <v>1009</v>
+      </c>
       <c r="E60" s="158" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" s="256" t="s">
+        <v>1010</v>
+      </c>
       <c r="E61" s="165" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" s="170" t="s">
+        <v>1011</v>
+      </c>
       <c r="E62" s="166" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" s="170" t="s">
+        <v>1012</v>
+      </c>
       <c r="E63" s="167" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64" s="170" t="s">
+        <v>1013</v>
+      </c>
       <c r="E64" s="168" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="65" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E65" s="182" t="s">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A65" s="170" t="s">
+        <v>1014</v>
+      </c>
+      <c r="E65" s="181" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="66" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E66" s="183" t="s">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A66" s="170" t="s">
+        <v>1015</v>
+      </c>
+      <c r="E66" s="182" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="67" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E67" s="184" t="s">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A67" s="170" t="s">
+        <v>1016</v>
+      </c>
+      <c r="E67" s="183" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="68" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E68" s="185" t="s">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E68" s="184" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="69" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E69" s="1" t="s">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E69" s="192" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="70" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E70" s="1" t="s">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E70" s="193" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="71" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E71" s="1" t="s">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E71" s="194" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="72" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E72" s="1" t="s">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E72" s="195" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="73" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E73" s="1" t="s">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E73" s="212" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="74" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E74" s="1" t="s">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E74" s="213" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="75" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E75" s="1" t="s">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E75" s="214" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="76" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E76" s="1" t="s">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E76" s="215" t="s">
         <v>295</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E77" s="228" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E78" s="229" t="s">
+        <v>983</v>
+      </c>
+      <c r="F78" s="217"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E79" s="240" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E80" s="241" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="81" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E81" s="242" t="s">
+        <v>985</v>
+      </c>
+      <c r="F81" s="217"/>
+    </row>
+    <row r="82" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E82" s="250" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="83" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E83" s="251" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="84" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E84" s="252" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="85" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E85" s="253" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="86" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E86" s="261" t="s">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="87" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E87" s="262" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="88" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E88" s="263" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="89" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E89" s="264" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="90" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E90" s="170" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="91" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E91" s="170" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="92" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E92" s="170" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="93" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E93" s="170" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="94" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E94" s="170" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="95" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E95" s="170" t="s">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="96" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E96" s="170" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="97" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E97" s="170" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="98" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E98" s="170" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="99" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E99" s="170" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="100" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E100" s="170" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="101" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E101" s="170" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="102" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E102" s="170" t="s">
+        <v>1006</v>
       </c>
     </row>
   </sheetData>
@@ -4586,90 +4906,87 @@
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="26.90625"/>
-    <col min="2" max="2" customWidth="true" width="29.453125"/>
-    <col min="3" max="3" customWidth="true" width="35.6328125"/>
-    <col min="4" max="4" customWidth="true" width="30.90625"/>
-    <col min="5" max="5" customWidth="true" width="32.7265625"/>
-    <col min="6" max="6" customWidth="true" width="32.1796875"/>
-    <col min="7" max="7" customWidth="true" width="33.6328125"/>
-    <col min="8" max="8" customWidth="true" width="31.26953125"/>
+    <col min="1" max="1" width="26.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" customWidth="1"/>
+    <col min="4" max="4" width="30.90625" customWidth="1"/>
+    <col min="5" max="5" width="32.7265625" customWidth="1"/>
+    <col min="6" max="6" width="32.1796875" customWidth="1"/>
+    <col min="7" max="7" width="33.6328125" customWidth="1"/>
+    <col min="8" max="8" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>16</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>29</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>29</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>29</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>29</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>29</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>29</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>988</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35"/>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35"/>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D7" t="s" s="0">
+      <c r="D7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D8" t="s" s="0">
+      <c r="D8" t="s">
         <v>29</v>
       </c>
     </row>
@@ -4690,41 +5007,41 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:I201"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.08984375"/>
-    <col min="2" max="2" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" customWidth="true" width="17.36328125"/>
-    <col min="4" max="5" customWidth="true" width="17.26953125"/>
-    <col min="6" max="6" customWidth="true" width="17.1796875"/>
-    <col min="7" max="7" customWidth="true" width="15.36328125"/>
-    <col min="8" max="8" customWidth="true" width="17.1796875"/>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="4" max="5" width="17.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="169" t="s">
         <v>296</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>297</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>298</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>299</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>300</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>301</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>302</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>303</v>
       </c>
     </row>
@@ -4749,7 +5066,7 @@
       <c r="B3" s="170" t="s">
         <v>625</v>
       </c>
-      <c r="C3" s="181" t="s">
+      <c r="C3" s="180" t="s">
         <v>305</v>
       </c>
       <c r="D3" s="173" t="s">
@@ -4763,7 +5080,7 @@
       <c r="B4" s="170" t="s">
         <v>626</v>
       </c>
-      <c r="C4" s="172" t="s">
+      <c r="C4" s="191" t="s">
         <v>306</v>
       </c>
       <c r="D4" s="173" t="s">
@@ -4777,7 +5094,7 @@
       <c r="B5" s="170" t="s">
         <v>627</v>
       </c>
-      <c r="C5" s="172" t="s">
+      <c r="C5" s="211" t="s">
         <v>307</v>
       </c>
       <c r="D5" s="173" t="s">
@@ -4791,7 +5108,7 @@
       <c r="B6" s="170" t="s">
         <v>628</v>
       </c>
-      <c r="C6" s="172" t="s">
+      <c r="C6" s="227" t="s">
         <v>308</v>
       </c>
       <c r="D6" s="173" t="s">
@@ -4805,7 +5122,7 @@
       <c r="B7" s="170" t="s">
         <v>629</v>
       </c>
-      <c r="C7" s="172" t="s">
+      <c r="C7" s="239" t="s">
         <v>309</v>
       </c>
       <c r="D7" s="173" t="s">
@@ -4819,7 +5136,7 @@
       <c r="B8" s="170" t="s">
         <v>630</v>
       </c>
-      <c r="C8" s="172" t="s">
+      <c r="C8" s="249" t="s">
         <v>310</v>
       </c>
       <c r="D8" s="173" t="s">
@@ -4833,7 +5150,7 @@
       <c r="B9" s="170" t="s">
         <v>631</v>
       </c>
-      <c r="C9" s="172" t="s">
+      <c r="C9" s="260" t="s">
         <v>311</v>
       </c>
       <c r="D9" s="173" t="s">

</xml_diff>

<commit_message>
Lines of code updated for user_horse,cat
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14410" windowHeight="2780" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13970" windowHeight="2690" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
@@ -12,12 +12,12 @@
     <sheet name="ADD_PET" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:G7"/>
+  <oleSize ref="A1:D7"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="1017">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="1033">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -3068,12 +3068,61 @@
   </si>
   <si>
     <t>ER76DX</t>
+  </si>
+  <si>
+    <t>YFTAXD</t>
+  </si>
+  <si>
+    <t>ECGUPJ</t>
+  </si>
+  <si>
+    <t>JRTJR7</t>
+  </si>
+  <si>
+    <t>KU4K7D</t>
+  </si>
+  <si>
+    <t>G4RJEA</t>
+  </si>
+  <si>
+    <t>NKEGFM</t>
+  </si>
+  <si>
+    <t>JVXX6F</t>
+  </si>
+  <si>
+    <t>39YTKH</t>
+  </si>
+  <si>
+    <t>DFTJEP</t>
+  </si>
+  <si>
+    <t>Charlie48</t>
+  </si>
+  <si>
+    <t>Milo39</t>
+  </si>
+  <si>
+    <t>Taffy37</t>
+  </si>
+  <si>
+    <t>Cutie26</t>
+  </si>
+  <si>
+    <t>Cinder26</t>
+  </si>
+  <si>
+    <t>pony19</t>
+  </si>
+  <si>
+    <t>fury18</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3129,7 +3178,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="265">
+  <cellXfs count="301">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -3397,6 +3446,42 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3703,21 +3788,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K102"/>
+  <dimension ref="A1:J102"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" customWidth="true" style="1" width="17.81640625"/>
+    <col min="2" max="2" customWidth="true" style="1" width="15.0"/>
+    <col min="3" max="3" customWidth="true" style="1" width="15.36328125"/>
+    <col min="4" max="4" customWidth="true" style="1" width="17.453125"/>
+    <col min="5" max="5" customWidth="true" style="1" width="16.6328125"/>
+    <col min="6" max="6" customWidth="true" style="1" width="18.0"/>
+    <col min="7" max="7" customWidth="true" style="1" width="17.26953125"/>
+    <col min="8" max="8" customWidth="true" style="1" width="18.1796875"/>
+    <col min="9" max="9" customWidth="true" style="1" width="18.36328125"/>
+    <col min="10" max="10" customWidth="true" style="1" width="17.453125"/>
+    <col min="11" max="11" customWidth="true" style="1" width="17.36328125"/>
+    <col min="12" max="16384" style="1" width="8.7265625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -4283,7 +4368,7 @@
       <c r="A33" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="266" t="s">
         <v>131</v>
       </c>
       <c r="C33" s="188" t="s">
@@ -4300,7 +4385,7 @@
       <c r="A34" s="149" t="s">
         <v>76</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="275" t="s">
         <v>132</v>
       </c>
       <c r="C34" s="208" t="s">
@@ -4317,7 +4402,7 @@
       <c r="A35" s="151" t="s">
         <v>77</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="284" t="s">
         <v>133</v>
       </c>
       <c r="C35" s="224" t="s">
@@ -4334,13 +4419,13 @@
       <c r="A36" s="159" t="s">
         <v>78</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="293" t="s">
         <v>134</v>
       </c>
       <c r="C36" s="236" t="s">
         <v>184</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D36" s="269" t="s">
         <v>234</v>
       </c>
       <c r="E36" s="91" t="s">
@@ -4357,7 +4442,7 @@
       <c r="C37" s="246" t="s">
         <v>185</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" s="270" t="s">
         <v>235</v>
       </c>
       <c r="E37" s="92" t="s">
@@ -4374,7 +4459,7 @@
       <c r="C38" s="257" t="s">
         <v>186</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" s="278" t="s">
         <v>236</v>
       </c>
       <c r="E38" s="93" t="s">
@@ -4388,10 +4473,10 @@
       <c r="B39" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="268" t="s">
         <v>187</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D39" s="279" t="s">
         <v>237</v>
       </c>
       <c r="E39" s="94" t="s">
@@ -4405,10 +4490,10 @@
       <c r="B40" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="277" t="s">
         <v>188</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D40" s="287" t="s">
         <v>238</v>
       </c>
       <c r="E40" s="103" t="s">
@@ -4422,10 +4507,10 @@
       <c r="B41" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" s="286" t="s">
         <v>189</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D41" s="288" t="s">
         <v>239</v>
       </c>
       <c r="E41" s="104" t="s">
@@ -4439,10 +4524,10 @@
       <c r="B42" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="295" t="s">
         <v>190</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D42" s="296" t="s">
         <v>240</v>
       </c>
       <c r="E42" s="105" t="s">
@@ -4459,7 +4544,7 @@
       <c r="C43" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D43" s="297" t="s">
         <v>241</v>
       </c>
       <c r="E43" s="106" t="s">
@@ -4671,7 +4756,7 @@
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A62" s="170" t="s">
+      <c r="A62" s="265" t="s">
         <v>1011</v>
       </c>
       <c r="E62" s="166" t="s">
@@ -4679,7 +4764,7 @@
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A63" s="170" t="s">
+      <c r="A63" s="267" t="s">
         <v>1012</v>
       </c>
       <c r="E63" s="167" t="s">
@@ -4687,7 +4772,7 @@
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A64" s="170" t="s">
+      <c r="A64" s="274" t="s">
         <v>1013</v>
       </c>
       <c r="E64" s="168" t="s">
@@ -4695,7 +4780,7 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A65" s="170" t="s">
+      <c r="A65" s="276" t="s">
         <v>1014</v>
       </c>
       <c r="E65" s="181" t="s">
@@ -4703,7 +4788,7 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A66" s="170" t="s">
+      <c r="A66" s="283" t="s">
         <v>1015</v>
       </c>
       <c r="E66" s="182" t="s">
@@ -4711,7 +4796,7 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A67" s="170" t="s">
+      <c r="A67" s="285" t="s">
         <v>1016</v>
       </c>
       <c r="E67" s="183" t="s">
@@ -4719,46 +4804,73 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A68" s="292" t="s">
+        <v>1017</v>
+      </c>
       <c r="E68" s="184" t="s">
         <v>287</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A69" s="294" t="s">
+        <v>1018</v>
+      </c>
       <c r="E69" s="192" t="s">
         <v>288</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70" s="1" t="s">
+        <v>1019</v>
+      </c>
       <c r="E70" s="193" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
+        <v>1020</v>
+      </c>
       <c r="E71" s="194" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A72" s="1" t="s">
+        <v>1021</v>
+      </c>
       <c r="E72" s="195" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
+        <v>1022</v>
+      </c>
       <c r="E73" s="212" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A74" s="1" t="s">
+        <v>1023</v>
+      </c>
       <c r="E74" s="213" t="s">
         <v>293</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A75" s="1" t="s">
+        <v>1024</v>
+      </c>
       <c r="E75" s="214" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A76" s="1" t="s">
+        <v>1025</v>
+      </c>
       <c r="E76" s="215" t="s">
         <v>295</v>
       </c>
@@ -4831,42 +4943,42 @@
       </c>
     </row>
     <row r="90" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E90" s="170" t="s">
+      <c r="E90" s="272" t="s">
         <v>994</v>
       </c>
     </row>
     <row r="91" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E91" s="170" t="s">
+      <c r="E91" s="273" t="s">
         <v>995</v>
       </c>
     </row>
     <row r="92" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E92" s="170" t="s">
+      <c r="E92" s="281" t="s">
         <v>996</v>
       </c>
     </row>
     <row r="93" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E93" s="170" t="s">
+      <c r="E93" s="282" t="s">
         <v>997</v>
       </c>
     </row>
     <row r="94" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E94" s="170" t="s">
+      <c r="E94" s="290" t="s">
         <v>998</v>
       </c>
     </row>
     <row r="95" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E95" s="170" t="s">
+      <c r="E95" s="291" t="s">
         <v>999</v>
       </c>
     </row>
     <row r="96" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E96" s="170" t="s">
+      <c r="E96" s="299" t="s">
         <v>1000</v>
       </c>
     </row>
     <row r="97" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E97" s="170" t="s">
+      <c r="E97" s="300" t="s">
         <v>1001</v>
       </c>
     </row>
@@ -4906,90 +5018,87 @@
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.90625" customWidth="1"/>
-    <col min="2" max="2" width="29.453125" customWidth="1"/>
-    <col min="3" max="3" width="35.6328125" customWidth="1"/>
-    <col min="4" max="4" width="30.90625" customWidth="1"/>
-    <col min="5" max="5" width="32.7265625" customWidth="1"/>
-    <col min="6" max="6" width="32.1796875" customWidth="1"/>
-    <col min="7" max="7" width="33.6328125" customWidth="1"/>
-    <col min="8" max="8" width="31.26953125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="26.90625"/>
+    <col min="2" max="2" customWidth="true" width="29.453125"/>
+    <col min="3" max="3" customWidth="true" width="35.6328125"/>
+    <col min="4" max="4" customWidth="true" width="30.90625"/>
+    <col min="5" max="5" customWidth="true" width="32.7265625"/>
+    <col min="6" max="6" customWidth="true" width="32.1796875"/>
+    <col min="7" max="7" customWidth="true" width="33.6328125"/>
+    <col min="8" max="8" customWidth="true" width="31.26953125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>11</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s" s="0">
         <v>29</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="B4" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D5" t="s" s="0">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35"/>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D7" t="s">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D6" t="s" s="0">
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35"/>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35"/>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35"/>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35"/>
@@ -5002,46 +5111,47 @@
     <row r="18" spans="1:4" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I201"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.08984375" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" customWidth="1"/>
-    <col min="3" max="3" width="17.36328125" customWidth="1"/>
-    <col min="4" max="5" width="17.26953125" customWidth="1"/>
-    <col min="6" max="6" width="17.1796875" customWidth="1"/>
-    <col min="7" max="7" width="15.36328125" customWidth="1"/>
-    <col min="8" max="8" width="17.1796875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="20.08984375"/>
+    <col min="2" max="2" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" customWidth="true" width="17.36328125"/>
+    <col min="4" max="5" customWidth="true" width="17.26953125"/>
+    <col min="6" max="6" customWidth="true" width="17.1796875"/>
+    <col min="7" max="7" customWidth="true" width="15.36328125"/>
+    <col min="8" max="8" customWidth="true" width="17.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="169" t="s">
         <v>296</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>297</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>298</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>299</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>300</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>301</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>302</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>303</v>
       </c>
     </row>
@@ -5164,7 +5274,7 @@
       <c r="B10" s="170" t="s">
         <v>632</v>
       </c>
-      <c r="C10" s="172" t="s">
+      <c r="C10" s="271" t="s">
         <v>312</v>
       </c>
       <c r="D10" s="173" t="s">
@@ -5178,7 +5288,7 @@
       <c r="B11" s="170" t="s">
         <v>633</v>
       </c>
-      <c r="C11" s="172" t="s">
+      <c r="C11" s="280" t="s">
         <v>313</v>
       </c>
       <c r="D11" s="173" t="s">
@@ -5192,7 +5302,7 @@
       <c r="B12" s="170" t="s">
         <v>634</v>
       </c>
-      <c r="C12" s="172" t="s">
+      <c r="C12" s="289" t="s">
         <v>314</v>
       </c>
       <c r="D12" s="173" t="s">
@@ -5206,7 +5316,7 @@
       <c r="B13" s="170" t="s">
         <v>635</v>
       </c>
-      <c r="C13" s="172" t="s">
+      <c r="C13" s="298" t="s">
         <v>315</v>
       </c>
       <c r="D13" s="173" t="s">

</xml_diff>

<commit_message>
Updated the lines of code for the excelutil class and updated the petname counter file
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13970" windowHeight="2690" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14020" windowHeight="6080"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
@@ -12,12 +12,12 @@
     <sheet name="ADD_PET" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:D7"/>
+  <oleSize ref="A34:G51"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="1033">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="1045">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -3097,32 +3097,67 @@
     <t>DFTJEP</t>
   </si>
   <si>
-    <t>Charlie48</t>
-  </si>
-  <si>
-    <t>Milo39</t>
-  </si>
-  <si>
-    <t>Taffy37</t>
-  </si>
-  <si>
-    <t>Cutie26</t>
-  </si>
-  <si>
-    <t>Cinder26</t>
-  </si>
-  <si>
-    <t>pony19</t>
-  </si>
-  <si>
-    <t>fury18</t>
+    <t>XMNYRP</t>
+  </si>
+  <si>
+    <t>DGRAVD</t>
+  </si>
+  <si>
+    <t>MGPXCA</t>
+  </si>
+  <si>
+    <t>GCHR9P</t>
+  </si>
+  <si>
+    <t>HANTAF</t>
+  </si>
+  <si>
+    <t>UCXJPU</t>
+  </si>
+  <si>
+    <t>3HTVRG</t>
+  </si>
+  <si>
+    <t>EAUVNA</t>
+  </si>
+  <si>
+    <t>XACPDY</t>
+  </si>
+  <si>
+    <t>EXRTGT</t>
+  </si>
+  <si>
+    <t>F9JDEF</t>
+  </si>
+  <si>
+    <t>CADMX6</t>
+  </si>
+  <si>
+    <t>H4NC3U</t>
+  </si>
+  <si>
+    <t>NHM4VX</t>
+  </si>
+  <si>
+    <t>JYCTNK</t>
+  </si>
+  <si>
+    <t>AXKHEA</t>
+  </si>
+  <si>
+    <t>7UYNC7</t>
+  </si>
+  <si>
+    <t>TUCEPN</t>
+  </si>
+  <si>
+    <t>NDCUX3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3178,7 +3213,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="301">
+  <cellXfs count="312">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -3473,15 +3508,26 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3788,21 +3834,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J102"/>
+  <dimension ref="A1:K109"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="17.81640625"/>
-    <col min="2" max="2" customWidth="true" style="1" width="15.0"/>
-    <col min="3" max="3" customWidth="true" style="1" width="15.36328125"/>
-    <col min="4" max="4" customWidth="true" style="1" width="17.453125"/>
-    <col min="5" max="5" customWidth="true" style="1" width="16.6328125"/>
-    <col min="6" max="6" customWidth="true" style="1" width="18.0"/>
-    <col min="7" max="7" customWidth="true" style="1" width="17.26953125"/>
-    <col min="8" max="8" customWidth="true" style="1" width="18.1796875"/>
-    <col min="9" max="9" customWidth="true" style="1" width="18.36328125"/>
-    <col min="10" max="10" customWidth="true" style="1" width="17.453125"/>
-    <col min="11" max="11" customWidth="true" style="1" width="17.36328125"/>
-    <col min="12" max="16384" style="1" width="8.7265625"/>
+    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -4436,7 +4482,7 @@
       <c r="A37" s="161" t="s">
         <v>79</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="302" t="s">
         <v>135</v>
       </c>
       <c r="C37" s="246" t="s">
@@ -4541,7 +4587,7 @@
       <c r="B43" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" s="304" t="s">
         <v>191</v>
       </c>
       <c r="D43" s="297" t="s">
@@ -4561,7 +4607,7 @@
       <c r="C44" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D44" s="305" t="s">
         <v>242</v>
       </c>
       <c r="E44" s="113" t="s">
@@ -4578,7 +4624,7 @@
       <c r="C45" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="D45" s="306" t="s">
         <v>243</v>
       </c>
       <c r="E45" s="114" t="s">
@@ -4629,6 +4675,9 @@
       <c r="C48" s="1" t="s">
         <v>196</v>
       </c>
+      <c r="D48" s="170" t="s">
+        <v>1039</v>
+      </c>
       <c r="E48" s="117" t="s">
         <v>267</v>
       </c>
@@ -4643,6 +4692,9 @@
       <c r="C49" s="1" t="s">
         <v>197</v>
       </c>
+      <c r="D49" s="170" t="s">
+        <v>1040</v>
+      </c>
       <c r="E49" s="118" t="s">
         <v>268</v>
       </c>
@@ -4657,6 +4709,9 @@
       <c r="C50" s="1" t="s">
         <v>198</v>
       </c>
+      <c r="D50" s="170" t="s">
+        <v>1041</v>
+      </c>
       <c r="E50" s="119" t="s">
         <v>269</v>
       </c>
@@ -4671,6 +4726,9 @@
       <c r="C51" s="1" t="s">
         <v>199</v>
       </c>
+      <c r="D51" s="170" t="s">
+        <v>1042</v>
+      </c>
       <c r="E51" s="120" t="s">
         <v>270</v>
       </c>
@@ -4679,6 +4737,9 @@
       <c r="A52" s="221" t="s">
         <v>94</v>
       </c>
+      <c r="D52" s="170" t="s">
+        <v>1043</v>
+      </c>
       <c r="E52" s="121" t="s">
         <v>271</v>
       </c>
@@ -4687,6 +4748,9 @@
       <c r="A53" s="223" t="s">
         <v>95</v>
       </c>
+      <c r="D53" s="170" t="s">
+        <v>1044</v>
+      </c>
       <c r="E53" s="122" t="s">
         <v>272</v>
       </c>
@@ -4820,7 +4884,7 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A70" s="1" t="s">
+      <c r="A70" s="301" t="s">
         <v>1019</v>
       </c>
       <c r="E70" s="193" t="s">
@@ -4828,7 +4892,7 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A71" s="1" t="s">
+      <c r="A71" s="303" t="s">
         <v>1020</v>
       </c>
       <c r="E71" s="194" t="s">
@@ -4876,103 +4940,121 @@
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A77" s="170" t="s">
+        <v>1026</v>
+      </c>
       <c r="E77" s="228" t="s">
         <v>981</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A78" s="170" t="s">
+        <v>1027</v>
+      </c>
       <c r="E78" s="229" t="s">
         <v>983</v>
       </c>
       <c r="F78" s="217"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" s="170" t="s">
+        <v>1028</v>
+      </c>
       <c r="E79" s="240" t="s">
         <v>982</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A80" s="170" t="s">
+        <v>1029</v>
+      </c>
       <c r="E80" s="241" t="s">
         <v>984</v>
       </c>
     </row>
-    <row r="81" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A81" s="170" t="s">
+        <v>1030</v>
+      </c>
       <c r="E81" s="242" t="s">
         <v>985</v>
       </c>
       <c r="F81" s="217"/>
     </row>
-    <row r="82" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A82" s="170" t="s">
+        <v>1031</v>
+      </c>
       <c r="E82" s="250" t="s">
         <v>986</v>
       </c>
     </row>
-    <row r="83" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E83" s="251" t="s">
         <v>987</v>
       </c>
     </row>
-    <row r="84" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E84" s="252" t="s">
         <v>988</v>
       </c>
     </row>
-    <row r="85" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E85" s="253" t="s">
         <v>989</v>
       </c>
     </row>
-    <row r="86" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E86" s="261" t="s">
         <v>990</v>
       </c>
     </row>
-    <row r="87" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E87" s="262" t="s">
         <v>991</v>
       </c>
     </row>
-    <row r="88" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E88" s="263" t="s">
         <v>992</v>
       </c>
     </row>
-    <row r="89" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E89" s="264" t="s">
         <v>993</v>
       </c>
     </row>
-    <row r="90" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E90" s="272" t="s">
         <v>994</v>
       </c>
     </row>
-    <row r="91" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E91" s="273" t="s">
         <v>995</v>
       </c>
     </row>
-    <row r="92" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E92" s="281" t="s">
         <v>996</v>
       </c>
     </row>
-    <row r="93" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E93" s="282" t="s">
         <v>997</v>
       </c>
     </row>
-    <row r="94" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E94" s="290" t="s">
         <v>998</v>
       </c>
     </row>
-    <row r="95" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E95" s="291" t="s">
         <v>999</v>
       </c>
     </row>
-    <row r="96" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E96" s="299" t="s">
         <v>1000</v>
       </c>
@@ -4983,28 +5065,63 @@
       </c>
     </row>
     <row r="98" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E98" s="170" t="s">
+      <c r="E98" s="308" t="s">
         <v>1002</v>
       </c>
     </row>
     <row r="99" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E99" s="170" t="s">
+      <c r="E99" s="309" t="s">
         <v>1003</v>
       </c>
     </row>
     <row r="100" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E100" s="170" t="s">
+      <c r="E100" s="310" t="s">
         <v>1004</v>
       </c>
     </row>
     <row r="101" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E101" s="170" t="s">
+      <c r="E101" s="311" t="s">
         <v>1005</v>
       </c>
     </row>
     <row r="102" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E102" s="170" t="s">
         <v>1006</v>
+      </c>
+    </row>
+    <row r="103" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E103" s="170" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="104" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E104" s="170" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="105" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E105" s="170" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="106" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E106" s="170" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="107" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E107" s="170" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="108" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E108" s="170" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="109" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E109" s="170" t="s">
+        <v>1038</v>
       </c>
     </row>
   </sheetData>
@@ -5018,82 +5135,85 @@
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="26.90625"/>
-    <col min="2" max="2" customWidth="true" width="29.453125"/>
-    <col min="3" max="3" customWidth="true" width="35.6328125"/>
-    <col min="4" max="4" customWidth="true" width="30.90625"/>
-    <col min="5" max="5" customWidth="true" width="32.7265625"/>
-    <col min="6" max="6" customWidth="true" width="32.1796875"/>
-    <col min="7" max="7" customWidth="true" width="33.6328125"/>
-    <col min="8" max="8" customWidth="true" width="31.26953125"/>
+    <col min="1" max="1" width="26.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" customWidth="1"/>
+    <col min="4" max="4" width="30.90625" customWidth="1"/>
+    <col min="5" max="5" width="32.7265625" customWidth="1"/>
+    <col min="6" max="6" width="32.1796875" customWidth="1"/>
+    <col min="7" max="7" width="33.6328125" customWidth="1"/>
+    <col min="8" max="8" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>16</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>29</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>29</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>29</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>29</v>
       </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>29</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D5" t="s" s="0">
+      <c r="D5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D6" t="s" s="0">
+      <c r="D6" t="s">
         <v>29</v>
       </c>
     </row>
@@ -5117,41 +5237,41 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:I201"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.08984375"/>
-    <col min="2" max="2" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" customWidth="true" width="17.36328125"/>
-    <col min="4" max="5" customWidth="true" width="17.26953125"/>
-    <col min="6" max="6" customWidth="true" width="17.1796875"/>
-    <col min="7" max="7" customWidth="true" width="15.36328125"/>
-    <col min="8" max="8" customWidth="true" width="17.1796875"/>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="4" max="5" width="17.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="169" t="s">
         <v>296</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>297</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>298</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>299</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>300</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>301</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>302</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>303</v>
       </c>
     </row>
@@ -5330,7 +5450,7 @@
       <c r="B14" s="170" t="s">
         <v>636</v>
       </c>
-      <c r="C14" s="172" t="s">
+      <c r="C14" s="307" t="s">
         <v>316</v>
       </c>
       <c r="D14" s="173" t="s">

</xml_diff>

<commit_message>
user_dog gut samples updated
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14020" windowHeight="6080"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14020" windowHeight="4810"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="1045">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="1047">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -3152,6 +3152,12 @@
   </si>
   <si>
     <t>NDCUX3</t>
+  </si>
+  <si>
+    <t>Charlie54</t>
+  </si>
+  <si>
+    <t>Charlie55</t>
   </si>
 </sst>
 </file>
@@ -3181,7 +3187,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3196,6 +3202,12 @@
     <fill>
       <patternFill patternType="none">
         <fgColor indexed="13"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -3213,7 +3225,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="312">
+  <cellXfs count="313">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -3528,6 +3540,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4900,7 +4913,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A72" s="1" t="s">
+      <c r="A72" s="312" t="s">
         <v>1021</v>
       </c>
       <c r="E72" s="195" t="s">
@@ -4908,7 +4921,7 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A73" s="1" t="s">
+      <c r="A73" s="312" t="s">
         <v>1022</v>
       </c>
       <c r="E73" s="212" t="s">
@@ -4916,7 +4929,7 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A74" s="1" t="s">
+      <c r="A74" s="312" t="s">
         <v>1023</v>
       </c>
       <c r="E74" s="213" t="s">
@@ -5173,7 +5186,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>1045</v>
       </c>
       <c r="B2" t="s">
         <v>29</v>
@@ -5187,7 +5200,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>1046</v>
       </c>
       <c r="B3" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
Commited from Jenkins Server
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="1047">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="1053">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -3158,12 +3158,31 @@
   </si>
   <si>
     <t>Charlie55</t>
+  </si>
+  <si>
+    <t>Charlie61</t>
+  </si>
+  <si>
+    <t>Milo44</t>
+  </si>
+  <si>
+    <t>Taffy42</t>
+  </si>
+  <si>
+    <t>Cutie30</t>
+  </si>
+  <si>
+    <t>Cinder30</t>
+  </si>
+  <si>
+    <t>pony23</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3225,7 +3244,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="313">
+  <cellXfs count="317">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -3541,6 +3560,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3847,21 +3870,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K109"/>
+  <dimension ref="A1:J109"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" customWidth="true" style="1" width="17.81640625"/>
+    <col min="2" max="2" customWidth="true" style="1" width="15.0"/>
+    <col min="3" max="3" customWidth="true" style="1" width="15.36328125"/>
+    <col min="4" max="4" customWidth="true" style="1" width="17.453125"/>
+    <col min="5" max="5" customWidth="true" style="1" width="16.6328125"/>
+    <col min="6" max="6" customWidth="true" style="1" width="18.0"/>
+    <col min="7" max="7" customWidth="true" style="1" width="17.26953125"/>
+    <col min="8" max="8" customWidth="true" style="1" width="18.1796875"/>
+    <col min="9" max="9" customWidth="true" style="1" width="18.36328125"/>
+    <col min="10" max="10" customWidth="true" style="1" width="17.453125"/>
+    <col min="11" max="11" customWidth="true" style="1" width="17.36328125"/>
+    <col min="12" max="16384" style="1" width="8.7265625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -4617,7 +4640,7 @@
       <c r="B44" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="315" t="s">
         <v>192</v>
       </c>
       <c r="D44" s="305" t="s">
@@ -4654,7 +4677,7 @@
       <c r="C46" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D46" s="316" t="s">
         <v>244</v>
       </c>
       <c r="E46" s="115" t="s">
@@ -4913,7 +4936,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A72" s="312" t="s">
+      <c r="A72" s="313" t="s">
         <v>1021</v>
       </c>
       <c r="E72" s="195" t="s">
@@ -4921,7 +4944,7 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A73" s="312" t="s">
+      <c r="A73" s="314" t="s">
         <v>1022</v>
       </c>
       <c r="E73" s="212" t="s">
@@ -5148,85 +5171,91 @@
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.90625" customWidth="1"/>
-    <col min="2" max="2" width="29.453125" customWidth="1"/>
-    <col min="3" max="3" width="35.6328125" customWidth="1"/>
-    <col min="4" max="4" width="30.90625" customWidth="1"/>
-    <col min="5" max="5" width="32.7265625" customWidth="1"/>
-    <col min="6" max="6" width="32.1796875" customWidth="1"/>
-    <col min="7" max="7" width="33.6328125" customWidth="1"/>
-    <col min="8" max="8" width="31.26953125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="26.90625"/>
+    <col min="2" max="2" customWidth="true" width="29.453125"/>
+    <col min="3" max="3" customWidth="true" width="35.6328125"/>
+    <col min="4" max="4" customWidth="true" width="30.90625"/>
+    <col min="5" max="5" customWidth="true" width="32.7265625"/>
+    <col min="6" max="6" customWidth="true" width="32.1796875"/>
+    <col min="7" max="7" customWidth="true" width="33.6328125"/>
+    <col min="8" max="8" customWidth="true" width="31.26953125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>11</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>1045</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="A2" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C2" t="s" s="0">
         <v>29</v>
       </c>
+      <c r="D2" t="s" s="0">
+        <v>29</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>1046</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="A3" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B3" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C3" t="s" s="0">
         <v>29</v>
       </c>
+      <c r="D3" t="s" s="0">
+        <v>29</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
+        <v>1047</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s" s="0">
+        <v>1048</v>
+      </c>
+      <c r="D5" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="B4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D5" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D6" t="s">
+      <c r="A6" t="s" s="0">
+        <v>1049</v>
+      </c>
+      <c r="D6" t="s" s="0">
         <v>29</v>
       </c>
     </row>
@@ -5250,41 +5279,41 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I201"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.08984375" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" customWidth="1"/>
-    <col min="3" max="3" width="17.36328125" customWidth="1"/>
-    <col min="4" max="5" width="17.26953125" customWidth="1"/>
-    <col min="6" max="6" width="17.1796875" customWidth="1"/>
-    <col min="7" max="7" width="15.36328125" customWidth="1"/>
-    <col min="8" max="8" width="17.1796875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="20.08984375"/>
+    <col min="2" max="2" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" customWidth="true" width="17.36328125"/>
+    <col min="4" max="5" customWidth="true" width="17.26953125"/>
+    <col min="6" max="6" customWidth="true" width="17.1796875"/>
+    <col min="7" max="7" customWidth="true" width="15.36328125"/>
+    <col min="8" max="8" customWidth="true" width="17.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="169" t="s">
         <v>296</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>297</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>298</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>299</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>300</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>301</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>302</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>303</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated pet name counter file and sample id's file.
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13590" windowHeight="4800"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13980" windowHeight="2810" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
@@ -12,12 +12,12 @@
     <sheet name="ADD_PET" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
+  <oleSize ref="A28:G34"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="764">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="743">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -49,108 +49,45 @@
     <t>Vet_Fauna</t>
   </si>
   <si>
-    <t>7PVMUV</t>
-  </si>
-  <si>
-    <t>RYCXKM</t>
-  </si>
-  <si>
-    <t>Y6G4FM</t>
-  </si>
-  <si>
     <t>CYGKE6</t>
   </si>
   <si>
     <t>NA6V7C</t>
   </si>
   <si>
-    <t>PATJTJ</t>
-  </si>
-  <si>
     <t>V63CMY</t>
   </si>
   <si>
-    <t>VJYGJP</t>
-  </si>
-  <si>
     <t>MPYAKP</t>
   </si>
   <si>
     <t>XD7DT3</t>
   </si>
   <si>
-    <t>NDCUX3</t>
-  </si>
-  <si>
     <t>394JV9</t>
   </si>
   <si>
     <t>EV6UEC</t>
   </si>
   <si>
-    <t>FK4JHP</t>
-  </si>
-  <si>
     <t>KAR9NK</t>
   </si>
   <si>
     <t>6GAFRG</t>
   </si>
   <si>
-    <t>EECV7H</t>
-  </si>
-  <si>
     <t>FEMHMK</t>
   </si>
   <si>
     <t>X6RDRC</t>
   </si>
   <si>
-    <t>HRFKDJ</t>
-  </si>
-  <si>
-    <t>RRDJNJ</t>
-  </si>
-  <si>
     <t>NNTHRC</t>
   </si>
   <si>
-    <t>HANTAF</t>
-  </si>
-  <si>
-    <t>UCXJPU</t>
-  </si>
-  <si>
-    <t>XEC9NE</t>
-  </si>
-  <si>
-    <t>6MT3TH</t>
-  </si>
-  <si>
-    <t>UKPPVN</t>
-  </si>
-  <si>
-    <t>AUTJHD</t>
-  </si>
-  <si>
     <t>7H6YMR</t>
   </si>
   <si>
-    <t>EAUVNA</t>
-  </si>
-  <si>
-    <t>XACPDY</t>
-  </si>
-  <si>
-    <t>EXRTGT</t>
-  </si>
-  <si>
-    <t>F9JDEF</t>
-  </si>
-  <si>
-    <t>CADMX6</t>
-  </si>
-  <si>
     <t>H4NC3U</t>
   </si>
   <si>
@@ -2266,56 +2203,55 @@
     <t>Nexra</t>
   </si>
   <si>
-    <t>Charlie74</t>
-  </si>
-  <si>
-    <t>Milo51</t>
-  </si>
-  <si>
-    <t>Taffy49</t>
-  </si>
-  <si>
-    <t>Charlie75</t>
-  </si>
-  <si>
-    <t>Milo52</t>
-  </si>
-  <si>
-    <t>Taffy50</t>
-  </si>
-  <si>
-    <t>Cutie39</t>
-  </si>
-  <si>
-    <t>Cinder39</t>
-  </si>
-  <si>
-    <t>pony32</t>
-  </si>
-  <si>
-    <t>Charlie76</t>
-  </si>
-  <si>
-    <t>Milo53</t>
-  </si>
-  <si>
-    <t>Taffy51</t>
-  </si>
-  <si>
-    <t>Cutie40</t>
-  </si>
-  <si>
-    <t>Cinder40</t>
-  </si>
-  <si>
-    <t>fury25</t>
+    <t>GVVFEP</t>
+  </si>
+  <si>
+    <t>FUTHNN</t>
+  </si>
+  <si>
+    <t>XKTDYU</t>
+  </si>
+  <si>
+    <t>J7PTRT</t>
+  </si>
+  <si>
+    <t>FAA9TM</t>
+  </si>
+  <si>
+    <t>HNECET</t>
+  </si>
+  <si>
+    <t>DCHJFC</t>
+  </si>
+  <si>
+    <t>GGYTUT</t>
+  </si>
+  <si>
+    <t>E47DUV</t>
+  </si>
+  <si>
+    <t>E4NC6K</t>
+  </si>
+  <si>
+    <t>PDNXE7</t>
+  </si>
+  <si>
+    <t>VGCJEJ</t>
+  </si>
+  <si>
+    <t>KRRUUJ</t>
+  </si>
+  <si>
+    <t>CKUGMJ</t>
+  </si>
+  <si>
+    <t>FENAMV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2370,7 +2306,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -2381,23 +2317,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2704,21 +2624,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:K119"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="17.81640625"/>
-    <col min="2" max="2" customWidth="true" style="1" width="15.0"/>
-    <col min="3" max="3" customWidth="true" style="1" width="15.36328125"/>
-    <col min="4" max="4" customWidth="true" style="1" width="17.453125"/>
-    <col min="5" max="5" customWidth="true" style="1" width="16.6328125"/>
-    <col min="6" max="6" customWidth="true" style="1" width="18.0"/>
-    <col min="7" max="7" customWidth="true" style="1" width="17.26953125"/>
-    <col min="8" max="8" customWidth="true" style="1" width="18.1796875"/>
-    <col min="9" max="9" customWidth="true" style="1" width="18.36328125"/>
-    <col min="10" max="10" customWidth="true" style="1" width="17.453125"/>
-    <col min="11" max="11" customWidth="true" style="1" width="17.36328125"/>
-    <col min="12" max="16384" style="1" width="8.7265625"/>
+    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -2754,172 +2674,149 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="9" t="s">
+      <c r="A2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>39</v>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="12" t="s">
+      <c r="A3" t="s">
+        <v>728</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>40</v>
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>737</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="18" t="s">
+      <c r="A4" t="s">
+        <v>729</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="24" t="s">
-        <v>41</v>
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>738</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="13" t="s">
-        <v>35</v>
+      <c r="A5" t="s">
+        <v>730</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>739</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>731</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>734</v>
+      </c>
+      <c r="D6" t="s">
+        <v>740</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>732</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>735</v>
+      </c>
+      <c r="D7" t="s">
+        <v>741</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>733</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>736</v>
+      </c>
+      <c r="D8" t="s">
+        <v>742</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="1" t="s">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E9" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="1" t="s">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>47</v>
-      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B11" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="E12" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E13" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E14" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E15" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E16" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E17" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35"/>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35"/>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35"/>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35"/>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35"/>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35"/>
@@ -3037,86 +2934,83 @@
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="26.90625"/>
-    <col min="2" max="2" customWidth="true" width="29.453125"/>
-    <col min="3" max="3" customWidth="true" width="35.6328125"/>
-    <col min="4" max="4" customWidth="true" width="30.90625"/>
-    <col min="5" max="5" customWidth="true" width="32.7265625"/>
-    <col min="6" max="6" customWidth="true" width="32.1796875"/>
-    <col min="7" max="7" customWidth="true" width="33.6328125"/>
-    <col min="8" max="8" customWidth="true" width="31.26953125"/>
+    <col min="1" max="1" width="26.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" customWidth="1"/>
+    <col min="4" max="4" width="30.90625" customWidth="1"/>
+    <col min="5" max="5" width="32.7265625" customWidth="1"/>
+    <col min="6" max="6" width="32.1796875" customWidth="1"/>
+    <col min="7" max="7" width="33.6328125" customWidth="1"/>
+    <col min="8" max="8" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
-        <v>55</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>56</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>57</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>58</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>59</v>
-      </c>
-      <c r="F1" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="G1" t="s" s="0">
-        <v>61</v>
-      </c>
-      <c r="H1" t="s" s="0">
-        <v>62</v>
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>63</v>
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>762</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>63</v>
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>63</v>
+      <c r="A4" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D5" t="s" s="0">
-        <v>63</v>
+      <c r="D5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D6" t="s" s="0">
-        <v>63</v>
+      <c r="D6" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -3130,2470 +3024,2470 @@
   <dimension ref="A1:H201"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.08984375"/>
-    <col min="2" max="2" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" customWidth="true" width="17.36328125"/>
-    <col min="4" max="5" customWidth="true" width="17.26953125"/>
-    <col min="6" max="6" customWidth="true" width="17.1796875"/>
-    <col min="7" max="7" customWidth="true" width="15.36328125"/>
-    <col min="8" max="8" customWidth="true" width="17.1796875"/>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="4" max="5" width="17.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" t="s">
         <v>64</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="C5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="D5" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D1" t="s" s="0">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>67</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="B6" t="s">
         <v>68</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="D6" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="H1" t="s" s="0">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="B7" t="s">
         <v>72</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="C7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D7" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D2" s="6" t="s">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="B8" t="s">
         <v>76</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="C8" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D8" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="6" t="s">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="B9" t="s">
         <v>80</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="C9" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D9" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D4" s="6" t="s">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s" s="0">
+      <c r="B10" t="s">
         <v>84</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="C10" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D10" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D5" s="6" t="s">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" t="s" s="0">
+      <c r="B11" t="s">
         <v>88</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="C11" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D11" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="D6" s="6" t="s">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" t="s" s="0">
+      <c r="B12" t="s">
         <v>92</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="C12" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D12" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="D7" s="6" t="s">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" t="s" s="0">
+      <c r="B13" t="s">
         <v>96</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="C13" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D13" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="6" t="s">
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" t="s" s="0">
+      <c r="B14" t="s">
         <v>100</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="C14" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D14" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D9" s="6" t="s">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" t="s" s="0">
+      <c r="B15" t="s">
         <v>104</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="C15" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D15" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D10" s="6" t="s">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" t="s" s="0">
+      <c r="B16" t="s">
         <v>108</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="C16" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D16" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="6" t="s">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" t="s" s="0">
+      <c r="B17" t="s">
         <v>112</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="C17" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D17" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D12" s="6" t="s">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" t="s" s="0">
+      <c r="B18" t="s">
         <v>116</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="C18" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D18" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="D13" s="6" t="s">
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" t="s" s="0">
+      <c r="B19" t="s">
         <v>120</v>
       </c>
-      <c r="B14" t="s" s="0">
+      <c r="C19" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D19" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="D14" s="6" t="s">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" t="s" s="0">
+      <c r="B20" t="s">
         <v>124</v>
       </c>
-      <c r="B15" t="s" s="0">
+      <c r="C20" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="D20" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="D15" s="6" t="s">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" t="s" s="0">
+      <c r="B21" t="s">
         <v>128</v>
       </c>
-      <c r="B16" t="s" s="0">
+      <c r="C21" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D21" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="D16" s="6" t="s">
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" t="s" s="0">
+      <c r="B22" t="s">
         <v>132</v>
       </c>
-      <c r="B17" t="s" s="0">
+      <c r="C22" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="D17" s="6" t="s">
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" t="s" s="0">
+      <c r="B23" t="s">
         <v>136</v>
       </c>
-      <c r="B18" t="s" s="0">
+      <c r="C23" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D23" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="D18" s="6" t="s">
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" t="s" s="0">
+      <c r="B24" t="s">
         <v>140</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="C24" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D24" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="D19" s="6" t="s">
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" t="s" s="0">
+      <c r="B25" t="s">
         <v>144</v>
       </c>
-      <c r="B20" t="s" s="0">
+      <c r="C25" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="D25" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="D20" s="6" t="s">
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" t="s" s="0">
+      <c r="B26" t="s">
         <v>148</v>
       </c>
-      <c r="B21" t="s" s="0">
+      <c r="C26" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="D26" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="D21" s="6" t="s">
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" t="s" s="0">
+      <c r="B27" t="s">
         <v>152</v>
       </c>
-      <c r="B22" t="s" s="0">
+      <c r="C27" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="D27" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="D22" s="6" t="s">
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" t="s" s="0">
+      <c r="B28" t="s">
         <v>156</v>
       </c>
-      <c r="B23" t="s" s="0">
+      <c r="C28" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="D28" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D23" s="6" t="s">
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" t="s" s="0">
+      <c r="B29" t="s">
         <v>160</v>
       </c>
-      <c r="B24" t="s" s="0">
+      <c r="C29" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="D29" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="D24" s="6" t="s">
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" t="s" s="0">
+      <c r="B30" t="s">
         <v>164</v>
       </c>
-      <c r="B25" t="s" s="0">
+      <c r="C30" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D30" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="D25" s="6" t="s">
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" t="s" s="0">
+      <c r="B31" t="s">
         <v>168</v>
       </c>
-      <c r="B26" t="s" s="0">
+      <c r="C31" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="D31" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="D26" s="6" t="s">
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" t="s" s="0">
+      <c r="B32" t="s">
         <v>172</v>
       </c>
-      <c r="B27" t="s" s="0">
+      <c r="C32" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="D32" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="D27" s="6" t="s">
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" t="s" s="0">
+      <c r="B33" t="s">
         <v>176</v>
       </c>
-      <c r="B28" t="s" s="0">
+      <c r="C33" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="D33" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="D28" s="6" t="s">
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" t="s" s="0">
+      <c r="B34" t="s">
         <v>180</v>
       </c>
-      <c r="B29" t="s" s="0">
+      <c r="C34" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="D34" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="D29" s="6" t="s">
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" t="s" s="0">
+      <c r="B35" t="s">
         <v>184</v>
       </c>
-      <c r="B30" t="s" s="0">
+      <c r="C35" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="D35" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="D30" s="6" t="s">
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" t="s" s="0">
+      <c r="B36" t="s">
         <v>188</v>
       </c>
-      <c r="B31" t="s" s="0">
+      <c r="C36" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="D36" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="D31" s="6" t="s">
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" t="s" s="0">
+      <c r="B37" t="s">
         <v>192</v>
       </c>
-      <c r="B32" t="s" s="0">
+      <c r="C37" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="D37" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="D32" s="6" t="s">
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" t="s" s="0">
+      <c r="B38" t="s">
         <v>196</v>
       </c>
-      <c r="B33" t="s" s="0">
+      <c r="C38" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="D38" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="D33" s="6" t="s">
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" t="s" s="0">
+      <c r="B39" t="s">
         <v>200</v>
       </c>
-      <c r="B34" t="s" s="0">
+      <c r="C39" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="D39" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="D34" s="6" t="s">
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" t="s" s="0">
+      <c r="B40" t="s">
         <v>204</v>
       </c>
-      <c r="B35" t="s" s="0">
+      <c r="C40" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="D40" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="D35" s="6" t="s">
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" t="s" s="0">
+      <c r="B41" t="s">
         <v>208</v>
       </c>
-      <c r="B36" t="s" s="0">
+      <c r="C41" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="D41" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="D36" s="6" t="s">
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" t="s" s="0">
+      <c r="B42" t="s">
         <v>212</v>
       </c>
-      <c r="B37" t="s" s="0">
+      <c r="C42" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="D42" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="D37" s="6" t="s">
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" t="s" s="0">
+      <c r="B43" t="s">
         <v>216</v>
       </c>
-      <c r="B38" t="s" s="0">
+      <c r="C43" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="D43" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="D38" s="6" t="s">
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" t="s" s="0">
+      <c r="B44" t="s">
         <v>220</v>
       </c>
-      <c r="B39" t="s" s="0">
+      <c r="C44" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="D44" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="D39" s="6" t="s">
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" t="s" s="0">
+      <c r="B45" t="s">
         <v>224</v>
       </c>
-      <c r="B40" t="s" s="0">
+      <c r="C45" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="D45" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="D40" s="6" t="s">
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" t="s" s="0">
+      <c r="B46" t="s">
         <v>228</v>
       </c>
-      <c r="B41" t="s" s="0">
+      <c r="C46" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="C41" s="7" t="s">
+      <c r="D46" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="D41" s="6" t="s">
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" t="s" s="0">
+      <c r="B47" t="s">
         <v>232</v>
       </c>
-      <c r="B42" t="s" s="0">
+      <c r="C47" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="D47" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="D42" s="6" t="s">
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" t="s" s="0">
+      <c r="B48" t="s">
         <v>236</v>
       </c>
-      <c r="B43" t="s" s="0">
+      <c r="C48" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="D48" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="D43" s="6" t="s">
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" t="s" s="0">
+      <c r="B49" t="s">
         <v>240</v>
       </c>
-      <c r="B44" t="s" s="0">
+      <c r="C49" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="D49" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="D44" s="6" t="s">
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" t="s" s="0">
+      <c r="B50" t="s">
         <v>244</v>
       </c>
-      <c r="B45" t="s" s="0">
+      <c r="C50" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="C45" s="7" t="s">
+      <c r="D50" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="D45" s="6" t="s">
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" t="s" s="0">
+      <c r="B51" t="s">
         <v>248</v>
       </c>
-      <c r="B46" t="s" s="0">
+      <c r="C51" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="D51" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="D46" s="6" t="s">
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A47" t="s" s="0">
+      <c r="B52" t="s">
         <v>252</v>
       </c>
-      <c r="B47" t="s" s="0">
+      <c r="C52" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="D52" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="D47" s="6" t="s">
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A48" t="s" s="0">
+      <c r="B53" t="s">
         <v>256</v>
       </c>
-      <c r="B48" t="s" s="0">
+      <c r="C53" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="D53" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="D48" s="6" t="s">
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" t="s" s="0">
+      <c r="B54" t="s">
         <v>260</v>
       </c>
-      <c r="B49" t="s" s="0">
+      <c r="C54" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="D54" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="D49" s="6" t="s">
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" t="s" s="0">
+      <c r="B55" t="s">
         <v>264</v>
       </c>
-      <c r="B50" t="s" s="0">
+      <c r="C55" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="D55" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="D50" s="6" t="s">
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" t="s" s="0">
+      <c r="B56" t="s">
         <v>268</v>
       </c>
-      <c r="B51" t="s" s="0">
+      <c r="C56" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="D56" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="D51" s="6" t="s">
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" t="s" s="0">
+      <c r="B57" t="s">
         <v>272</v>
       </c>
-      <c r="B52" t="s" s="0">
+      <c r="C57" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="C52" s="7" t="s">
+      <c r="D57" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="D52" s="6" t="s">
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" t="s" s="0">
+      <c r="B58" t="s">
         <v>276</v>
       </c>
-      <c r="B53" t="s" s="0">
+      <c r="C58" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="C53" s="7" t="s">
+      <c r="D58" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="D53" s="6" t="s">
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A54" t="s" s="0">
+      <c r="B59" t="s">
         <v>280</v>
       </c>
-      <c r="B54" t="s" s="0">
+      <c r="C59" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="D59" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="D54" s="6" t="s">
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A55" t="s" s="0">
+      <c r="B60" t="s">
         <v>284</v>
       </c>
-      <c r="B55" t="s" s="0">
+      <c r="C60" s="7" t="s">
         <v>285</v>
       </c>
-      <c r="C55" s="7" t="s">
+      <c r="D60" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="D55" s="6" t="s">
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" t="s" s="0">
+      <c r="B61" t="s">
         <v>288</v>
       </c>
-      <c r="B56" t="s" s="0">
+      <c r="C61" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="C56" s="7" t="s">
+      <c r="D61" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="D56" s="6" t="s">
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" t="s" s="0">
+      <c r="B62" t="s">
         <v>292</v>
       </c>
-      <c r="B57" t="s" s="0">
+      <c r="C62" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="D62" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="D57" s="6" t="s">
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" t="s" s="0">
+      <c r="B63" t="s">
         <v>296</v>
       </c>
-      <c r="B58" t="s" s="0">
+      <c r="C63" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="C58" s="7" t="s">
+      <c r="D63" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="D58" s="6" t="s">
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" t="s" s="0">
+      <c r="B64" t="s">
         <v>300</v>
       </c>
-      <c r="B59" t="s" s="0">
+      <c r="C64" s="7" t="s">
         <v>301</v>
       </c>
-      <c r="C59" s="7" t="s">
+      <c r="D64" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="D59" s="6" t="s">
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" t="s" s="0">
+      <c r="B65" t="s">
         <v>304</v>
       </c>
-      <c r="B60" t="s" s="0">
+      <c r="C65" s="7" t="s">
         <v>305</v>
       </c>
-      <c r="C60" s="7" t="s">
+      <c r="D65" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="D60" s="6" t="s">
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" t="s" s="0">
+      <c r="B66" t="s">
         <v>308</v>
       </c>
-      <c r="B61" t="s" s="0">
+      <c r="C66" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="D66" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="D61" s="6" t="s">
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" t="s" s="0">
+      <c r="B67" t="s">
         <v>312</v>
       </c>
-      <c r="B62" t="s" s="0">
+      <c r="C67" s="7" t="s">
         <v>313</v>
       </c>
-      <c r="C62" s="7" t="s">
+      <c r="D67" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="D62" s="6" t="s">
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A63" t="s" s="0">
+      <c r="B68" t="s">
         <v>316</v>
       </c>
-      <c r="B63" t="s" s="0">
+      <c r="C68" s="7" t="s">
         <v>317</v>
       </c>
-      <c r="C63" s="7" t="s">
+      <c r="D68" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="D63" s="6" t="s">
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A64" t="s" s="0">
+      <c r="B69" t="s">
         <v>320</v>
       </c>
-      <c r="B64" t="s" s="0">
+      <c r="C69" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="C64" s="7" t="s">
+      <c r="D69" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="D64" s="6" t="s">
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" t="s" s="0">
+      <c r="B70" t="s">
         <v>324</v>
       </c>
-      <c r="B65" t="s" s="0">
+      <c r="C70" s="7" t="s">
         <v>325</v>
       </c>
-      <c r="C65" s="7" t="s">
+      <c r="D70" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="D65" s="6" t="s">
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" t="s" s="0">
+      <c r="B71" t="s">
         <v>328</v>
       </c>
-      <c r="B66" t="s" s="0">
+      <c r="C71" s="7" t="s">
         <v>329</v>
       </c>
-      <c r="C66" s="7" t="s">
+      <c r="D71" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="D66" s="6" t="s">
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A67" t="s" s="0">
+      <c r="B72" t="s">
         <v>332</v>
       </c>
-      <c r="B67" t="s" s="0">
+      <c r="C72" s="7" t="s">
         <v>333</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="D72" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="D67" s="6" t="s">
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" t="s" s="0">
+      <c r="B73" t="s">
         <v>336</v>
       </c>
-      <c r="B68" t="s" s="0">
+      <c r="C73" s="7" t="s">
         <v>337</v>
       </c>
-      <c r="C68" s="7" t="s">
+      <c r="D73" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="D68" s="6" t="s">
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" t="s" s="0">
+      <c r="B74" t="s">
         <v>340</v>
       </c>
-      <c r="B69" t="s" s="0">
+      <c r="C74" s="7" t="s">
         <v>341</v>
       </c>
-      <c r="C69" s="7" t="s">
+      <c r="D74" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="D69" s="6" t="s">
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" t="s" s="0">
+      <c r="B75" t="s">
         <v>344</v>
       </c>
-      <c r="B70" t="s" s="0">
+      <c r="C75" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="C70" s="7" t="s">
+      <c r="D75" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="D70" s="6" t="s">
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A71" t="s" s="0">
+      <c r="B76" t="s">
         <v>348</v>
       </c>
-      <c r="B71" t="s" s="0">
+      <c r="C76" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="C71" s="7" t="s">
+      <c r="D76" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="D71" s="6" t="s">
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A72" t="s" s="0">
+      <c r="B77" t="s">
         <v>352</v>
       </c>
-      <c r="B72" t="s" s="0">
+      <c r="C77" s="7" t="s">
         <v>353</v>
       </c>
-      <c r="C72" s="7" t="s">
+      <c r="D77" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="D72" s="6" t="s">
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A73" t="s" s="0">
+      <c r="B78" t="s">
         <v>356</v>
       </c>
-      <c r="B73" t="s" s="0">
+      <c r="C78" s="7" t="s">
         <v>357</v>
       </c>
-      <c r="C73" s="7" t="s">
+      <c r="D78" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="D73" s="6" t="s">
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" t="s" s="0">
+      <c r="B79" t="s">
         <v>360</v>
       </c>
-      <c r="B74" t="s" s="0">
+      <c r="C79" s="7" t="s">
         <v>361</v>
       </c>
-      <c r="C74" s="7" t="s">
+      <c r="D79" s="6" t="s">
         <v>362</v>
       </c>
-      <c r="D74" s="6" t="s">
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" t="s" s="0">
+      <c r="B80" t="s">
         <v>364</v>
       </c>
-      <c r="B75" t="s" s="0">
+      <c r="C80" s="7" t="s">
         <v>365</v>
       </c>
-      <c r="C75" s="7" t="s">
+      <c r="D80" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="D75" s="6" t="s">
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" t="s" s="0">
+      <c r="B81" t="s">
         <v>368</v>
       </c>
-      <c r="B76" t="s" s="0">
+      <c r="C81" s="7" t="s">
         <v>369</v>
       </c>
-      <c r="C76" s="7" t="s">
+      <c r="D81" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="D76" s="6" t="s">
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A77" t="s" s="0">
+      <c r="B82" t="s">
         <v>372</v>
       </c>
-      <c r="B77" t="s" s="0">
+      <c r="C82" s="7" t="s">
         <v>373</v>
       </c>
-      <c r="C77" s="7" t="s">
+      <c r="D82" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="D77" s="6" t="s">
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A78" t="s" s="0">
+      <c r="B83" t="s">
         <v>376</v>
       </c>
-      <c r="B78" t="s" s="0">
+      <c r="C83" s="7" t="s">
         <v>377</v>
       </c>
-      <c r="C78" s="7" t="s">
+      <c r="D83" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="D78" s="6" t="s">
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A79" t="s" s="0">
+      <c r="B84" t="s">
         <v>380</v>
       </c>
-      <c r="B79" t="s" s="0">
+      <c r="C84" s="7" t="s">
         <v>381</v>
       </c>
-      <c r="C79" s="7" t="s">
+      <c r="D84" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="D79" s="6" t="s">
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
         <v>383</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A80" t="s" s="0">
+      <c r="B85" t="s">
         <v>384</v>
       </c>
-      <c r="B80" t="s" s="0">
+      <c r="C85" s="7" t="s">
         <v>385</v>
       </c>
-      <c r="C80" s="7" t="s">
+      <c r="D85" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="D80" s="6" t="s">
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A81" t="s" s="0">
+      <c r="B86" t="s">
         <v>388</v>
       </c>
-      <c r="B81" t="s" s="0">
+      <c r="C86" s="7" t="s">
         <v>389</v>
       </c>
-      <c r="C81" s="7" t="s">
+      <c r="D86" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="D81" s="6" t="s">
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" t="s" s="0">
+      <c r="B87" t="s">
         <v>392</v>
       </c>
-      <c r="B82" t="s" s="0">
+      <c r="C87" s="7" t="s">
         <v>393</v>
       </c>
-      <c r="C82" s="7" t="s">
+      <c r="D87" s="6" t="s">
         <v>394</v>
       </c>
-      <c r="D82" s="6" t="s">
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A83" t="s" s="0">
+      <c r="B88" t="s">
         <v>396</v>
       </c>
-      <c r="B83" t="s" s="0">
+      <c r="C88" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="C83" s="7" t="s">
+      <c r="D88" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="D83" s="6" t="s">
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A84" t="s" s="0">
+      <c r="B89" t="s">
         <v>400</v>
       </c>
-      <c r="B84" t="s" s="0">
+      <c r="C89" s="7" t="s">
         <v>401</v>
       </c>
-      <c r="C84" s="7" t="s">
+      <c r="D89" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="D84" s="6" t="s">
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A85" t="s" s="0">
+      <c r="B90" t="s">
         <v>404</v>
       </c>
-      <c r="B85" t="s" s="0">
+      <c r="C90" s="7" t="s">
         <v>405</v>
       </c>
-      <c r="C85" s="7" t="s">
+      <c r="D90" s="6" t="s">
         <v>406</v>
       </c>
-      <c r="D85" s="6" t="s">
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
         <v>407</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A86" t="s" s="0">
+      <c r="B91" t="s">
         <v>408</v>
       </c>
-      <c r="B86" t="s" s="0">
+      <c r="C91" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="C86" s="7" t="s">
+      <c r="D91" s="6" t="s">
         <v>410</v>
       </c>
-      <c r="D86" s="6" t="s">
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A87" t="s" s="0">
+      <c r="B92" t="s">
         <v>412</v>
       </c>
-      <c r="B87" t="s" s="0">
+      <c r="C92" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="C87" s="7" t="s">
+      <c r="D92" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="D87" s="6" t="s">
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A88" t="s" s="0">
+      <c r="B93" t="s">
         <v>416</v>
       </c>
-      <c r="B88" t="s" s="0">
+      <c r="C93" s="7" t="s">
         <v>417</v>
       </c>
-      <c r="C88" s="7" t="s">
+      <c r="D93" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="D88" s="6" t="s">
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A89" t="s" s="0">
+      <c r="B94" t="s">
         <v>420</v>
       </c>
-      <c r="B89" t="s" s="0">
+      <c r="C94" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="C89" s="7" t="s">
+      <c r="D94" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="D89" s="6" t="s">
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>423</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A90" t="s" s="0">
+      <c r="B95" t="s">
         <v>424</v>
       </c>
-      <c r="B90" t="s" s="0">
+      <c r="C95" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="C90" s="7" t="s">
+      <c r="D95" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="D90" s="6" t="s">
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A91" t="s" s="0">
+      <c r="B96" t="s">
         <v>428</v>
       </c>
-      <c r="B91" t="s" s="0">
+      <c r="C96" s="7" t="s">
         <v>429</v>
       </c>
-      <c r="C91" s="7" t="s">
+      <c r="D96" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="D91" s="6" t="s">
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
         <v>431</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A92" t="s" s="0">
+      <c r="B97" t="s">
         <v>432</v>
       </c>
-      <c r="B92" t="s" s="0">
+      <c r="C97" s="7" t="s">
         <v>433</v>
       </c>
-      <c r="C92" s="7" t="s">
+      <c r="D97" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="D92" s="6" t="s">
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
         <v>435</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A93" t="s" s="0">
+      <c r="B98" t="s">
         <v>436</v>
       </c>
-      <c r="B93" t="s" s="0">
+      <c r="C98" s="7" t="s">
         <v>437</v>
       </c>
-      <c r="C93" s="7" t="s">
+      <c r="D98" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="D93" s="6" t="s">
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
         <v>439</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A94" t="s" s="0">
+      <c r="B99" t="s">
         <v>440</v>
       </c>
-      <c r="B94" t="s" s="0">
+      <c r="C99" s="7" t="s">
         <v>441</v>
       </c>
-      <c r="C94" s="7" t="s">
+      <c r="D99" s="6" t="s">
         <v>442</v>
       </c>
-      <c r="D94" s="6" t="s">
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
         <v>443</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A95" t="s" s="0">
+      <c r="B100" t="s">
         <v>444</v>
       </c>
-      <c r="B95" t="s" s="0">
+      <c r="C100" s="7" t="s">
         <v>445</v>
       </c>
-      <c r="C95" s="7" t="s">
+      <c r="D100" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="D95" s="6" t="s">
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>447</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A96" t="s" s="0">
+      <c r="B101" t="s">
         <v>448</v>
       </c>
-      <c r="B96" t="s" s="0">
+      <c r="C101" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="C96" s="7" t="s">
+      <c r="D101" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="D96" s="6" t="s">
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
         <v>451</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A97" t="s" s="0">
+      <c r="B102" t="s">
         <v>452</v>
       </c>
-      <c r="B97" t="s" s="0">
+      <c r="C102" s="7" t="s">
         <v>453</v>
       </c>
-      <c r="C97" s="7" t="s">
+      <c r="D102" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="D97" s="6" t="s">
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A98" t="s" s="0">
+      <c r="B103" t="s">
         <v>456</v>
       </c>
-      <c r="B98" t="s" s="0">
+      <c r="C103" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="C98" s="7" t="s">
+      <c r="D103" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="D98" s="6" t="s">
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
         <v>459</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A99" t="s" s="0">
+      <c r="B104" t="s">
         <v>460</v>
       </c>
-      <c r="B99" t="s" s="0">
+      <c r="C104" s="7" t="s">
         <v>461</v>
       </c>
-      <c r="C99" s="7" t="s">
+      <c r="D104" s="6" t="s">
         <v>462</v>
       </c>
-      <c r="D99" s="6" t="s">
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
         <v>463</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A100" t="s" s="0">
+      <c r="B105" t="s">
         <v>464</v>
       </c>
-      <c r="B100" t="s" s="0">
+      <c r="C105" s="7" t="s">
         <v>465</v>
       </c>
-      <c r="C100" s="7" t="s">
+      <c r="D105" s="6" t="s">
         <v>466</v>
       </c>
-      <c r="D100" s="6" t="s">
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
         <v>467</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A101" t="s" s="0">
+      <c r="B106" t="s">
         <v>468</v>
       </c>
-      <c r="B101" t="s" s="0">
+      <c r="C106" s="7" t="s">
         <v>469</v>
       </c>
-      <c r="C101" s="7" t="s">
+      <c r="D106" s="6" t="s">
         <v>470</v>
       </c>
-      <c r="D101" s="6" t="s">
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
         <v>471</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A102" t="s" s="0">
+      <c r="B107" t="s">
         <v>472</v>
       </c>
-      <c r="B102" t="s" s="0">
+      <c r="C107" s="7" t="s">
         <v>473</v>
       </c>
-      <c r="C102" s="7" t="s">
+      <c r="D107" s="6" t="s">
         <v>474</v>
       </c>
-      <c r="D102" s="6" t="s">
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
         <v>475</v>
       </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A103" t="s" s="0">
+      <c r="B108" t="s">
         <v>476</v>
       </c>
-      <c r="B103" t="s" s="0">
+      <c r="C108" s="7" t="s">
         <v>477</v>
       </c>
-      <c r="C103" s="7" t="s">
+      <c r="D108" s="6" t="s">
         <v>478</v>
       </c>
-      <c r="D103" s="6" t="s">
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
         <v>479</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A104" t="s" s="0">
+      <c r="B109" t="s">
         <v>480</v>
       </c>
-      <c r="B104" t="s" s="0">
+      <c r="C109" s="7" t="s">
         <v>481</v>
       </c>
-      <c r="C104" s="7" t="s">
+      <c r="D109" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="D104" s="6" t="s">
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
         <v>483</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A105" t="s" s="0">
+      <c r="B110" t="s">
         <v>484</v>
       </c>
-      <c r="B105" t="s" s="0">
+      <c r="C110" s="7" t="s">
         <v>485</v>
       </c>
-      <c r="C105" s="7" t="s">
+      <c r="D110" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="D105" s="6" t="s">
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A106" t="s" s="0">
+      <c r="B111" t="s">
         <v>488</v>
       </c>
-      <c r="B106" t="s" s="0">
+      <c r="C111" s="7" t="s">
         <v>489</v>
       </c>
-      <c r="C106" s="7" t="s">
+      <c r="D111" s="6" t="s">
         <v>490</v>
       </c>
-      <c r="D106" s="6" t="s">
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
         <v>491</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A107" t="s" s="0">
+      <c r="B112" t="s">
         <v>492</v>
       </c>
-      <c r="B107" t="s" s="0">
+      <c r="C112" s="7" t="s">
         <v>493</v>
       </c>
-      <c r="C107" s="7" t="s">
+      <c r="D112" s="6" t="s">
         <v>494</v>
       </c>
-      <c r="D107" s="6" t="s">
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
         <v>495</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A108" t="s" s="0">
+      <c r="B113" t="s">
         <v>496</v>
       </c>
-      <c r="B108" t="s" s="0">
+      <c r="C113" s="7" t="s">
         <v>497</v>
       </c>
-      <c r="C108" s="7" t="s">
+      <c r="D113" s="6" t="s">
         <v>498</v>
       </c>
-      <c r="D108" s="6" t="s">
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
         <v>499</v>
       </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A109" t="s" s="0">
+      <c r="B114" t="s">
         <v>500</v>
       </c>
-      <c r="B109" t="s" s="0">
+      <c r="C114" s="7" t="s">
         <v>501</v>
       </c>
-      <c r="C109" s="7" t="s">
+      <c r="D114" s="6" t="s">
         <v>502</v>
       </c>
-      <c r="D109" s="6" t="s">
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
         <v>503</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A110" t="s" s="0">
+      <c r="B115" t="s">
         <v>504</v>
       </c>
-      <c r="B110" t="s" s="0">
+      <c r="C115" s="7" t="s">
         <v>505</v>
       </c>
-      <c r="C110" s="7" t="s">
+      <c r="D115" s="6" t="s">
         <v>506</v>
       </c>
-      <c r="D110" s="6" t="s">
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
         <v>507</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A111" t="s" s="0">
+      <c r="B116" t="s">
         <v>508</v>
       </c>
-      <c r="B111" t="s" s="0">
+      <c r="C116" s="7" t="s">
         <v>509</v>
       </c>
-      <c r="C111" s="7" t="s">
+      <c r="D116" s="6" t="s">
         <v>510</v>
       </c>
-      <c r="D111" s="6" t="s">
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
         <v>511</v>
       </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A112" t="s" s="0">
+      <c r="B117" t="s">
         <v>512</v>
       </c>
-      <c r="B112" t="s" s="0">
+      <c r="C117" s="7" t="s">
         <v>513</v>
       </c>
-      <c r="C112" s="7" t="s">
+      <c r="D117" s="6" t="s">
         <v>514</v>
       </c>
-      <c r="D112" s="6" t="s">
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
         <v>515</v>
       </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A113" t="s" s="0">
+      <c r="B118" t="s">
         <v>516</v>
       </c>
-      <c r="B113" t="s" s="0">
+      <c r="C118" s="7" t="s">
         <v>517</v>
       </c>
-      <c r="C113" s="7" t="s">
+      <c r="D118" s="6" t="s">
         <v>518</v>
       </c>
-      <c r="D113" s="6" t="s">
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
         <v>519</v>
       </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A114" t="s" s="0">
+      <c r="B119" t="s">
         <v>520</v>
       </c>
-      <c r="B114" t="s" s="0">
+      <c r="C119" s="7" t="s">
         <v>521</v>
       </c>
-      <c r="C114" s="7" t="s">
+      <c r="D119" s="6" t="s">
         <v>522</v>
       </c>
-      <c r="D114" s="6" t="s">
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
         <v>523</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A115" t="s" s="0">
+      <c r="B120" t="s">
         <v>524</v>
       </c>
-      <c r="B115" t="s" s="0">
+      <c r="C120" s="7" t="s">
         <v>525</v>
       </c>
-      <c r="C115" s="7" t="s">
+      <c r="D120" s="6" t="s">
         <v>526</v>
       </c>
-      <c r="D115" s="6" t="s">
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A116" t="s" s="0">
+      <c r="B121" t="s">
         <v>528</v>
       </c>
-      <c r="B116" t="s" s="0">
+      <c r="C121" s="7" t="s">
         <v>529</v>
       </c>
-      <c r="C116" s="7" t="s">
+      <c r="D121" s="6" t="s">
         <v>530</v>
       </c>
-      <c r="D116" s="6" t="s">
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A117" t="s" s="0">
+      <c r="B122" t="s">
         <v>532</v>
       </c>
-      <c r="B117" t="s" s="0">
+      <c r="C122" s="7" t="s">
         <v>533</v>
       </c>
-      <c r="C117" s="7" t="s">
+      <c r="D122" s="6" t="s">
         <v>534</v>
       </c>
-      <c r="D117" s="6" t="s">
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
         <v>535</v>
       </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A118" t="s" s="0">
+      <c r="B123" t="s">
         <v>536</v>
       </c>
-      <c r="B118" t="s" s="0">
+      <c r="C123" s="7" t="s">
         <v>537</v>
       </c>
-      <c r="C118" s="7" t="s">
+      <c r="D123" s="6" t="s">
         <v>538</v>
       </c>
-      <c r="D118" s="6" t="s">
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
         <v>539</v>
       </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A119" t="s" s="0">
+      <c r="B124" t="s">
         <v>540</v>
       </c>
-      <c r="B119" t="s" s="0">
+      <c r="C124" s="7" t="s">
         <v>541</v>
       </c>
-      <c r="C119" s="7" t="s">
+      <c r="D124" s="6" t="s">
         <v>542</v>
       </c>
-      <c r="D119" s="6" t="s">
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
         <v>543</v>
       </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A120" t="s" s="0">
+      <c r="B125" t="s">
         <v>544</v>
       </c>
-      <c r="B120" t="s" s="0">
+      <c r="C125" s="7" t="s">
         <v>545</v>
       </c>
-      <c r="C120" s="7" t="s">
+      <c r="D125" s="6" t="s">
         <v>546</v>
       </c>
-      <c r="D120" s="6" t="s">
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
         <v>547</v>
       </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A121" t="s" s="0">
+      <c r="B126" t="s">
         <v>548</v>
       </c>
-      <c r="B121" t="s" s="0">
+      <c r="C126" s="7" t="s">
         <v>549</v>
       </c>
-      <c r="C121" s="7" t="s">
+      <c r="D126" s="6" t="s">
         <v>550</v>
       </c>
-      <c r="D121" s="6" t="s">
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
         <v>551</v>
       </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A122" t="s" s="0">
+      <c r="B127" t="s">
         <v>552</v>
       </c>
-      <c r="B122" t="s" s="0">
+      <c r="C127" s="7" t="s">
         <v>553</v>
       </c>
-      <c r="C122" s="7" t="s">
+      <c r="D127" s="6" t="s">
         <v>554</v>
       </c>
-      <c r="D122" s="6" t="s">
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
         <v>555</v>
       </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A123" t="s" s="0">
+      <c r="B128" t="s">
         <v>556</v>
       </c>
-      <c r="B123" t="s" s="0">
+      <c r="C128" s="7" t="s">
         <v>557</v>
       </c>
-      <c r="C123" s="7" t="s">
+      <c r="D128" s="6" t="s">
         <v>558</v>
       </c>
-      <c r="D123" s="6" t="s">
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
         <v>559</v>
       </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A124" t="s" s="0">
+      <c r="B129" t="s">
         <v>560</v>
       </c>
-      <c r="B124" t="s" s="0">
+      <c r="C129" s="7" t="s">
         <v>561</v>
       </c>
-      <c r="C124" s="7" t="s">
+      <c r="D129" s="6" t="s">
         <v>562</v>
       </c>
-      <c r="D124" s="6" t="s">
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
         <v>563</v>
       </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A125" t="s" s="0">
+      <c r="B130" t="s">
         <v>564</v>
       </c>
-      <c r="B125" t="s" s="0">
+      <c r="C130" s="7" t="s">
         <v>565</v>
       </c>
-      <c r="C125" s="7" t="s">
+      <c r="D130" s="6" t="s">
         <v>566</v>
       </c>
-      <c r="D125" s="6" t="s">
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
         <v>567</v>
       </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A126" t="s" s="0">
+      <c r="B131" t="s">
         <v>568</v>
       </c>
-      <c r="B126" t="s" s="0">
+      <c r="C131" s="7" t="s">
         <v>569</v>
       </c>
-      <c r="C126" s="7" t="s">
+      <c r="D131" s="6" t="s">
         <v>570</v>
       </c>
-      <c r="D126" s="6" t="s">
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
         <v>571</v>
       </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A127" t="s" s="0">
+      <c r="B132" t="s">
         <v>572</v>
       </c>
-      <c r="B127" t="s" s="0">
+      <c r="C132" s="7" t="s">
         <v>573</v>
       </c>
-      <c r="C127" s="7" t="s">
+      <c r="D132" s="6" t="s">
         <v>574</v>
       </c>
-      <c r="D127" s="6" t="s">
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
         <v>575</v>
       </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A128" t="s" s="0">
+      <c r="B133" t="s">
         <v>576</v>
       </c>
-      <c r="B128" t="s" s="0">
+      <c r="C133" s="7" t="s">
         <v>577</v>
       </c>
-      <c r="C128" s="7" t="s">
+      <c r="D133" s="6" t="s">
         <v>578</v>
       </c>
-      <c r="D128" s="6" t="s">
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
         <v>579</v>
       </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A129" t="s" s="0">
+      <c r="B134" t="s">
         <v>580</v>
       </c>
-      <c r="B129" t="s" s="0">
+      <c r="C134" s="7" t="s">
         <v>581</v>
       </c>
-      <c r="C129" s="7" t="s">
+      <c r="D134" s="6" t="s">
         <v>582</v>
       </c>
-      <c r="D129" s="6" t="s">
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
         <v>583</v>
       </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A130" t="s" s="0">
+      <c r="B135" t="s">
         <v>584</v>
       </c>
-      <c r="B130" t="s" s="0">
+      <c r="C135" s="7" t="s">
         <v>585</v>
       </c>
-      <c r="C130" s="7" t="s">
+      <c r="D135" s="6" t="s">
         <v>586</v>
       </c>
-      <c r="D130" s="6" t="s">
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
         <v>587</v>
       </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A131" t="s" s="0">
+      <c r="B136" t="s">
         <v>588</v>
       </c>
-      <c r="B131" t="s" s="0">
+      <c r="C136" s="7" t="s">
         <v>589</v>
       </c>
-      <c r="C131" s="7" t="s">
+      <c r="D136" s="6" t="s">
         <v>590</v>
       </c>
-      <c r="D131" s="6" t="s">
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
         <v>591</v>
       </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A132" t="s" s="0">
+      <c r="B137" t="s">
         <v>592</v>
       </c>
-      <c r="B132" t="s" s="0">
+      <c r="C137" s="7" t="s">
         <v>593</v>
       </c>
-      <c r="C132" s="7" t="s">
+      <c r="D137" s="6" t="s">
         <v>594</v>
       </c>
-      <c r="D132" s="6" t="s">
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
         <v>595</v>
       </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A133" t="s" s="0">
+      <c r="B138" t="s">
         <v>596</v>
       </c>
-      <c r="B133" t="s" s="0">
+      <c r="C138" s="7" t="s">
         <v>597</v>
       </c>
-      <c r="C133" s="7" t="s">
+      <c r="D138" s="6" t="s">
         <v>598</v>
       </c>
-      <c r="D133" s="6" t="s">
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
         <v>599</v>
       </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A134" t="s" s="0">
+      <c r="B139" t="s">
         <v>600</v>
       </c>
-      <c r="B134" t="s" s="0">
+      <c r="C139" s="7" t="s">
         <v>601</v>
       </c>
-      <c r="C134" s="7" t="s">
+      <c r="D139" s="6" t="s">
         <v>602</v>
       </c>
-      <c r="D134" s="6" t="s">
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
         <v>603</v>
       </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A135" t="s" s="0">
+      <c r="B140" t="s">
         <v>604</v>
       </c>
-      <c r="B135" t="s" s="0">
+      <c r="C140" s="7" t="s">
         <v>605</v>
       </c>
-      <c r="C135" s="7" t="s">
+      <c r="D140" s="6" t="s">
         <v>606</v>
       </c>
-      <c r="D135" s="6" t="s">
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
         <v>607</v>
       </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A136" t="s" s="0">
+      <c r="B141" t="s">
         <v>608</v>
       </c>
-      <c r="B136" t="s" s="0">
+      <c r="C141" s="7" t="s">
         <v>609</v>
       </c>
-      <c r="C136" s="7" t="s">
+      <c r="D141" s="6" t="s">
         <v>610</v>
       </c>
-      <c r="D136" s="6" t="s">
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
         <v>611</v>
       </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A137" t="s" s="0">
+      <c r="B142" t="s">
         <v>612</v>
       </c>
-      <c r="B137" t="s" s="0">
+      <c r="C142" s="7" t="s">
         <v>613</v>
       </c>
-      <c r="C137" s="7" t="s">
+      <c r="D142" s="6" t="s">
         <v>614</v>
       </c>
-      <c r="D137" s="6" t="s">
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A138" t="s" s="0">
+      <c r="B143" t="s">
         <v>616</v>
       </c>
-      <c r="B138" t="s" s="0">
+      <c r="C143" s="7" t="s">
         <v>617</v>
       </c>
-      <c r="C138" s="7" t="s">
+      <c r="D143" s="6" t="s">
         <v>618</v>
       </c>
-      <c r="D138" s="6" t="s">
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
         <v>619</v>
       </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A139" t="s" s="0">
+      <c r="B144" t="s">
         <v>620</v>
       </c>
-      <c r="B139" t="s" s="0">
+      <c r="C144" s="7" t="s">
         <v>621</v>
       </c>
-      <c r="C139" s="7" t="s">
+      <c r="D144" s="6" t="s">
         <v>622</v>
       </c>
-      <c r="D139" s="6" t="s">
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
         <v>623</v>
       </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A140" t="s" s="0">
+      <c r="B145" t="s">
         <v>624</v>
       </c>
-      <c r="B140" t="s" s="0">
+      <c r="C145" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="C140" s="7" t="s">
+      <c r="D145" s="6" t="s">
         <v>626</v>
       </c>
-      <c r="D140" s="6" t="s">
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
         <v>627</v>
       </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A141" t="s" s="0">
+      <c r="B146" t="s">
         <v>628</v>
       </c>
-      <c r="B141" t="s" s="0">
+      <c r="C146" s="7" t="s">
         <v>629</v>
       </c>
-      <c r="C141" s="7" t="s">
+      <c r="D146" s="6" t="s">
         <v>630</v>
       </c>
-      <c r="D141" s="6" t="s">
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A142" t="s" s="0">
+      <c r="B147" t="s">
         <v>632</v>
       </c>
-      <c r="B142" t="s" s="0">
+      <c r="C147" s="7" t="s">
         <v>633</v>
       </c>
-      <c r="C142" s="7" t="s">
+      <c r="D147" s="6" t="s">
         <v>634</v>
       </c>
-      <c r="D142" s="6" t="s">
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A143" t="s" s="0">
+      <c r="B148" t="s">
         <v>636</v>
       </c>
-      <c r="B143" t="s" s="0">
+      <c r="C148" s="7" t="s">
         <v>637</v>
       </c>
-      <c r="C143" s="7" t="s">
+      <c r="D148" s="6" t="s">
         <v>638</v>
       </c>
-      <c r="D143" s="6" t="s">
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
         <v>639</v>
       </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A144" t="s" s="0">
+      <c r="B149" t="s">
         <v>640</v>
       </c>
-      <c r="B144" t="s" s="0">
+      <c r="C149" s="7" t="s">
         <v>641</v>
       </c>
-      <c r="C144" s="7" t="s">
+      <c r="D149" s="6" t="s">
         <v>642</v>
       </c>
-      <c r="D144" s="6" t="s">
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
         <v>643</v>
       </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A145" t="s" s="0">
+      <c r="B150" t="s">
         <v>644</v>
       </c>
-      <c r="B145" t="s" s="0">
+      <c r="C150" s="7" t="s">
         <v>645</v>
       </c>
-      <c r="C145" s="7" t="s">
+      <c r="D150" s="6" t="s">
         <v>646</v>
       </c>
-      <c r="D145" s="6" t="s">
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
         <v>647</v>
       </c>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A146" t="s" s="0">
+      <c r="B151" t="s">
         <v>648</v>
       </c>
-      <c r="B146" t="s" s="0">
+      <c r="C151" s="7" t="s">
         <v>649</v>
       </c>
-      <c r="C146" s="7" t="s">
+      <c r="D151" s="6" t="s">
         <v>650</v>
       </c>
-      <c r="D146" s="6" t="s">
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
         <v>651</v>
       </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A147" t="s" s="0">
+      <c r="B152" t="s">
         <v>652</v>
       </c>
-      <c r="B147" t="s" s="0">
+      <c r="C152" s="7" t="s">
         <v>653</v>
       </c>
-      <c r="C147" s="7" t="s">
+      <c r="D152" s="6" t="s">
         <v>654</v>
       </c>
-      <c r="D147" s="6" t="s">
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B153" t="s">
         <v>655</v>
       </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A148" t="s" s="0">
+      <c r="C153" s="7" t="s">
         <v>656</v>
       </c>
-      <c r="B148" t="s" s="0">
+      <c r="D153" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="C148" s="7" t="s">
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B154" t="s">
         <v>658</v>
       </c>
-      <c r="D148" s="6" t="s">
+      <c r="C154" s="7" t="s">
         <v>659</v>
       </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A149" t="s" s="0">
+      <c r="D154" s="6" t="s">
         <v>660</v>
       </c>
-      <c r="B149" t="s" s="0">
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B155" t="s">
         <v>661</v>
       </c>
-      <c r="C149" s="7" t="s">
+      <c r="C155" s="7" t="s">
         <v>662</v>
       </c>
-      <c r="D149" s="6" t="s">
+      <c r="D155" s="6" t="s">
         <v>663</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A150" t="s" s="0">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B156" t="s">
         <v>664</v>
       </c>
-      <c r="B150" t="s" s="0">
+      <c r="C156" s="7" t="s">
         <v>665</v>
       </c>
-      <c r="C150" s="7" t="s">
+      <c r="D156" s="6" t="s">
         <v>666</v>
       </c>
-      <c r="D150" s="6" t="s">
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B157" t="s">
         <v>667</v>
       </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A151" t="s" s="0">
+      <c r="C157" s="7" t="s">
         <v>668</v>
       </c>
-      <c r="B151" t="s" s="0">
+      <c r="D157" s="6" t="s">
         <v>669</v>
       </c>
-      <c r="C151" s="7" t="s">
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B158" t="s">
         <v>670</v>
       </c>
-      <c r="D151" s="6" t="s">
+      <c r="C158" s="7" t="s">
         <v>671</v>
       </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A152" t="s" s="0">
+      <c r="D158" s="6" t="s">
         <v>672</v>
-      </c>
-      <c r="B152" t="s" s="0">
-        <v>673</v>
-      </c>
-      <c r="C152" s="7" t="s">
-        <v>674</v>
-      </c>
-      <c r="D152" s="6" t="s">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B153" t="s" s="0">
-        <v>676</v>
-      </c>
-      <c r="C153" s="7" t="s">
-        <v>677</v>
-      </c>
-      <c r="D153" s="6" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B154" t="s" s="0">
-        <v>679</v>
-      </c>
-      <c r="C154" s="7" t="s">
-        <v>680</v>
-      </c>
-      <c r="D154" s="6" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B155" t="s" s="0">
-        <v>682</v>
-      </c>
-      <c r="C155" s="7" t="s">
-        <v>683</v>
-      </c>
-      <c r="D155" s="6" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B156" t="s" s="0">
-        <v>685</v>
-      </c>
-      <c r="C156" s="7" t="s">
-        <v>686</v>
-      </c>
-      <c r="D156" s="6" t="s">
-        <v>687</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B157" t="s" s="0">
-        <v>688</v>
-      </c>
-      <c r="C157" s="7" t="s">
-        <v>689</v>
-      </c>
-      <c r="D157" s="6" t="s">
-        <v>690</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B158" t="s" s="0">
-        <v>691</v>
-      </c>
-      <c r="C158" s="7" t="s">
-        <v>692</v>
-      </c>
-      <c r="D158" s="6" t="s">
-        <v>693</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C159" s="7" t="s">
-        <v>694</v>
+        <v>673</v>
       </c>
       <c r="D159" s="6" t="s">
-        <v>695</v>
+        <v>674</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C160" s="7" t="s">
-        <v>696</v>
+        <v>675</v>
       </c>
       <c r="D160" s="6" t="s">
-        <v>697</v>
+        <v>676</v>
       </c>
     </row>
     <row r="161" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C161" s="7" t="s">
-        <v>698</v>
+        <v>677</v>
       </c>
       <c r="D161" s="6" t="s">
-        <v>699</v>
+        <v>678</v>
       </c>
     </row>
     <row r="162" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C162" s="7" t="s">
-        <v>700</v>
+        <v>679</v>
       </c>
       <c r="D162" s="6" t="s">
-        <v>701</v>
+        <v>680</v>
       </c>
     </row>
     <row r="163" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C163" s="7" t="s">
-        <v>702</v>
+        <v>681</v>
       </c>
       <c r="D163" s="6" t="s">
-        <v>703</v>
+        <v>682</v>
       </c>
     </row>
     <row r="164" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C164" s="7" t="s">
-        <v>704</v>
+        <v>683</v>
       </c>
       <c r="D164" s="6" t="s">
-        <v>705</v>
+        <v>684</v>
       </c>
     </row>
     <row r="165" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C165" s="7" t="s">
-        <v>706</v>
+        <v>685</v>
       </c>
       <c r="D165" s="6" t="s">
-        <v>707</v>
+        <v>686</v>
       </c>
     </row>
     <row r="166" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C166" s="7" t="s">
-        <v>708</v>
+        <v>687</v>
       </c>
       <c r="D166" s="6" t="s">
-        <v>709</v>
+        <v>688</v>
       </c>
     </row>
     <row r="167" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C167" s="7" t="s">
-        <v>710</v>
+        <v>689</v>
       </c>
       <c r="D167" s="6" t="s">
-        <v>711</v>
+        <v>690</v>
       </c>
     </row>
     <row r="168" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C168" s="7" t="s">
-        <v>712</v>
+        <v>691</v>
       </c>
       <c r="D168" s="6" t="s">
-        <v>713</v>
+        <v>692</v>
       </c>
     </row>
     <row r="169" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C169" s="7" t="s">
-        <v>714</v>
+        <v>693</v>
       </c>
       <c r="D169" s="6" t="s">
-        <v>715</v>
+        <v>694</v>
       </c>
     </row>
     <row r="170" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C170" s="7" t="s">
-        <v>716</v>
+        <v>695</v>
       </c>
       <c r="D170" s="6" t="s">
-        <v>717</v>
+        <v>696</v>
       </c>
     </row>
     <row r="171" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D171" s="6" t="s">
-        <v>718</v>
+        <v>697</v>
       </c>
     </row>
     <row r="172" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D172" s="6" t="s">
-        <v>719</v>
+        <v>698</v>
       </c>
     </row>
     <row r="173" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D173" s="6" t="s">
-        <v>720</v>
+        <v>699</v>
       </c>
     </row>
     <row r="174" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D174" s="6" t="s">
-        <v>721</v>
+        <v>700</v>
       </c>
     </row>
     <row r="175" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D175" s="6" t="s">
-        <v>722</v>
+        <v>701</v>
       </c>
     </row>
     <row r="176" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D176" s="6" t="s">
-        <v>723</v>
+        <v>702</v>
       </c>
     </row>
     <row r="177" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D177" s="6" t="s">
-        <v>724</v>
+        <v>703</v>
       </c>
     </row>
     <row r="178" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D178" s="6" t="s">
-        <v>725</v>
+        <v>704</v>
       </c>
     </row>
     <row r="179" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D179" s="6" t="s">
-        <v>726</v>
+        <v>705</v>
       </c>
     </row>
     <row r="180" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D180" s="6" t="s">
-        <v>727</v>
+        <v>706</v>
       </c>
     </row>
     <row r="181" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D181" s="6" t="s">
-        <v>728</v>
+        <v>707</v>
       </c>
     </row>
     <row r="182" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D182" s="6" t="s">
-        <v>729</v>
+        <v>708</v>
       </c>
     </row>
     <row r="183" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D183" s="6" t="s">
-        <v>730</v>
+        <v>709</v>
       </c>
     </row>
     <row r="184" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D184" s="6" t="s">
-        <v>731</v>
+        <v>710</v>
       </c>
     </row>
     <row r="185" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D185" s="6" t="s">
-        <v>732</v>
+        <v>711</v>
       </c>
     </row>
     <row r="186" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D186" s="6" t="s">
-        <v>733</v>
+        <v>712</v>
       </c>
     </row>
     <row r="187" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D187" s="6" t="s">
-        <v>734</v>
+        <v>713</v>
       </c>
     </row>
     <row r="188" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D188" s="6" t="s">
-        <v>735</v>
+        <v>714</v>
       </c>
     </row>
     <row r="189" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D189" s="6" t="s">
-        <v>736</v>
+        <v>715</v>
       </c>
     </row>
     <row r="190" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D190" s="6" t="s">
-        <v>737</v>
+        <v>716</v>
       </c>
     </row>
     <row r="191" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D191" s="6" t="s">
-        <v>738</v>
+        <v>717</v>
       </c>
     </row>
     <row r="192" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D192" s="6" t="s">
-        <v>739</v>
+        <v>718</v>
       </c>
     </row>
     <row r="193" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D193" s="6" t="s">
-        <v>740</v>
+        <v>719</v>
       </c>
     </row>
     <row r="194" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D194" s="6" t="s">
-        <v>741</v>
+        <v>720</v>
       </c>
     </row>
     <row r="195" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D195" s="6" t="s">
-        <v>742</v>
+        <v>721</v>
       </c>
     </row>
     <row r="196" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D196" s="6" t="s">
-        <v>743</v>
+        <v>722</v>
       </c>
     </row>
     <row r="197" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D197" s="6" t="s">
-        <v>744</v>
+        <v>723</v>
       </c>
     </row>
     <row r="198" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D198" s="6" t="s">
-        <v>745</v>
+        <v>724</v>
       </c>
     </row>
     <row r="199" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D199" s="6" t="s">
-        <v>746</v>
+        <v>725</v>
       </c>
     </row>
     <row r="200" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D200" s="6" t="s">
-        <v>747</v>
+        <v>726</v>
       </c>
     </row>
     <row r="201" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D201" s="6" t="s">
-        <v>748</v>
+        <v>727</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated line of code for add pet_others scenario,pet name
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13980" windowHeight="2810" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13980" windowHeight="3150" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
@@ -12,12 +12,12 @@
     <sheet name="ADD_PET" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A28:G34"/>
+  <oleSize ref="A1:D9"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="743">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -2246,37 +2246,12 @@
   </si>
   <si>
     <t>FENAMV</t>
-  </si>
-  <si>
-    <t>Charlie77</t>
-  </si>
-  <si>
-    <t>Milo54</t>
-  </si>
-  <si>
-    <t>Taffy52</t>
-  </si>
-  <si>
-    <t>Cutie42</t>
-  </si>
-  <si>
-    <t>Cinder42</t>
-  </si>
-  <si>
-    <t>pony34</t>
-  </si>
-  <si>
-    <t>fury26</t>
-  </si>
-  <si>
-    <t>Sheep27</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2331,28 +2306,27 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2659,21 +2633,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:K119"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="17.81640625"/>
-    <col min="2" max="2" customWidth="true" style="1" width="15.0"/>
-    <col min="3" max="3" customWidth="true" style="1" width="15.36328125"/>
-    <col min="4" max="4" customWidth="true" style="1" width="17.453125"/>
-    <col min="5" max="5" customWidth="true" style="1" width="16.6328125"/>
-    <col min="6" max="6" customWidth="true" style="1" width="18.0"/>
-    <col min="7" max="7" customWidth="true" style="1" width="17.26953125"/>
-    <col min="8" max="8" customWidth="true" style="1" width="18.1796875"/>
-    <col min="9" max="9" customWidth="true" style="1" width="18.36328125"/>
-    <col min="10" max="10" customWidth="true" style="1" width="17.453125"/>
-    <col min="11" max="11" customWidth="true" style="1" width="17.36328125"/>
-    <col min="12" max="16384" style="1" width="8.7265625"/>
+    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -2709,24 +2683,24 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="15" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="11">
+      <c r="A3" s="10" t="s">
         <v>728</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -2735,15 +2709,15 @@
       <c r="C3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s" s="14">
+      <c r="D3" s="13" t="s">
         <v>737</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="16" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="1">
+      <c r="A4" s="1" t="s">
         <v>729</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -2752,15 +2726,15 @@
       <c r="C4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s" s="1">
+      <c r="D4" s="1" t="s">
         <v>738</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="17" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" t="s" s="1">
+      <c r="A5" s="1" t="s">
         <v>730</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -2769,7 +2743,7 @@
       <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D5" t="s" s="1">
+      <c r="D5" s="1" t="s">
         <v>739</v>
       </c>
       <c r="E5" s="1" t="s">
@@ -2777,16 +2751,16 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" t="s" s="1">
+      <c r="A6" s="1" t="s">
         <v>731</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s" s="1">
+      <c r="C6" s="1" t="s">
         <v>734</v>
       </c>
-      <c r="D6" t="s" s="1">
+      <c r="D6" s="1" t="s">
         <v>740</v>
       </c>
       <c r="E6" s="1" t="s">
@@ -2794,16 +2768,16 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" t="s" s="1">
+      <c r="A7" s="1" t="s">
         <v>732</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s" s="1">
+      <c r="C7" s="1" t="s">
         <v>735</v>
       </c>
-      <c r="D7" t="s" s="1">
+      <c r="D7" s="1" t="s">
         <v>741</v>
       </c>
       <c r="E7" s="1" t="s">
@@ -2811,16 +2785,16 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" t="s" s="1">
+      <c r="A8" s="1" t="s">
         <v>733</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C8" t="s" s="1">
+      <c r="C8" s="1" t="s">
         <v>736</v>
       </c>
-      <c r="D8" t="s" s="1">
+      <c r="D8" s="1" t="s">
         <v>742</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -2969,88 +2943,80 @@
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="26.90625"/>
-    <col min="2" max="2" customWidth="true" width="29.453125"/>
-    <col min="3" max="3" customWidth="true" width="35.6328125"/>
-    <col min="4" max="4" customWidth="true" width="30.90625"/>
-    <col min="5" max="5" customWidth="true" width="32.7265625"/>
-    <col min="6" max="6" customWidth="true" width="32.1796875"/>
-    <col min="7" max="7" customWidth="true" width="33.6328125"/>
-    <col min="8" max="8" customWidth="true" width="31.26953125"/>
+    <col min="1" max="1" width="26.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" customWidth="1"/>
+    <col min="4" max="4" width="30.90625" customWidth="1"/>
+    <col min="5" max="5" width="32.7265625" customWidth="1"/>
+    <col min="6" max="6" width="32.1796875" customWidth="1"/>
+    <col min="7" max="7" width="33.6328125" customWidth="1"/>
+    <col min="8" max="8" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>37</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>38</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>39</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>40</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>42</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>42</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>42</v>
       </c>
-      <c r="D2" t="s" s="0">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="B3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="C3" t="s">
         <v>42</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="D3" t="s">
         <v>42</v>
       </c>
-      <c r="D3" t="s" s="0">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="B4" t="s">
         <v>42</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="D4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D5" t="s" s="0">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D6" t="s" s="0">
-        <v>42</v>
-      </c>
-    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3062,2469 +3028,2469 @@
   <dimension ref="A1:H201"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.08984375"/>
-    <col min="2" max="2" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" customWidth="true" width="17.36328125"/>
-    <col min="4" max="5" customWidth="true" width="17.26953125"/>
-    <col min="6" max="6" customWidth="true" width="17.1796875"/>
-    <col min="7" max="7" customWidth="true" width="15.36328125"/>
-    <col min="8" max="8" customWidth="true" width="17.1796875"/>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="4" max="5" width="17.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>44</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>45</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>46</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>47</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>48</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>49</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>51</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>52</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>55</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>56</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>59</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>60</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>63</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>64</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>67</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>68</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>71</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s">
         <v>72</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>75</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="B8" t="s">
         <v>76</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="5" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>79</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="B9" t="s">
         <v>80</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="5" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" t="s" s="0">
+      <c r="A10" t="s">
         <v>83</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="B10" t="s">
         <v>84</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="5" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" t="s" s="0">
+      <c r="A11" t="s">
         <v>87</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="B11" t="s">
         <v>88</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="5" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" t="s" s="0">
+      <c r="A12" t="s">
         <v>91</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="B12" t="s">
         <v>92</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="5" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" t="s" s="0">
+      <c r="A13" t="s">
         <v>95</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="B13" t="s">
         <v>96</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="5" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" t="s" s="0">
+      <c r="A14" t="s">
         <v>99</v>
       </c>
-      <c r="B14" t="s" s="0">
+      <c r="B14" t="s">
         <v>100</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="5" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" t="s" s="0">
+      <c r="A15" t="s">
         <v>103</v>
       </c>
-      <c r="B15" t="s" s="0">
+      <c r="B15" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="5" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" t="s" s="0">
+      <c r="A16" t="s">
         <v>107</v>
       </c>
-      <c r="B16" t="s" s="0">
+      <c r="B16" t="s">
         <v>108</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="5" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" t="s" s="0">
+      <c r="A17" t="s">
         <v>111</v>
       </c>
-      <c r="B17" t="s" s="0">
+      <c r="B17" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="5" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" t="s" s="0">
+      <c r="A18" t="s">
         <v>115</v>
       </c>
-      <c r="B18" t="s" s="0">
+      <c r="B18" t="s">
         <v>116</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="5" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" t="s" s="0">
+      <c r="A19" t="s">
         <v>119</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="B19" t="s">
         <v>120</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="5" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" t="s" s="0">
+      <c r="A20" t="s">
         <v>123</v>
       </c>
-      <c r="B20" t="s" s="0">
+      <c r="B20" t="s">
         <v>124</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="5" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" t="s" s="0">
+      <c r="A21" t="s">
         <v>127</v>
       </c>
-      <c r="B21" t="s" s="0">
+      <c r="B21" t="s">
         <v>128</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="5" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" t="s" s="0">
+      <c r="A22" t="s">
         <v>131</v>
       </c>
-      <c r="B22" t="s" s="0">
+      <c r="B22" t="s">
         <v>132</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="5" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" t="s" s="0">
+      <c r="A23" t="s">
         <v>135</v>
       </c>
-      <c r="B23" t="s" s="0">
+      <c r="B23" t="s">
         <v>136</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="5" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" t="s" s="0">
+      <c r="A24" t="s">
         <v>139</v>
       </c>
-      <c r="B24" t="s" s="0">
+      <c r="B24" t="s">
         <v>140</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="5" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" t="s" s="0">
+      <c r="A25" t="s">
         <v>143</v>
       </c>
-      <c r="B25" t="s" s="0">
+      <c r="B25" t="s">
         <v>144</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="5" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" t="s" s="0">
+      <c r="A26" t="s">
         <v>147</v>
       </c>
-      <c r="B26" t="s" s="0">
+      <c r="B26" t="s">
         <v>148</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="5" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" t="s" s="0">
+      <c r="A27" t="s">
         <v>151</v>
       </c>
-      <c r="B27" t="s" s="0">
+      <c r="B27" t="s">
         <v>152</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="5" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" t="s" s="0">
+      <c r="A28" t="s">
         <v>155</v>
       </c>
-      <c r="B28" t="s" s="0">
+      <c r="B28" t="s">
         <v>156</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="5" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" t="s" s="0">
+      <c r="A29" t="s">
         <v>159</v>
       </c>
-      <c r="B29" t="s" s="0">
+      <c r="B29" t="s">
         <v>160</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="5" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" t="s" s="0">
+      <c r="A30" t="s">
         <v>163</v>
       </c>
-      <c r="B30" t="s" s="0">
+      <c r="B30" t="s">
         <v>164</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="5" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" t="s" s="0">
+      <c r="A31" t="s">
         <v>167</v>
       </c>
-      <c r="B31" t="s" s="0">
+      <c r="B31" t="s">
         <v>168</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="5" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" t="s" s="0">
+      <c r="A32" t="s">
         <v>171</v>
       </c>
-      <c r="B32" t="s" s="0">
+      <c r="B32" t="s">
         <v>172</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="5" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" t="s" s="0">
+      <c r="A33" t="s">
         <v>175</v>
       </c>
-      <c r="B33" t="s" s="0">
+      <c r="B33" t="s">
         <v>176</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" s="5" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" t="s" s="0">
+      <c r="A34" t="s">
         <v>179</v>
       </c>
-      <c r="B34" t="s" s="0">
+      <c r="B34" t="s">
         <v>180</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="D34" s="5" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" t="s" s="0">
+      <c r="A35" t="s">
         <v>183</v>
       </c>
-      <c r="B35" t="s" s="0">
+      <c r="B35" t="s">
         <v>184</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D35" s="5" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" t="s" s="0">
+      <c r="A36" t="s">
         <v>187</v>
       </c>
-      <c r="B36" t="s" s="0">
+      <c r="B36" t="s">
         <v>188</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="C36" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" s="5" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" t="s" s="0">
+      <c r="A37" t="s">
         <v>191</v>
       </c>
-      <c r="B37" t="s" s="0">
+      <c r="B37" t="s">
         <v>192</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C37" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D37" s="5" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" t="s" s="0">
+      <c r="A38" t="s">
         <v>195</v>
       </c>
-      <c r="B38" t="s" s="0">
+      <c r="B38" t="s">
         <v>196</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D38" s="5" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" t="s" s="0">
+      <c r="A39" t="s">
         <v>199</v>
       </c>
-      <c r="B39" t="s" s="0">
+      <c r="B39" t="s">
         <v>200</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C39" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D39" s="5" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" t="s" s="0">
+      <c r="A40" t="s">
         <v>203</v>
       </c>
-      <c r="B40" t="s" s="0">
+      <c r="B40" t="s">
         <v>204</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="D40" s="5" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" t="s" s="0">
+      <c r="A41" t="s">
         <v>207</v>
       </c>
-      <c r="B41" t="s" s="0">
+      <c r="B41" t="s">
         <v>208</v>
       </c>
-      <c r="C41" s="7" t="s">
+      <c r="C41" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="D41" s="5" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" t="s" s="0">
+      <c r="A42" t="s">
         <v>211</v>
       </c>
-      <c r="B42" t="s" s="0">
+      <c r="B42" t="s">
         <v>212</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D42" s="5" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" t="s" s="0">
+      <c r="A43" t="s">
         <v>215</v>
       </c>
-      <c r="B43" t="s" s="0">
+      <c r="B43" t="s">
         <v>216</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="C43" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="D43" s="5" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" t="s" s="0">
+      <c r="A44" t="s">
         <v>219</v>
       </c>
-      <c r="B44" t="s" s="0">
+      <c r="B44" t="s">
         <v>220</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="C44" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="D44" s="5" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" t="s" s="0">
+      <c r="A45" t="s">
         <v>223</v>
       </c>
-      <c r="B45" t="s" s="0">
+      <c r="B45" t="s">
         <v>224</v>
       </c>
-      <c r="C45" s="7" t="s">
+      <c r="C45" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D45" s="5" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" t="s" s="0">
+      <c r="A46" t="s">
         <v>227</v>
       </c>
-      <c r="B46" t="s" s="0">
+      <c r="B46" t="s">
         <v>228</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="C46" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="D46" s="5" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A47" t="s" s="0">
+      <c r="A47" t="s">
         <v>231</v>
       </c>
-      <c r="B47" t="s" s="0">
+      <c r="B47" t="s">
         <v>232</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="C47" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="D47" s="6" t="s">
+      <c r="D47" s="5" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A48" t="s" s="0">
+      <c r="A48" t="s">
         <v>235</v>
       </c>
-      <c r="B48" t="s" s="0">
+      <c r="B48" t="s">
         <v>236</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="C48" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="D48" s="5" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" t="s" s="0">
+      <c r="A49" t="s">
         <v>239</v>
       </c>
-      <c r="B49" t="s" s="0">
+      <c r="B49" t="s">
         <v>240</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="C49" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="D49" s="5" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" t="s" s="0">
+      <c r="A50" t="s">
         <v>243</v>
       </c>
-      <c r="B50" t="s" s="0">
+      <c r="B50" t="s">
         <v>244</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="C50" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="D50" s="5" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" t="s" s="0">
+      <c r="A51" t="s">
         <v>247</v>
       </c>
-      <c r="B51" t="s" s="0">
+      <c r="B51" t="s">
         <v>248</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="C51" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="D51" s="6" t="s">
+      <c r="D51" s="5" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" t="s" s="0">
+      <c r="A52" t="s">
         <v>251</v>
       </c>
-      <c r="B52" t="s" s="0">
+      <c r="B52" t="s">
         <v>252</v>
       </c>
-      <c r="C52" s="7" t="s">
+      <c r="C52" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="D52" s="6" t="s">
+      <c r="D52" s="5" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" t="s" s="0">
+      <c r="A53" t="s">
         <v>255</v>
       </c>
-      <c r="B53" t="s" s="0">
+      <c r="B53" t="s">
         <v>256</v>
       </c>
-      <c r="C53" s="7" t="s">
+      <c r="C53" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="D53" s="6" t="s">
+      <c r="D53" s="5" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A54" t="s" s="0">
+      <c r="A54" t="s">
         <v>259</v>
       </c>
-      <c r="B54" t="s" s="0">
+      <c r="B54" t="s">
         <v>260</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="C54" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="D54" s="6" t="s">
+      <c r="D54" s="5" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A55" t="s" s="0">
+      <c r="A55" t="s">
         <v>263</v>
       </c>
-      <c r="B55" t="s" s="0">
+      <c r="B55" t="s">
         <v>264</v>
       </c>
-      <c r="C55" s="7" t="s">
+      <c r="C55" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="D55" s="6" t="s">
+      <c r="D55" s="5" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" t="s" s="0">
+      <c r="A56" t="s">
         <v>267</v>
       </c>
-      <c r="B56" t="s" s="0">
+      <c r="B56" t="s">
         <v>268</v>
       </c>
-      <c r="C56" s="7" t="s">
+      <c r="C56" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="D56" s="6" t="s">
+      <c r="D56" s="5" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" t="s" s="0">
+      <c r="A57" t="s">
         <v>271</v>
       </c>
-      <c r="B57" t="s" s="0">
+      <c r="B57" t="s">
         <v>272</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="C57" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="D57" s="6" t="s">
+      <c r="D57" s="5" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" t="s" s="0">
+      <c r="A58" t="s">
         <v>275</v>
       </c>
-      <c r="B58" t="s" s="0">
+      <c r="B58" t="s">
         <v>276</v>
       </c>
-      <c r="C58" s="7" t="s">
+      <c r="C58" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="D58" s="6" t="s">
+      <c r="D58" s="5" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" t="s" s="0">
+      <c r="A59" t="s">
         <v>279</v>
       </c>
-      <c r="B59" t="s" s="0">
+      <c r="B59" t="s">
         <v>280</v>
       </c>
-      <c r="C59" s="7" t="s">
+      <c r="C59" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="D59" s="6" t="s">
+      <c r="D59" s="5" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" t="s" s="0">
+      <c r="A60" t="s">
         <v>283</v>
       </c>
-      <c r="B60" t="s" s="0">
+      <c r="B60" t="s">
         <v>284</v>
       </c>
-      <c r="C60" s="7" t="s">
+      <c r="C60" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="D60" s="6" t="s">
+      <c r="D60" s="5" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" t="s" s="0">
+      <c r="A61" t="s">
         <v>287</v>
       </c>
-      <c r="B61" t="s" s="0">
+      <c r="B61" t="s">
         <v>288</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="C61" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="D61" s="6" t="s">
+      <c r="D61" s="5" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" t="s" s="0">
+      <c r="A62" t="s">
         <v>291</v>
       </c>
-      <c r="B62" t="s" s="0">
+      <c r="B62" t="s">
         <v>292</v>
       </c>
-      <c r="C62" s="7" t="s">
+      <c r="C62" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="D62" s="6" t="s">
+      <c r="D62" s="5" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A63" t="s" s="0">
+      <c r="A63" t="s">
         <v>295</v>
       </c>
-      <c r="B63" t="s" s="0">
+      <c r="B63" t="s">
         <v>296</v>
       </c>
-      <c r="C63" s="7" t="s">
+      <c r="C63" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="D63" s="6" t="s">
+      <c r="D63" s="5" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A64" t="s" s="0">
+      <c r="A64" t="s">
         <v>299</v>
       </c>
-      <c r="B64" t="s" s="0">
+      <c r="B64" t="s">
         <v>300</v>
       </c>
-      <c r="C64" s="7" t="s">
+      <c r="C64" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="D64" s="6" t="s">
+      <c r="D64" s="5" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" t="s" s="0">
+      <c r="A65" t="s">
         <v>303</v>
       </c>
-      <c r="B65" t="s" s="0">
+      <c r="B65" t="s">
         <v>304</v>
       </c>
-      <c r="C65" s="7" t="s">
+      <c r="C65" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="D65" s="6" t="s">
+      <c r="D65" s="5" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" t="s" s="0">
+      <c r="A66" t="s">
         <v>307</v>
       </c>
-      <c r="B66" t="s" s="0">
+      <c r="B66" t="s">
         <v>308</v>
       </c>
-      <c r="C66" s="7" t="s">
+      <c r="C66" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="D66" s="6" t="s">
+      <c r="D66" s="5" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A67" t="s" s="0">
+      <c r="A67" t="s">
         <v>311</v>
       </c>
-      <c r="B67" t="s" s="0">
+      <c r="B67" t="s">
         <v>312</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="C67" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="D67" s="6" t="s">
+      <c r="D67" s="5" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" t="s" s="0">
+      <c r="A68" t="s">
         <v>315</v>
       </c>
-      <c r="B68" t="s" s="0">
+      <c r="B68" t="s">
         <v>316</v>
       </c>
-      <c r="C68" s="7" t="s">
+      <c r="C68" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="D68" s="6" t="s">
+      <c r="D68" s="5" t="s">
         <v>318</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" t="s" s="0">
+      <c r="A69" t="s">
         <v>319</v>
       </c>
-      <c r="B69" t="s" s="0">
+      <c r="B69" t="s">
         <v>320</v>
       </c>
-      <c r="C69" s="7" t="s">
+      <c r="C69" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="D69" s="6" t="s">
+      <c r="D69" s="5" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" t="s" s="0">
+      <c r="A70" t="s">
         <v>323</v>
       </c>
-      <c r="B70" t="s" s="0">
+      <c r="B70" t="s">
         <v>324</v>
       </c>
-      <c r="C70" s="7" t="s">
+      <c r="C70" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="D70" s="6" t="s">
+      <c r="D70" s="5" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A71" t="s" s="0">
+      <c r="A71" t="s">
         <v>327</v>
       </c>
-      <c r="B71" t="s" s="0">
+      <c r="B71" t="s">
         <v>328</v>
       </c>
-      <c r="C71" s="7" t="s">
+      <c r="C71" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="D71" s="6" t="s">
+      <c r="D71" s="5" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A72" t="s" s="0">
+      <c r="A72" t="s">
         <v>331</v>
       </c>
-      <c r="B72" t="s" s="0">
+      <c r="B72" t="s">
         <v>332</v>
       </c>
-      <c r="C72" s="7" t="s">
+      <c r="C72" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="D72" s="6" t="s">
+      <c r="D72" s="5" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A73" t="s" s="0">
+      <c r="A73" t="s">
         <v>335</v>
       </c>
-      <c r="B73" t="s" s="0">
+      <c r="B73" t="s">
         <v>336</v>
       </c>
-      <c r="C73" s="7" t="s">
+      <c r="C73" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="D73" s="6" t="s">
+      <c r="D73" s="5" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" t="s" s="0">
+      <c r="A74" t="s">
         <v>339</v>
       </c>
-      <c r="B74" t="s" s="0">
+      <c r="B74" t="s">
         <v>340</v>
       </c>
-      <c r="C74" s="7" t="s">
+      <c r="C74" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="D74" s="6" t="s">
+      <c r="D74" s="5" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" t="s" s="0">
+      <c r="A75" t="s">
         <v>343</v>
       </c>
-      <c r="B75" t="s" s="0">
+      <c r="B75" t="s">
         <v>344</v>
       </c>
-      <c r="C75" s="7" t="s">
+      <c r="C75" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="D75" s="6" t="s">
+      <c r="D75" s="5" t="s">
         <v>346</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" t="s" s="0">
+      <c r="A76" t="s">
         <v>347</v>
       </c>
-      <c r="B76" t="s" s="0">
+      <c r="B76" t="s">
         <v>348</v>
       </c>
-      <c r="C76" s="7" t="s">
+      <c r="C76" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="D76" s="6" t="s">
+      <c r="D76" s="5" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A77" t="s" s="0">
+      <c r="A77" t="s">
         <v>351</v>
       </c>
-      <c r="B77" t="s" s="0">
+      <c r="B77" t="s">
         <v>352</v>
       </c>
-      <c r="C77" s="7" t="s">
+      <c r="C77" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="D77" s="6" t="s">
+      <c r="D77" s="5" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A78" t="s" s="0">
+      <c r="A78" t="s">
         <v>355</v>
       </c>
-      <c r="B78" t="s" s="0">
+      <c r="B78" t="s">
         <v>356</v>
       </c>
-      <c r="C78" s="7" t="s">
+      <c r="C78" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="D78" s="6" t="s">
+      <c r="D78" s="5" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A79" t="s" s="0">
+      <c r="A79" t="s">
         <v>359</v>
       </c>
-      <c r="B79" t="s" s="0">
+      <c r="B79" t="s">
         <v>360</v>
       </c>
-      <c r="C79" s="7" t="s">
+      <c r="C79" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="D79" s="6" t="s">
+      <c r="D79" s="5" t="s">
         <v>362</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A80" t="s" s="0">
+      <c r="A80" t="s">
         <v>363</v>
       </c>
-      <c r="B80" t="s" s="0">
+      <c r="B80" t="s">
         <v>364</v>
       </c>
-      <c r="C80" s="7" t="s">
+      <c r="C80" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="D80" s="6" t="s">
+      <c r="D80" s="5" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A81" t="s" s="0">
+      <c r="A81" t="s">
         <v>367</v>
       </c>
-      <c r="B81" t="s" s="0">
+      <c r="B81" t="s">
         <v>368</v>
       </c>
-      <c r="C81" s="7" t="s">
+      <c r="C81" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="D81" s="6" t="s">
+      <c r="D81" s="5" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" t="s" s="0">
+      <c r="A82" t="s">
         <v>371</v>
       </c>
-      <c r="B82" t="s" s="0">
+      <c r="B82" t="s">
         <v>372</v>
       </c>
-      <c r="C82" s="7" t="s">
+      <c r="C82" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="D82" s="6" t="s">
+      <c r="D82" s="5" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A83" t="s" s="0">
+      <c r="A83" t="s">
         <v>375</v>
       </c>
-      <c r="B83" t="s" s="0">
+      <c r="B83" t="s">
         <v>376</v>
       </c>
-      <c r="C83" s="7" t="s">
+      <c r="C83" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="D83" s="6" t="s">
+      <c r="D83" s="5" t="s">
         <v>378</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A84" t="s" s="0">
+      <c r="A84" t="s">
         <v>379</v>
       </c>
-      <c r="B84" t="s" s="0">
+      <c r="B84" t="s">
         <v>380</v>
       </c>
-      <c r="C84" s="7" t="s">
+      <c r="C84" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="D84" s="6" t="s">
+      <c r="D84" s="5" t="s">
         <v>382</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A85" t="s" s="0">
+      <c r="A85" t="s">
         <v>383</v>
       </c>
-      <c r="B85" t="s" s="0">
+      <c r="B85" t="s">
         <v>384</v>
       </c>
-      <c r="C85" s="7" t="s">
+      <c r="C85" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="D85" s="6" t="s">
+      <c r="D85" s="5" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A86" t="s" s="0">
+      <c r="A86" t="s">
         <v>387</v>
       </c>
-      <c r="B86" t="s" s="0">
+      <c r="B86" t="s">
         <v>388</v>
       </c>
-      <c r="C86" s="7" t="s">
+      <c r="C86" s="6" t="s">
         <v>389</v>
       </c>
-      <c r="D86" s="6" t="s">
+      <c r="D86" s="5" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A87" t="s" s="0">
+      <c r="A87" t="s">
         <v>391</v>
       </c>
-      <c r="B87" t="s" s="0">
+      <c r="B87" t="s">
         <v>392</v>
       </c>
-      <c r="C87" s="7" t="s">
+      <c r="C87" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="D87" s="6" t="s">
+      <c r="D87" s="5" t="s">
         <v>394</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A88" t="s" s="0">
+      <c r="A88" t="s">
         <v>395</v>
       </c>
-      <c r="B88" t="s" s="0">
+      <c r="B88" t="s">
         <v>396</v>
       </c>
-      <c r="C88" s="7" t="s">
+      <c r="C88" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="D88" s="6" t="s">
+      <c r="D88" s="5" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A89" t="s" s="0">
+      <c r="A89" t="s">
         <v>399</v>
       </c>
-      <c r="B89" t="s" s="0">
+      <c r="B89" t="s">
         <v>400</v>
       </c>
-      <c r="C89" s="7" t="s">
+      <c r="C89" s="6" t="s">
         <v>401</v>
       </c>
-      <c r="D89" s="6" t="s">
+      <c r="D89" s="5" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A90" t="s" s="0">
+      <c r="A90" t="s">
         <v>403</v>
       </c>
-      <c r="B90" t="s" s="0">
+      <c r="B90" t="s">
         <v>404</v>
       </c>
-      <c r="C90" s="7" t="s">
+      <c r="C90" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="D90" s="6" t="s">
+      <c r="D90" s="5" t="s">
         <v>406</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A91" t="s" s="0">
+      <c r="A91" t="s">
         <v>407</v>
       </c>
-      <c r="B91" t="s" s="0">
+      <c r="B91" t="s">
         <v>408</v>
       </c>
-      <c r="C91" s="7" t="s">
+      <c r="C91" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="D91" s="6" t="s">
+      <c r="D91" s="5" t="s">
         <v>410</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A92" t="s" s="0">
+      <c r="A92" t="s">
         <v>411</v>
       </c>
-      <c r="B92" t="s" s="0">
+      <c r="B92" t="s">
         <v>412</v>
       </c>
-      <c r="C92" s="7" t="s">
+      <c r="C92" s="6" t="s">
         <v>413</v>
       </c>
-      <c r="D92" s="6" t="s">
+      <c r="D92" s="5" t="s">
         <v>414</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A93" t="s" s="0">
+      <c r="A93" t="s">
         <v>415</v>
       </c>
-      <c r="B93" t="s" s="0">
+      <c r="B93" t="s">
         <v>416</v>
       </c>
-      <c r="C93" s="7" t="s">
+      <c r="C93" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="D93" s="6" t="s">
+      <c r="D93" s="5" t="s">
         <v>418</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A94" t="s" s="0">
+      <c r="A94" t="s">
         <v>419</v>
       </c>
-      <c r="B94" t="s" s="0">
+      <c r="B94" t="s">
         <v>420</v>
       </c>
-      <c r="C94" s="7" t="s">
+      <c r="C94" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="D94" s="6" t="s">
+      <c r="D94" s="5" t="s">
         <v>422</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A95" t="s" s="0">
+      <c r="A95" t="s">
         <v>423</v>
       </c>
-      <c r="B95" t="s" s="0">
+      <c r="B95" t="s">
         <v>424</v>
       </c>
-      <c r="C95" s="7" t="s">
+      <c r="C95" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="D95" s="6" t="s">
+      <c r="D95" s="5" t="s">
         <v>426</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A96" t="s" s="0">
+      <c r="A96" t="s">
         <v>427</v>
       </c>
-      <c r="B96" t="s" s="0">
+      <c r="B96" t="s">
         <v>428</v>
       </c>
-      <c r="C96" s="7" t="s">
+      <c r="C96" s="6" t="s">
         <v>429</v>
       </c>
-      <c r="D96" s="6" t="s">
+      <c r="D96" s="5" t="s">
         <v>430</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A97" t="s" s="0">
+      <c r="A97" t="s">
         <v>431</v>
       </c>
-      <c r="B97" t="s" s="0">
+      <c r="B97" t="s">
         <v>432</v>
       </c>
-      <c r="C97" s="7" t="s">
+      <c r="C97" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="D97" s="6" t="s">
+      <c r="D97" s="5" t="s">
         <v>434</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A98" t="s" s="0">
+      <c r="A98" t="s">
         <v>435</v>
       </c>
-      <c r="B98" t="s" s="0">
+      <c r="B98" t="s">
         <v>436</v>
       </c>
-      <c r="C98" s="7" t="s">
+      <c r="C98" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="D98" s="6" t="s">
+      <c r="D98" s="5" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A99" t="s" s="0">
+      <c r="A99" t="s">
         <v>439</v>
       </c>
-      <c r="B99" t="s" s="0">
+      <c r="B99" t="s">
         <v>440</v>
       </c>
-      <c r="C99" s="7" t="s">
+      <c r="C99" s="6" t="s">
         <v>441</v>
       </c>
-      <c r="D99" s="6" t="s">
+      <c r="D99" s="5" t="s">
         <v>442</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A100" t="s" s="0">
+      <c r="A100" t="s">
         <v>443</v>
       </c>
-      <c r="B100" t="s" s="0">
+      <c r="B100" t="s">
         <v>444</v>
       </c>
-      <c r="C100" s="7" t="s">
+      <c r="C100" s="6" t="s">
         <v>445</v>
       </c>
-      <c r="D100" s="6" t="s">
+      <c r="D100" s="5" t="s">
         <v>446</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A101" t="s" s="0">
+      <c r="A101" t="s">
         <v>447</v>
       </c>
-      <c r="B101" t="s" s="0">
+      <c r="B101" t="s">
         <v>448</v>
       </c>
-      <c r="C101" s="7" t="s">
+      <c r="C101" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="D101" s="6" t="s">
+      <c r="D101" s="5" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A102" t="s" s="0">
+      <c r="A102" t="s">
         <v>451</v>
       </c>
-      <c r="B102" t="s" s="0">
+      <c r="B102" t="s">
         <v>452</v>
       </c>
-      <c r="C102" s="7" t="s">
+      <c r="C102" s="6" t="s">
         <v>453</v>
       </c>
-      <c r="D102" s="6" t="s">
+      <c r="D102" s="5" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A103" t="s" s="0">
+      <c r="A103" t="s">
         <v>455</v>
       </c>
-      <c r="B103" t="s" s="0">
+      <c r="B103" t="s">
         <v>456</v>
       </c>
-      <c r="C103" s="7" t="s">
+      <c r="C103" s="6" t="s">
         <v>457</v>
       </c>
-      <c r="D103" s="6" t="s">
+      <c r="D103" s="5" t="s">
         <v>458</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A104" t="s" s="0">
+      <c r="A104" t="s">
         <v>459</v>
       </c>
-      <c r="B104" t="s" s="0">
+      <c r="B104" t="s">
         <v>460</v>
       </c>
-      <c r="C104" s="7" t="s">
+      <c r="C104" s="6" t="s">
         <v>461</v>
       </c>
-      <c r="D104" s="6" t="s">
+      <c r="D104" s="5" t="s">
         <v>462</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A105" t="s" s="0">
+      <c r="A105" t="s">
         <v>463</v>
       </c>
-      <c r="B105" t="s" s="0">
+      <c r="B105" t="s">
         <v>464</v>
       </c>
-      <c r="C105" s="7" t="s">
+      <c r="C105" s="6" t="s">
         <v>465</v>
       </c>
-      <c r="D105" s="6" t="s">
+      <c r="D105" s="5" t="s">
         <v>466</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A106" t="s" s="0">
+      <c r="A106" t="s">
         <v>467</v>
       </c>
-      <c r="B106" t="s" s="0">
+      <c r="B106" t="s">
         <v>468</v>
       </c>
-      <c r="C106" s="7" t="s">
+      <c r="C106" s="6" t="s">
         <v>469</v>
       </c>
-      <c r="D106" s="6" t="s">
+      <c r="D106" s="5" t="s">
         <v>470</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A107" t="s" s="0">
+      <c r="A107" t="s">
         <v>471</v>
       </c>
-      <c r="B107" t="s" s="0">
+      <c r="B107" t="s">
         <v>472</v>
       </c>
-      <c r="C107" s="7" t="s">
+      <c r="C107" s="6" t="s">
         <v>473</v>
       </c>
-      <c r="D107" s="6" t="s">
+      <c r="D107" s="5" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A108" t="s" s="0">
+      <c r="A108" t="s">
         <v>475</v>
       </c>
-      <c r="B108" t="s" s="0">
+      <c r="B108" t="s">
         <v>476</v>
       </c>
-      <c r="C108" s="7" t="s">
+      <c r="C108" s="6" t="s">
         <v>477</v>
       </c>
-      <c r="D108" s="6" t="s">
+      <c r="D108" s="5" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A109" t="s" s="0">
+      <c r="A109" t="s">
         <v>479</v>
       </c>
-      <c r="B109" t="s" s="0">
+      <c r="B109" t="s">
         <v>480</v>
       </c>
-      <c r="C109" s="7" t="s">
+      <c r="C109" s="6" t="s">
         <v>481</v>
       </c>
-      <c r="D109" s="6" t="s">
+      <c r="D109" s="5" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A110" t="s" s="0">
+      <c r="A110" t="s">
         <v>483</v>
       </c>
-      <c r="B110" t="s" s="0">
+      <c r="B110" t="s">
         <v>484</v>
       </c>
-      <c r="C110" s="7" t="s">
+      <c r="C110" s="6" t="s">
         <v>485</v>
       </c>
-      <c r="D110" s="6" t="s">
+      <c r="D110" s="5" t="s">
         <v>486</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A111" t="s" s="0">
+      <c r="A111" t="s">
         <v>487</v>
       </c>
-      <c r="B111" t="s" s="0">
+      <c r="B111" t="s">
         <v>488</v>
       </c>
-      <c r="C111" s="7" t="s">
+      <c r="C111" s="6" t="s">
         <v>489</v>
       </c>
-      <c r="D111" s="6" t="s">
+      <c r="D111" s="5" t="s">
         <v>490</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A112" t="s" s="0">
+      <c r="A112" t="s">
         <v>491</v>
       </c>
-      <c r="B112" t="s" s="0">
+      <c r="B112" t="s">
         <v>492</v>
       </c>
-      <c r="C112" s="7" t="s">
+      <c r="C112" s="6" t="s">
         <v>493</v>
       </c>
-      <c r="D112" s="6" t="s">
+      <c r="D112" s="5" t="s">
         <v>494</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A113" t="s" s="0">
+      <c r="A113" t="s">
         <v>495</v>
       </c>
-      <c r="B113" t="s" s="0">
+      <c r="B113" t="s">
         <v>496</v>
       </c>
-      <c r="C113" s="7" t="s">
+      <c r="C113" s="6" t="s">
         <v>497</v>
       </c>
-      <c r="D113" s="6" t="s">
+      <c r="D113" s="5" t="s">
         <v>498</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A114" t="s" s="0">
+      <c r="A114" t="s">
         <v>499</v>
       </c>
-      <c r="B114" t="s" s="0">
+      <c r="B114" t="s">
         <v>500</v>
       </c>
-      <c r="C114" s="7" t="s">
+      <c r="C114" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="D114" s="6" t="s">
+      <c r="D114" s="5" t="s">
         <v>502</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A115" t="s" s="0">
+      <c r="A115" t="s">
         <v>503</v>
       </c>
-      <c r="B115" t="s" s="0">
+      <c r="B115" t="s">
         <v>504</v>
       </c>
-      <c r="C115" s="7" t="s">
+      <c r="C115" s="6" t="s">
         <v>505</v>
       </c>
-      <c r="D115" s="6" t="s">
+      <c r="D115" s="5" t="s">
         <v>506</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A116" t="s" s="0">
+      <c r="A116" t="s">
         <v>507</v>
       </c>
-      <c r="B116" t="s" s="0">
+      <c r="B116" t="s">
         <v>508</v>
       </c>
-      <c r="C116" s="7" t="s">
+      <c r="C116" s="6" t="s">
         <v>509</v>
       </c>
-      <c r="D116" s="6" t="s">
+      <c r="D116" s="5" t="s">
         <v>510</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A117" t="s" s="0">
+      <c r="A117" t="s">
         <v>511</v>
       </c>
-      <c r="B117" t="s" s="0">
+      <c r="B117" t="s">
         <v>512</v>
       </c>
-      <c r="C117" s="7" t="s">
+      <c r="C117" s="6" t="s">
         <v>513</v>
       </c>
-      <c r="D117" s="6" t="s">
+      <c r="D117" s="5" t="s">
         <v>514</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A118" t="s" s="0">
+      <c r="A118" t="s">
         <v>515</v>
       </c>
-      <c r="B118" t="s" s="0">
+      <c r="B118" t="s">
         <v>516</v>
       </c>
-      <c r="C118" s="7" t="s">
+      <c r="C118" s="6" t="s">
         <v>517</v>
       </c>
-      <c r="D118" s="6" t="s">
+      <c r="D118" s="5" t="s">
         <v>518</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A119" t="s" s="0">
+      <c r="A119" t="s">
         <v>519</v>
       </c>
-      <c r="B119" t="s" s="0">
+      <c r="B119" t="s">
         <v>520</v>
       </c>
-      <c r="C119" s="7" t="s">
+      <c r="C119" s="6" t="s">
         <v>521</v>
       </c>
-      <c r="D119" s="6" t="s">
+      <c r="D119" s="5" t="s">
         <v>522</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A120" t="s" s="0">
+      <c r="A120" t="s">
         <v>523</v>
       </c>
-      <c r="B120" t="s" s="0">
+      <c r="B120" t="s">
         <v>524</v>
       </c>
-      <c r="C120" s="7" t="s">
+      <c r="C120" s="6" t="s">
         <v>525</v>
       </c>
-      <c r="D120" s="6" t="s">
+      <c r="D120" s="5" t="s">
         <v>526</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A121" t="s" s="0">
+      <c r="A121" t="s">
         <v>527</v>
       </c>
-      <c r="B121" t="s" s="0">
+      <c r="B121" t="s">
         <v>528</v>
       </c>
-      <c r="C121" s="7" t="s">
+      <c r="C121" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="D121" s="6" t="s">
+      <c r="D121" s="5" t="s">
         <v>530</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A122" t="s" s="0">
+      <c r="A122" t="s">
         <v>531</v>
       </c>
-      <c r="B122" t="s" s="0">
+      <c r="B122" t="s">
         <v>532</v>
       </c>
-      <c r="C122" s="7" t="s">
+      <c r="C122" s="6" t="s">
         <v>533</v>
       </c>
-      <c r="D122" s="6" t="s">
+      <c r="D122" s="5" t="s">
         <v>534</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A123" t="s" s="0">
+      <c r="A123" t="s">
         <v>535</v>
       </c>
-      <c r="B123" t="s" s="0">
+      <c r="B123" t="s">
         <v>536</v>
       </c>
-      <c r="C123" s="7" t="s">
+      <c r="C123" s="6" t="s">
         <v>537</v>
       </c>
-      <c r="D123" s="6" t="s">
+      <c r="D123" s="5" t="s">
         <v>538</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A124" t="s" s="0">
+      <c r="A124" t="s">
         <v>539</v>
       </c>
-      <c r="B124" t="s" s="0">
+      <c r="B124" t="s">
         <v>540</v>
       </c>
-      <c r="C124" s="7" t="s">
+      <c r="C124" s="6" t="s">
         <v>541</v>
       </c>
-      <c r="D124" s="6" t="s">
+      <c r="D124" s="5" t="s">
         <v>542</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A125" t="s" s="0">
+      <c r="A125" t="s">
         <v>543</v>
       </c>
-      <c r="B125" t="s" s="0">
+      <c r="B125" t="s">
         <v>544</v>
       </c>
-      <c r="C125" s="7" t="s">
+      <c r="C125" s="6" t="s">
         <v>545</v>
       </c>
-      <c r="D125" s="6" t="s">
+      <c r="D125" s="5" t="s">
         <v>546</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A126" t="s" s="0">
+      <c r="A126" t="s">
         <v>547</v>
       </c>
-      <c r="B126" t="s" s="0">
+      <c r="B126" t="s">
         <v>548</v>
       </c>
-      <c r="C126" s="7" t="s">
+      <c r="C126" s="6" t="s">
         <v>549</v>
       </c>
-      <c r="D126" s="6" t="s">
+      <c r="D126" s="5" t="s">
         <v>550</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A127" t="s" s="0">
+      <c r="A127" t="s">
         <v>551</v>
       </c>
-      <c r="B127" t="s" s="0">
+      <c r="B127" t="s">
         <v>552</v>
       </c>
-      <c r="C127" s="7" t="s">
+      <c r="C127" s="6" t="s">
         <v>553</v>
       </c>
-      <c r="D127" s="6" t="s">
+      <c r="D127" s="5" t="s">
         <v>554</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A128" t="s" s="0">
+      <c r="A128" t="s">
         <v>555</v>
       </c>
-      <c r="B128" t="s" s="0">
+      <c r="B128" t="s">
         <v>556</v>
       </c>
-      <c r="C128" s="7" t="s">
+      <c r="C128" s="6" t="s">
         <v>557</v>
       </c>
-      <c r="D128" s="6" t="s">
+      <c r="D128" s="5" t="s">
         <v>558</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A129" t="s" s="0">
+      <c r="A129" t="s">
         <v>559</v>
       </c>
-      <c r="B129" t="s" s="0">
+      <c r="B129" t="s">
         <v>560</v>
       </c>
-      <c r="C129" s="7" t="s">
+      <c r="C129" s="6" t="s">
         <v>561</v>
       </c>
-      <c r="D129" s="6" t="s">
+      <c r="D129" s="5" t="s">
         <v>562</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A130" t="s" s="0">
+      <c r="A130" t="s">
         <v>563</v>
       </c>
-      <c r="B130" t="s" s="0">
+      <c r="B130" t="s">
         <v>564</v>
       </c>
-      <c r="C130" s="7" t="s">
+      <c r="C130" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="D130" s="6" t="s">
+      <c r="D130" s="5" t="s">
         <v>566</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A131" t="s" s="0">
+      <c r="A131" t="s">
         <v>567</v>
       </c>
-      <c r="B131" t="s" s="0">
+      <c r="B131" t="s">
         <v>568</v>
       </c>
-      <c r="C131" s="7" t="s">
+      <c r="C131" s="6" t="s">
         <v>569</v>
       </c>
-      <c r="D131" s="6" t="s">
+      <c r="D131" s="5" t="s">
         <v>570</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A132" t="s" s="0">
+      <c r="A132" t="s">
         <v>571</v>
       </c>
-      <c r="B132" t="s" s="0">
+      <c r="B132" t="s">
         <v>572</v>
       </c>
-      <c r="C132" s="7" t="s">
+      <c r="C132" s="6" t="s">
         <v>573</v>
       </c>
-      <c r="D132" s="6" t="s">
+      <c r="D132" s="5" t="s">
         <v>574</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A133" t="s" s="0">
+      <c r="A133" t="s">
         <v>575</v>
       </c>
-      <c r="B133" t="s" s="0">
+      <c r="B133" t="s">
         <v>576</v>
       </c>
-      <c r="C133" s="7" t="s">
+      <c r="C133" s="6" t="s">
         <v>577</v>
       </c>
-      <c r="D133" s="6" t="s">
+      <c r="D133" s="5" t="s">
         <v>578</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A134" t="s" s="0">
+      <c r="A134" t="s">
         <v>579</v>
       </c>
-      <c r="B134" t="s" s="0">
+      <c r="B134" t="s">
         <v>580</v>
       </c>
-      <c r="C134" s="7" t="s">
+      <c r="C134" s="6" t="s">
         <v>581</v>
       </c>
-      <c r="D134" s="6" t="s">
+      <c r="D134" s="5" t="s">
         <v>582</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A135" t="s" s="0">
+      <c r="A135" t="s">
         <v>583</v>
       </c>
-      <c r="B135" t="s" s="0">
+      <c r="B135" t="s">
         <v>584</v>
       </c>
-      <c r="C135" s="7" t="s">
+      <c r="C135" s="6" t="s">
         <v>585</v>
       </c>
-      <c r="D135" s="6" t="s">
+      <c r="D135" s="5" t="s">
         <v>586</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A136" t="s" s="0">
+      <c r="A136" t="s">
         <v>587</v>
       </c>
-      <c r="B136" t="s" s="0">
+      <c r="B136" t="s">
         <v>588</v>
       </c>
-      <c r="C136" s="7" t="s">
+      <c r="C136" s="6" t="s">
         <v>589</v>
       </c>
-      <c r="D136" s="6" t="s">
+      <c r="D136" s="5" t="s">
         <v>590</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A137" t="s" s="0">
+      <c r="A137" t="s">
         <v>591</v>
       </c>
-      <c r="B137" t="s" s="0">
+      <c r="B137" t="s">
         <v>592</v>
       </c>
-      <c r="C137" s="7" t="s">
+      <c r="C137" s="6" t="s">
         <v>593</v>
       </c>
-      <c r="D137" s="6" t="s">
+      <c r="D137" s="5" t="s">
         <v>594</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A138" t="s" s="0">
+      <c r="A138" t="s">
         <v>595</v>
       </c>
-      <c r="B138" t="s" s="0">
+      <c r="B138" t="s">
         <v>596</v>
       </c>
-      <c r="C138" s="7" t="s">
+      <c r="C138" s="6" t="s">
         <v>597</v>
       </c>
-      <c r="D138" s="6" t="s">
+      <c r="D138" s="5" t="s">
         <v>598</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A139" t="s" s="0">
+      <c r="A139" t="s">
         <v>599</v>
       </c>
-      <c r="B139" t="s" s="0">
+      <c r="B139" t="s">
         <v>600</v>
       </c>
-      <c r="C139" s="7" t="s">
+      <c r="C139" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="D139" s="6" t="s">
+      <c r="D139" s="5" t="s">
         <v>602</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A140" t="s" s="0">
+      <c r="A140" t="s">
         <v>603</v>
       </c>
-      <c r="B140" t="s" s="0">
+      <c r="B140" t="s">
         <v>604</v>
       </c>
-      <c r="C140" s="7" t="s">
+      <c r="C140" s="6" t="s">
         <v>605</v>
       </c>
-      <c r="D140" s="6" t="s">
+      <c r="D140" s="5" t="s">
         <v>606</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A141" t="s" s="0">
+      <c r="A141" t="s">
         <v>607</v>
       </c>
-      <c r="B141" t="s" s="0">
+      <c r="B141" t="s">
         <v>608</v>
       </c>
-      <c r="C141" s="7" t="s">
+      <c r="C141" s="6" t="s">
         <v>609</v>
       </c>
-      <c r="D141" s="6" t="s">
+      <c r="D141" s="5" t="s">
         <v>610</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A142" t="s" s="0">
+      <c r="A142" t="s">
         <v>611</v>
       </c>
-      <c r="B142" t="s" s="0">
+      <c r="B142" t="s">
         <v>612</v>
       </c>
-      <c r="C142" s="7" t="s">
+      <c r="C142" s="6" t="s">
         <v>613</v>
       </c>
-      <c r="D142" s="6" t="s">
+      <c r="D142" s="5" t="s">
         <v>614</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A143" t="s" s="0">
+      <c r="A143" t="s">
         <v>615</v>
       </c>
-      <c r="B143" t="s" s="0">
+      <c r="B143" t="s">
         <v>616</v>
       </c>
-      <c r="C143" s="7" t="s">
+      <c r="C143" s="6" t="s">
         <v>617</v>
       </c>
-      <c r="D143" s="6" t="s">
+      <c r="D143" s="5" t="s">
         <v>618</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A144" t="s" s="0">
+      <c r="A144" t="s">
         <v>619</v>
       </c>
-      <c r="B144" t="s" s="0">
+      <c r="B144" t="s">
         <v>620</v>
       </c>
-      <c r="C144" s="7" t="s">
+      <c r="C144" s="6" t="s">
         <v>621</v>
       </c>
-      <c r="D144" s="6" t="s">
+      <c r="D144" s="5" t="s">
         <v>622</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A145" t="s" s="0">
+      <c r="A145" t="s">
         <v>623</v>
       </c>
-      <c r="B145" t="s" s="0">
+      <c r="B145" t="s">
         <v>624</v>
       </c>
-      <c r="C145" s="7" t="s">
+      <c r="C145" s="6" t="s">
         <v>625</v>
       </c>
-      <c r="D145" s="6" t="s">
+      <c r="D145" s="5" t="s">
         <v>626</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A146" t="s" s="0">
+      <c r="A146" t="s">
         <v>627</v>
       </c>
-      <c r="B146" t="s" s="0">
+      <c r="B146" t="s">
         <v>628</v>
       </c>
-      <c r="C146" s="7" t="s">
+      <c r="C146" s="6" t="s">
         <v>629</v>
       </c>
-      <c r="D146" s="6" t="s">
+      <c r="D146" s="5" t="s">
         <v>630</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A147" t="s" s="0">
+      <c r="A147" t="s">
         <v>631</v>
       </c>
-      <c r="B147" t="s" s="0">
+      <c r="B147" t="s">
         <v>632</v>
       </c>
-      <c r="C147" s="7" t="s">
+      <c r="C147" s="6" t="s">
         <v>633</v>
       </c>
-      <c r="D147" s="6" t="s">
+      <c r="D147" s="5" t="s">
         <v>634</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A148" t="s" s="0">
+      <c r="A148" t="s">
         <v>635</v>
       </c>
-      <c r="B148" t="s" s="0">
+      <c r="B148" t="s">
         <v>636</v>
       </c>
-      <c r="C148" s="7" t="s">
+      <c r="C148" s="6" t="s">
         <v>637</v>
       </c>
-      <c r="D148" s="6" t="s">
+      <c r="D148" s="5" t="s">
         <v>638</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A149" t="s" s="0">
+      <c r="A149" t="s">
         <v>639</v>
       </c>
-      <c r="B149" t="s" s="0">
+      <c r="B149" t="s">
         <v>640</v>
       </c>
-      <c r="C149" s="7" t="s">
+      <c r="C149" s="6" t="s">
         <v>641</v>
       </c>
-      <c r="D149" s="6" t="s">
+      <c r="D149" s="5" t="s">
         <v>642</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A150" t="s" s="0">
+      <c r="A150" t="s">
         <v>643</v>
       </c>
-      <c r="B150" t="s" s="0">
+      <c r="B150" t="s">
         <v>644</v>
       </c>
-      <c r="C150" s="7" t="s">
+      <c r="C150" s="6" t="s">
         <v>645</v>
       </c>
-      <c r="D150" s="6" t="s">
+      <c r="D150" s="5" t="s">
         <v>646</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A151" t="s" s="0">
+      <c r="A151" t="s">
         <v>647</v>
       </c>
-      <c r="B151" t="s" s="0">
+      <c r="B151" t="s">
         <v>648</v>
       </c>
-      <c r="C151" s="7" t="s">
+      <c r="C151" s="6" t="s">
         <v>649</v>
       </c>
-      <c r="D151" s="6" t="s">
+      <c r="D151" s="5" t="s">
         <v>650</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A152" t="s" s="0">
+      <c r="A152" t="s">
         <v>651</v>
       </c>
-      <c r="B152" t="s" s="0">
+      <c r="B152" t="s">
         <v>652</v>
       </c>
-      <c r="C152" s="7" t="s">
+      <c r="C152" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="D152" s="6" t="s">
+      <c r="D152" s="5" t="s">
         <v>654</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B153" t="s" s="0">
+      <c r="B153" t="s">
         <v>655</v>
       </c>
-      <c r="C153" s="7" t="s">
+      <c r="C153" s="6" t="s">
         <v>656</v>
       </c>
-      <c r="D153" s="6" t="s">
+      <c r="D153" s="5" t="s">
         <v>657</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B154" t="s" s="0">
+      <c r="B154" t="s">
         <v>658</v>
       </c>
-      <c r="C154" s="7" t="s">
+      <c r="C154" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="D154" s="6" t="s">
+      <c r="D154" s="5" t="s">
         <v>660</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B155" t="s" s="0">
+      <c r="B155" t="s">
         <v>661</v>
       </c>
-      <c r="C155" s="7" t="s">
+      <c r="C155" s="6" t="s">
         <v>662</v>
       </c>
-      <c r="D155" s="6" t="s">
+      <c r="D155" s="5" t="s">
         <v>663</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B156" t="s" s="0">
+      <c r="B156" t="s">
         <v>664</v>
       </c>
-      <c r="C156" s="7" t="s">
+      <c r="C156" s="6" t="s">
         <v>665</v>
       </c>
-      <c r="D156" s="6" t="s">
+      <c r="D156" s="5" t="s">
         <v>666</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B157" t="s" s="0">
+      <c r="B157" t="s">
         <v>667</v>
       </c>
-      <c r="C157" s="7" t="s">
+      <c r="C157" s="6" t="s">
         <v>668</v>
       </c>
-      <c r="D157" s="6" t="s">
+      <c r="D157" s="5" t="s">
         <v>669</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B158" t="s" s="0">
+      <c r="B158" t="s">
         <v>670</v>
       </c>
-      <c r="C158" s="7" t="s">
+      <c r="C158" s="6" t="s">
         <v>671</v>
       </c>
-      <c r="D158" s="6" t="s">
+      <c r="D158" s="5" t="s">
         <v>672</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C159" s="7" t="s">
+      <c r="C159" s="6" t="s">
         <v>673</v>
       </c>
-      <c r="D159" s="6" t="s">
+      <c r="D159" s="5" t="s">
         <v>674</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C160" s="7" t="s">
+      <c r="C160" s="6" t="s">
         <v>675</v>
       </c>
-      <c r="D160" s="6" t="s">
+      <c r="D160" s="5" t="s">
         <v>676</v>
       </c>
     </row>
     <row r="161" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C161" s="7" t="s">
+      <c r="C161" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="D161" s="6" t="s">
+      <c r="D161" s="5" t="s">
         <v>678</v>
       </c>
     </row>
     <row r="162" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C162" s="7" t="s">
+      <c r="C162" s="6" t="s">
         <v>679</v>
       </c>
-      <c r="D162" s="6" t="s">
+      <c r="D162" s="5" t="s">
         <v>680</v>
       </c>
     </row>
     <row r="163" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C163" s="7" t="s">
+      <c r="C163" s="6" t="s">
         <v>681</v>
       </c>
-      <c r="D163" s="6" t="s">
+      <c r="D163" s="5" t="s">
         <v>682</v>
       </c>
     </row>
     <row r="164" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C164" s="7" t="s">
+      <c r="C164" s="6" t="s">
         <v>683</v>
       </c>
-      <c r="D164" s="6" t="s">
+      <c r="D164" s="5" t="s">
         <v>684</v>
       </c>
     </row>
     <row r="165" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C165" s="7" t="s">
+      <c r="C165" s="6" t="s">
         <v>685</v>
       </c>
-      <c r="D165" s="6" t="s">
+      <c r="D165" s="5" t="s">
         <v>686</v>
       </c>
     </row>
     <row r="166" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C166" s="7" t="s">
+      <c r="C166" s="6" t="s">
         <v>687</v>
       </c>
-      <c r="D166" s="6" t="s">
+      <c r="D166" s="5" t="s">
         <v>688</v>
       </c>
     </row>
     <row r="167" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C167" s="7" t="s">
+      <c r="C167" s="6" t="s">
         <v>689</v>
       </c>
-      <c r="D167" s="6" t="s">
+      <c r="D167" s="5" t="s">
         <v>690</v>
       </c>
     </row>
     <row r="168" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C168" s="7" t="s">
+      <c r="C168" s="6" t="s">
         <v>691</v>
       </c>
-      <c r="D168" s="6" t="s">
+      <c r="D168" s="5" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="169" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C169" s="7" t="s">
+      <c r="C169" s="6" t="s">
         <v>693</v>
       </c>
-      <c r="D169" s="6" t="s">
+      <c r="D169" s="5" t="s">
         <v>694</v>
       </c>
     </row>
     <row r="170" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C170" s="7" t="s">
+      <c r="C170" s="6" t="s">
         <v>695</v>
       </c>
-      <c r="D170" s="6" t="s">
+      <c r="D170" s="5" t="s">
         <v>696</v>
       </c>
     </row>
     <row r="171" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="D171" s="6" t="s">
+      <c r="D171" s="5" t="s">
         <v>697</v>
       </c>
     </row>
     <row r="172" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="D172" s="6" t="s">
+      <c r="D172" s="5" t="s">
         <v>698</v>
       </c>
     </row>
     <row r="173" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="D173" s="6" t="s">
+      <c r="D173" s="5" t="s">
         <v>699</v>
       </c>
     </row>
     <row r="174" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="D174" s="6" t="s">
+      <c r="D174" s="5" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="175" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="D175" s="6" t="s">
+      <c r="D175" s="5" t="s">
         <v>701</v>
       </c>
     </row>
     <row r="176" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="D176" s="6" t="s">
+      <c r="D176" s="5" t="s">
         <v>702</v>
       </c>
     </row>
     <row r="177" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D177" s="6" t="s">
+      <c r="D177" s="5" t="s">
         <v>703</v>
       </c>
     </row>
     <row r="178" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D178" s="6" t="s">
+      <c r="D178" s="5" t="s">
         <v>704</v>
       </c>
     </row>
     <row r="179" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D179" s="6" t="s">
+      <c r="D179" s="5" t="s">
         <v>705</v>
       </c>
     </row>
     <row r="180" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D180" s="6" t="s">
+      <c r="D180" s="5" t="s">
         <v>706</v>
       </c>
     </row>
     <row r="181" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D181" s="6" t="s">
+      <c r="D181" s="5" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="182" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D182" s="6" t="s">
+      <c r="D182" s="5" t="s">
         <v>708</v>
       </c>
     </row>
     <row r="183" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D183" s="6" t="s">
+      <c r="D183" s="5" t="s">
         <v>709</v>
       </c>
     </row>
     <row r="184" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D184" s="6" t="s">
+      <c r="D184" s="5" t="s">
         <v>710</v>
       </c>
     </row>
     <row r="185" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D185" s="6" t="s">
+      <c r="D185" s="5" t="s">
         <v>711</v>
       </c>
     </row>
     <row r="186" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D186" s="6" t="s">
+      <c r="D186" s="5" t="s">
         <v>712</v>
       </c>
     </row>
     <row r="187" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D187" s="6" t="s">
+      <c r="D187" s="5" t="s">
         <v>713</v>
       </c>
     </row>
     <row r="188" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D188" s="6" t="s">
+      <c r="D188" s="5" t="s">
         <v>714</v>
       </c>
     </row>
     <row r="189" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D189" s="6" t="s">
+      <c r="D189" s="5" t="s">
         <v>715</v>
       </c>
     </row>
     <row r="190" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D190" s="6" t="s">
+      <c r="D190" s="5" t="s">
         <v>716</v>
       </c>
     </row>
     <row r="191" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D191" s="6" t="s">
+      <c r="D191" s="5" t="s">
         <v>717</v>
       </c>
     </row>
     <row r="192" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D192" s="6" t="s">
+      <c r="D192" s="5" t="s">
         <v>718</v>
       </c>
     </row>
     <row r="193" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D193" s="6" t="s">
+      <c r="D193" s="5" t="s">
         <v>719</v>
       </c>
     </row>
     <row r="194" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D194" s="6" t="s">
+      <c r="D194" s="5" t="s">
         <v>720</v>
       </c>
     </row>
     <row r="195" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D195" s="6" t="s">
+      <c r="D195" s="5" t="s">
         <v>721</v>
       </c>
     </row>
     <row r="196" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D196" s="6" t="s">
+      <c r="D196" s="5" t="s">
         <v>722</v>
       </c>
     </row>
     <row r="197" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D197" s="6" t="s">
+      <c r="D197" s="5" t="s">
         <v>723</v>
       </c>
     </row>
     <row r="198" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D198" s="6" t="s">
+      <c r="D198" s="5" t="s">
         <v>724</v>
       </c>
     </row>
     <row r="199" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D199" s="6" t="s">
+      <c r="D199" s="5" t="s">
         <v>725</v>
       </c>
     </row>
     <row r="200" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D200" s="6" t="s">
+      <c r="D200" s="5" t="s">
         <v>726</v>
       </c>
     </row>
     <row r="201" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D201" s="6" t="s">
+      <c r="D201" s="5" t="s">
         <v>727</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Eliminated lines of code for add and edit horse details scenarios.
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -1,27 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tools\workspace\testing\animalBiome_Automation\src\test\resources\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13980" windowHeight="3150" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13980" windowHeight="3090" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
     <sheet name="PET_NAME" sheetId="2" r:id="rId2"/>
     <sheet name="ADD_PET" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A28:G35"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="773">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -2252,36 +2248,101 @@
     <t>Nexra</t>
   </si>
   <si>
-    <t>Charlie79</t>
-  </si>
-  <si>
-    <t>Milo56</t>
-  </si>
-  <si>
-    <t>Taffy54</t>
-  </si>
-  <si>
-    <t>Cutie43</t>
-  </si>
-  <si>
-    <t>Cinder43</t>
-  </si>
-  <si>
-    <t>pony35</t>
-  </si>
-  <si>
-    <t>fury28</t>
-  </si>
-  <si>
-    <t>Sheep28</t>
+    <t>JDAGGA</t>
+  </si>
+  <si>
+    <t>AV9GCG</t>
+  </si>
+  <si>
+    <t>NKNGH7</t>
+  </si>
+  <si>
+    <t>J6MGVG</t>
+  </si>
+  <si>
+    <t>4F66HY</t>
+  </si>
+  <si>
+    <t>HHUXJN</t>
+  </si>
+  <si>
+    <t>GUMCDP</t>
+  </si>
+  <si>
+    <t>FVRDEY</t>
+  </si>
+  <si>
+    <t>CM4KEX</t>
+  </si>
+  <si>
+    <t>MVY7E7</t>
+  </si>
+  <si>
+    <t>E4FR3M</t>
+  </si>
+  <si>
+    <t>EMDDGE</t>
+  </si>
+  <si>
+    <t>4PEEDE</t>
+  </si>
+  <si>
+    <t>MT3YXX</t>
+  </si>
+  <si>
+    <t>XHFYNX</t>
+  </si>
+  <si>
+    <t>ENJTEH</t>
+  </si>
+  <si>
+    <t>VJFKAH</t>
+  </si>
+  <si>
+    <t>RVYMTD</t>
+  </si>
+  <si>
+    <t>HTD7FV</t>
+  </si>
+  <si>
+    <t>D7RM3G</t>
+  </si>
+  <si>
+    <t>DPXN44</t>
+  </si>
+  <si>
+    <t>EVAYHN</t>
+  </si>
+  <si>
+    <t>GTGXFA</t>
+  </si>
+  <si>
+    <t>HC7FGA</t>
+  </si>
+  <si>
+    <t>6G4AUX</t>
+  </si>
+  <si>
+    <t>FKCAP9</t>
+  </si>
+  <si>
+    <t>6C9EJE</t>
+  </si>
+  <si>
+    <t>HJ6NJX</t>
+  </si>
+  <si>
+    <t>PA7EFN</t>
+  </si>
+  <si>
+    <t>MJAPC7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2293,6 +2354,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2315,14 +2383,20 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -2330,25 +2404,36 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2"/>
     <cellStyle name="Normal 3" xfId="1"/>
-    <cellStyle name="Normal 2" xfId="2"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -2357,10 +2442,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -2492,7 +2577,6 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2516,11 +2600,10 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -2529,13 +2612,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cmpd="sng" algn="ctr">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2611,7 +2694,6 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2631,34 +2713,35 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J81"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K81"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="17.81641"/>
-    <col min="2" max="2" customWidth="true" style="1" width="15.0"/>
-    <col min="3" max="3" customWidth="true" style="1" width="15.36328"/>
-    <col min="4" max="4" customWidth="true" style="1" width="17.45313"/>
-    <col min="5" max="5" customWidth="true" style="1" width="16.63281"/>
-    <col min="6" max="6" customWidth="true" style="1" width="18.0"/>
-    <col min="7" max="7" customWidth="true" style="1" width="17.26953"/>
-    <col min="8" max="8" customWidth="true" style="1" width="18.17969"/>
-    <col min="9" max="9" customWidth="true" style="1" width="18.36328"/>
-    <col min="10" max="10" customWidth="true" style="1" width="17.45313"/>
-    <col min="11" max="11" customWidth="true" style="1" width="17.36328"/>
-    <col min="12" max="16384" style="1" width="8.726563"/>
+    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.5">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2690,7 +2773,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" ht="15.5">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2707,7 +2790,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" ht="15.5">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -2724,7 +2807,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" ht="15.5">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2741,7 +2824,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" ht="15.5">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>25</v>
       </c>
@@ -2758,7 +2841,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" ht="15.5">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>30</v>
       </c>
@@ -2775,7 +2858,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" ht="15.5">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>35</v>
       </c>
@@ -2792,7 +2875,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" ht="15.5">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>40</v>
       </c>
@@ -2809,167 +2892,266 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" ht="15.5">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="C9" t="s">
+        <v>765</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>749</v>
+      </c>
       <c r="E9" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="10" ht="15.5">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="C10" t="s">
+        <v>766</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>750</v>
+      </c>
       <c r="E10" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="11" ht="15.5">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="C11" t="s">
+        <v>767</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>751</v>
+      </c>
       <c r="E11" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="12" ht="15.5">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>772</v>
+      </c>
+      <c r="C12" t="s">
+        <v>768</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>752</v>
+      </c>
       <c r="E12" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="78" ht="15.5">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="E13" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>754</v>
+      </c>
+      <c r="E14" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E15" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E16" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E17" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E18" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E19" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E20" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E21" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="22" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E22" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="78" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F78" s="3"/>
     </row>
-    <row r="81" ht="15.5">
+    <row r="81" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F81" s="3"/>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="26.90625"/>
-    <col min="2" max="2" customWidth="true" width="29.45313"/>
-    <col min="3" max="3" customWidth="true" width="35.63281"/>
-    <col min="4" max="4" customWidth="true" width="30.90625"/>
-    <col min="5" max="5" customWidth="true" width="32.72656"/>
-    <col min="6" max="6" customWidth="true" width="32.17969"/>
-    <col min="7" max="7" customWidth="true" width="33.63281"/>
-    <col min="8" max="8" customWidth="true" width="31.26953"/>
+    <col min="1" max="1" width="26.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" customWidth="1"/>
+    <col min="4" max="4" width="30.90625" customWidth="1"/>
+    <col min="5" max="5" width="32.7265625" customWidth="1"/>
+    <col min="6" max="6" width="32.1796875" customWidth="1"/>
+    <col min="7" max="7" width="33.6328125" customWidth="1"/>
+    <col min="8" max="8" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>54</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>55</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>57</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>57</v>
       </c>
-      <c r="C2" t="s" s="0">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>57</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
+      <c r="B3" t="s">
         <v>57</v>
       </c>
-      <c r="B3" t="s" s="0">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>57</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="B4" t="s">
         <v>57</v>
       </c>
-      <c r="D3" t="s" s="0">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>57</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>57</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>57</v>
-      </c>
-    </row>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H201"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.08984"/>
-    <col min="2" max="2" customWidth="true" width="17.54297"/>
-    <col min="3" max="3" customWidth="true" width="17.36328"/>
-    <col min="4" max="5" customWidth="true" width="17.26953"/>
-    <col min="6" max="6" customWidth="true" width="17.17969"/>
-    <col min="7" max="7" customWidth="true" width="15.36328"/>
-    <col min="8" max="8" customWidth="true" width="17.17969"/>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="4" max="5" width="17.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.5">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>59</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>60</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>61</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>62</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>63</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" ht="14.5">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>66</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -2979,11 +3161,11 @@
         <v>69</v>
       </c>
     </row>
-    <row r="3" ht="14.5">
-      <c r="A3" t="s" s="0">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>70</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>71</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -2993,11 +3175,11 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" ht="14.5">
-      <c r="A4" t="s" s="0">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>74</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>75</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -3007,11 +3189,11 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" ht="14.5">
-      <c r="A5" t="s" s="0">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>78</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>79</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -3021,11 +3203,11 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" ht="14.5">
-      <c r="A6" t="s" s="0">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>82</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>83</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -3035,11 +3217,11 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" ht="14.5">
-      <c r="A7" t="s" s="0">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>86</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s">
         <v>87</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -3049,11 +3231,11 @@
         <v>89</v>
       </c>
     </row>
-    <row r="8" ht="14.5">
-      <c r="A8" t="s" s="0">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>90</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="B8" t="s">
         <v>91</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -3063,11 +3245,11 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" ht="14.5">
-      <c r="A9" t="s" s="0">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>94</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="B9" t="s">
         <v>95</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -3077,11 +3259,11 @@
         <v>97</v>
       </c>
     </row>
-    <row r="10" ht="14.5">
-      <c r="A10" t="s" s="0">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>98</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="B10" t="s">
         <v>99</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -3091,11 +3273,11 @@
         <v>101</v>
       </c>
     </row>
-    <row r="11" ht="14.5">
-      <c r="A11" t="s" s="0">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>102</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="B11" t="s">
         <v>103</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -3105,11 +3287,11 @@
         <v>105</v>
       </c>
     </row>
-    <row r="12" ht="14.5">
-      <c r="A12" t="s" s="0">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>106</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="B12" t="s">
         <v>107</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -3119,11 +3301,11 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" ht="14.5">
-      <c r="A13" t="s" s="0">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>110</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="B13" t="s">
         <v>111</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -3133,11 +3315,11 @@
         <v>113</v>
       </c>
     </row>
-    <row r="14" ht="14.5">
-      <c r="A14" t="s" s="0">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>114</v>
       </c>
-      <c r="B14" t="s" s="0">
+      <c r="B14" t="s">
         <v>115</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -3147,11 +3329,11 @@
         <v>117</v>
       </c>
     </row>
-    <row r="15" ht="14.5">
-      <c r="A15" t="s" s="0">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>118</v>
       </c>
-      <c r="B15" t="s" s="0">
+      <c r="B15" t="s">
         <v>119</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -3161,11 +3343,11 @@
         <v>121</v>
       </c>
     </row>
-    <row r="16" ht="14.5">
-      <c r="A16" t="s" s="0">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>122</v>
       </c>
-      <c r="B16" t="s" s="0">
+      <c r="B16" t="s">
         <v>123</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -3175,11 +3357,11 @@
         <v>125</v>
       </c>
     </row>
-    <row r="17" ht="14.5">
-      <c r="A17" t="s" s="0">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>126</v>
       </c>
-      <c r="B17" t="s" s="0">
+      <c r="B17" t="s">
         <v>127</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -3189,11 +3371,11 @@
         <v>129</v>
       </c>
     </row>
-    <row r="18" ht="14.5">
-      <c r="A18" t="s" s="0">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>130</v>
       </c>
-      <c r="B18" t="s" s="0">
+      <c r="B18" t="s">
         <v>131</v>
       </c>
       <c r="C18" s="13" t="s">
@@ -3203,53 +3385,53 @@
         <v>133</v>
       </c>
     </row>
-    <row r="19" ht="14.5">
-      <c r="A19" t="s" s="0">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>134</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="B19" t="s">
         <v>135</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="16" t="s">
         <v>136</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="20" ht="14.5">
-      <c r="A20" t="s" s="0">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>138</v>
       </c>
-      <c r="B20" t="s" s="0">
+      <c r="B20" t="s">
         <v>139</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="17" t="s">
         <v>140</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="21" ht="14.5">
-      <c r="A21" t="s" s="0">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>142</v>
       </c>
-      <c r="B21" t="s" s="0">
+      <c r="B21" t="s">
         <v>143</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="18" t="s">
         <v>144</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="22" ht="14.5">
-      <c r="A22" t="s" s="0">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>146</v>
       </c>
-      <c r="B22" t="s" s="0">
+      <c r="B22" t="s">
         <v>147</v>
       </c>
       <c r="C22" s="6" t="s">
@@ -3259,11 +3441,11 @@
         <v>149</v>
       </c>
     </row>
-    <row r="23" ht="14.5">
-      <c r="A23" t="s" s="0">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>150</v>
       </c>
-      <c r="B23" t="s" s="0">
+      <c r="B23" t="s">
         <v>151</v>
       </c>
       <c r="C23" s="6" t="s">
@@ -3273,11 +3455,11 @@
         <v>153</v>
       </c>
     </row>
-    <row r="24" ht="14.5">
-      <c r="A24" t="s" s="0">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>154</v>
       </c>
-      <c r="B24" t="s" s="0">
+      <c r="B24" t="s">
         <v>155</v>
       </c>
       <c r="C24" s="6" t="s">
@@ -3287,11 +3469,11 @@
         <v>157</v>
       </c>
     </row>
-    <row r="25" ht="14.5">
-      <c r="A25" t="s" s="0">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>158</v>
       </c>
-      <c r="B25" t="s" s="0">
+      <c r="B25" t="s">
         <v>159</v>
       </c>
       <c r="C25" s="6" t="s">
@@ -3301,11 +3483,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="26" ht="14.5">
-      <c r="A26" t="s" s="0">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>162</v>
       </c>
-      <c r="B26" t="s" s="0">
+      <c r="B26" t="s">
         <v>163</v>
       </c>
       <c r="C26" s="6" t="s">
@@ -3315,11 +3497,11 @@
         <v>165</v>
       </c>
     </row>
-    <row r="27" ht="14.5">
-      <c r="A27" t="s" s="0">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>166</v>
       </c>
-      <c r="B27" t="s" s="0">
+      <c r="B27" t="s">
         <v>167</v>
       </c>
       <c r="C27" s="6" t="s">
@@ -3329,11 +3511,11 @@
         <v>169</v>
       </c>
     </row>
-    <row r="28" ht="14.5">
-      <c r="A28" t="s" s="0">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>170</v>
       </c>
-      <c r="B28" t="s" s="0">
+      <c r="B28" t="s">
         <v>171</v>
       </c>
       <c r="C28" s="6" t="s">
@@ -3343,11 +3525,11 @@
         <v>173</v>
       </c>
     </row>
-    <row r="29" ht="14.5">
-      <c r="A29" t="s" s="0">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>174</v>
       </c>
-      <c r="B29" t="s" s="0">
+      <c r="B29" t="s">
         <v>175</v>
       </c>
       <c r="C29" s="6" t="s">
@@ -3357,11 +3539,11 @@
         <v>177</v>
       </c>
     </row>
-    <row r="30" ht="14.5">
-      <c r="A30" t="s" s="0">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>178</v>
       </c>
-      <c r="B30" t="s" s="0">
+      <c r="B30" t="s">
         <v>179</v>
       </c>
       <c r="C30" s="6" t="s">
@@ -3371,11 +3553,11 @@
         <v>181</v>
       </c>
     </row>
-    <row r="31" ht="14.5">
-      <c r="A31" t="s" s="0">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>182</v>
       </c>
-      <c r="B31" t="s" s="0">
+      <c r="B31" t="s">
         <v>183</v>
       </c>
       <c r="C31" s="6" t="s">
@@ -3385,11 +3567,11 @@
         <v>185</v>
       </c>
     </row>
-    <row r="32" ht="14.5">
-      <c r="A32" t="s" s="0">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>186</v>
       </c>
-      <c r="B32" t="s" s="0">
+      <c r="B32" t="s">
         <v>187</v>
       </c>
       <c r="C32" s="6" t="s">
@@ -3399,11 +3581,11 @@
         <v>189</v>
       </c>
     </row>
-    <row r="33" ht="14.5">
-      <c r="A33" t="s" s="0">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>190</v>
       </c>
-      <c r="B33" t="s" s="0">
+      <c r="B33" t="s">
         <v>191</v>
       </c>
       <c r="C33" s="6" t="s">
@@ -3413,11 +3595,11 @@
         <v>193</v>
       </c>
     </row>
-    <row r="34" ht="14.5">
-      <c r="A34" t="s" s="0">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>194</v>
       </c>
-      <c r="B34" t="s" s="0">
+      <c r="B34" t="s">
         <v>195</v>
       </c>
       <c r="C34" s="6" t="s">
@@ -3427,11 +3609,11 @@
         <v>197</v>
       </c>
     </row>
-    <row r="35" ht="14.5">
-      <c r="A35" t="s" s="0">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>198</v>
       </c>
-      <c r="B35" t="s" s="0">
+      <c r="B35" t="s">
         <v>199</v>
       </c>
       <c r="C35" s="6" t="s">
@@ -3441,11 +3623,11 @@
         <v>201</v>
       </c>
     </row>
-    <row r="36" ht="14.5">
-      <c r="A36" t="s" s="0">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>202</v>
       </c>
-      <c r="B36" t="s" s="0">
+      <c r="B36" t="s">
         <v>203</v>
       </c>
       <c r="C36" s="6" t="s">
@@ -3455,11 +3637,11 @@
         <v>205</v>
       </c>
     </row>
-    <row r="37" ht="14.5">
-      <c r="A37" t="s" s="0">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>206</v>
       </c>
-      <c r="B37" t="s" s="0">
+      <c r="B37" t="s">
         <v>207</v>
       </c>
       <c r="C37" s="6" t="s">
@@ -3469,11 +3651,11 @@
         <v>209</v>
       </c>
     </row>
-    <row r="38" ht="14.5">
-      <c r="A38" t="s" s="0">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>210</v>
       </c>
-      <c r="B38" t="s" s="0">
+      <c r="B38" t="s">
         <v>211</v>
       </c>
       <c r="C38" s="6" t="s">
@@ -3483,11 +3665,11 @@
         <v>213</v>
       </c>
     </row>
-    <row r="39" ht="14.5">
-      <c r="A39" t="s" s="0">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>214</v>
       </c>
-      <c r="B39" t="s" s="0">
+      <c r="B39" t="s">
         <v>215</v>
       </c>
       <c r="C39" s="6" t="s">
@@ -3497,11 +3679,11 @@
         <v>217</v>
       </c>
     </row>
-    <row r="40" ht="14.5">
-      <c r="A40" t="s" s="0">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>218</v>
       </c>
-      <c r="B40" t="s" s="0">
+      <c r="B40" t="s">
         <v>219</v>
       </c>
       <c r="C40" s="6" t="s">
@@ -3511,11 +3693,11 @@
         <v>221</v>
       </c>
     </row>
-    <row r="41" ht="14.5">
-      <c r="A41" t="s" s="0">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>222</v>
       </c>
-      <c r="B41" t="s" s="0">
+      <c r="B41" t="s">
         <v>223</v>
       </c>
       <c r="C41" s="6" t="s">
@@ -3525,11 +3707,11 @@
         <v>225</v>
       </c>
     </row>
-    <row r="42" ht="14.5">
-      <c r="A42" t="s" s="0">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>226</v>
       </c>
-      <c r="B42" t="s" s="0">
+      <c r="B42" t="s">
         <v>227</v>
       </c>
       <c r="C42" s="6" t="s">
@@ -3539,11 +3721,11 @@
         <v>229</v>
       </c>
     </row>
-    <row r="43" ht="14.5">
-      <c r="A43" t="s" s="0">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>230</v>
       </c>
-      <c r="B43" t="s" s="0">
+      <c r="B43" t="s">
         <v>231</v>
       </c>
       <c r="C43" s="6" t="s">
@@ -3553,11 +3735,11 @@
         <v>233</v>
       </c>
     </row>
-    <row r="44" ht="14.5">
-      <c r="A44" t="s" s="0">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>234</v>
       </c>
-      <c r="B44" t="s" s="0">
+      <c r="B44" t="s">
         <v>235</v>
       </c>
       <c r="C44" s="6" t="s">
@@ -3567,11 +3749,11 @@
         <v>237</v>
       </c>
     </row>
-    <row r="45" ht="14.5">
-      <c r="A45" t="s" s="0">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>238</v>
       </c>
-      <c r="B45" t="s" s="0">
+      <c r="B45" t="s">
         <v>239</v>
       </c>
       <c r="C45" s="6" t="s">
@@ -3581,11 +3763,11 @@
         <v>241</v>
       </c>
     </row>
-    <row r="46" ht="14.5">
-      <c r="A46" t="s" s="0">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>242</v>
       </c>
-      <c r="B46" t="s" s="0">
+      <c r="B46" t="s">
         <v>243</v>
       </c>
       <c r="C46" s="6" t="s">
@@ -3595,11 +3777,11 @@
         <v>245</v>
       </c>
     </row>
-    <row r="47" ht="14.5">
-      <c r="A47" t="s" s="0">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>246</v>
       </c>
-      <c r="B47" t="s" s="0">
+      <c r="B47" t="s">
         <v>247</v>
       </c>
       <c r="C47" s="6" t="s">
@@ -3609,11 +3791,11 @@
         <v>249</v>
       </c>
     </row>
-    <row r="48" ht="14.5">
-      <c r="A48" t="s" s="0">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>250</v>
       </c>
-      <c r="B48" t="s" s="0">
+      <c r="B48" t="s">
         <v>251</v>
       </c>
       <c r="C48" s="6" t="s">
@@ -3623,11 +3805,11 @@
         <v>253</v>
       </c>
     </row>
-    <row r="49" ht="14.5">
-      <c r="A49" t="s" s="0">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>254</v>
       </c>
-      <c r="B49" t="s" s="0">
+      <c r="B49" t="s">
         <v>255</v>
       </c>
       <c r="C49" s="6" t="s">
@@ -3637,11 +3819,11 @@
         <v>257</v>
       </c>
     </row>
-    <row r="50" ht="14.5">
-      <c r="A50" t="s" s="0">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>258</v>
       </c>
-      <c r="B50" t="s" s="0">
+      <c r="B50" t="s">
         <v>259</v>
       </c>
       <c r="C50" s="6" t="s">
@@ -3651,11 +3833,11 @@
         <v>261</v>
       </c>
     </row>
-    <row r="51" ht="14.5">
-      <c r="A51" t="s" s="0">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>262</v>
       </c>
-      <c r="B51" t="s" s="0">
+      <c r="B51" t="s">
         <v>263</v>
       </c>
       <c r="C51" s="6" t="s">
@@ -3665,11 +3847,11 @@
         <v>265</v>
       </c>
     </row>
-    <row r="52" ht="14.5">
-      <c r="A52" t="s" s="0">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>266</v>
       </c>
-      <c r="B52" t="s" s="0">
+      <c r="B52" t="s">
         <v>267</v>
       </c>
       <c r="C52" s="6" t="s">
@@ -3679,11 +3861,11 @@
         <v>269</v>
       </c>
     </row>
-    <row r="53" ht="14.5">
-      <c r="A53" t="s" s="0">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>270</v>
       </c>
-      <c r="B53" t="s" s="0">
+      <c r="B53" t="s">
         <v>271</v>
       </c>
       <c r="C53" s="6" t="s">
@@ -3693,11 +3875,11 @@
         <v>273</v>
       </c>
     </row>
-    <row r="54" ht="14.5">
-      <c r="A54" t="s" s="0">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
         <v>274</v>
       </c>
-      <c r="B54" t="s" s="0">
+      <c r="B54" t="s">
         <v>275</v>
       </c>
       <c r="C54" s="6" t="s">
@@ -3707,11 +3889,11 @@
         <v>277</v>
       </c>
     </row>
-    <row r="55" ht="14.5">
-      <c r="A55" t="s" s="0">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>278</v>
       </c>
-      <c r="B55" t="s" s="0">
+      <c r="B55" t="s">
         <v>279</v>
       </c>
       <c r="C55" s="6" t="s">
@@ -3721,11 +3903,11 @@
         <v>281</v>
       </c>
     </row>
-    <row r="56" ht="14.5">
-      <c r="A56" t="s" s="0">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>282</v>
       </c>
-      <c r="B56" t="s" s="0">
+      <c r="B56" t="s">
         <v>283</v>
       </c>
       <c r="C56" s="6" t="s">
@@ -3735,11 +3917,11 @@
         <v>285</v>
       </c>
     </row>
-    <row r="57" ht="14.5">
-      <c r="A57" t="s" s="0">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>286</v>
       </c>
-      <c r="B57" t="s" s="0">
+      <c r="B57" t="s">
         <v>287</v>
       </c>
       <c r="C57" s="6" t="s">
@@ -3749,11 +3931,11 @@
         <v>289</v>
       </c>
     </row>
-    <row r="58" ht="14.5">
-      <c r="A58" t="s" s="0">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>290</v>
       </c>
-      <c r="B58" t="s" s="0">
+      <c r="B58" t="s">
         <v>291</v>
       </c>
       <c r="C58" s="6" t="s">
@@ -3763,11 +3945,11 @@
         <v>293</v>
       </c>
     </row>
-    <row r="59" ht="14.5">
-      <c r="A59" t="s" s="0">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>294</v>
       </c>
-      <c r="B59" t="s" s="0">
+      <c r="B59" t="s">
         <v>295</v>
       </c>
       <c r="C59" s="6" t="s">
@@ -3777,11 +3959,11 @@
         <v>297</v>
       </c>
     </row>
-    <row r="60" ht="14.5">
-      <c r="A60" t="s" s="0">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>298</v>
       </c>
-      <c r="B60" t="s" s="0">
+      <c r="B60" t="s">
         <v>299</v>
       </c>
       <c r="C60" s="6" t="s">
@@ -3791,11 +3973,11 @@
         <v>301</v>
       </c>
     </row>
-    <row r="61" ht="14.5">
-      <c r="A61" t="s" s="0">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>302</v>
       </c>
-      <c r="B61" t="s" s="0">
+      <c r="B61" t="s">
         <v>303</v>
       </c>
       <c r="C61" s="6" t="s">
@@ -3805,11 +3987,11 @@
         <v>305</v>
       </c>
     </row>
-    <row r="62" ht="14.5">
-      <c r="A62" t="s" s="0">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>306</v>
       </c>
-      <c r="B62" t="s" s="0">
+      <c r="B62" t="s">
         <v>307</v>
       </c>
       <c r="C62" s="6" t="s">
@@ -3819,11 +4001,11 @@
         <v>309</v>
       </c>
     </row>
-    <row r="63" ht="14.5">
-      <c r="A63" t="s" s="0">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>310</v>
       </c>
-      <c r="B63" t="s" s="0">
+      <c r="B63" t="s">
         <v>311</v>
       </c>
       <c r="C63" s="6" t="s">
@@ -3833,11 +4015,11 @@
         <v>313</v>
       </c>
     </row>
-    <row r="64" ht="14.5">
-      <c r="A64" t="s" s="0">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>314</v>
       </c>
-      <c r="B64" t="s" s="0">
+      <c r="B64" t="s">
         <v>315</v>
       </c>
       <c r="C64" s="6" t="s">
@@ -3847,11 +4029,11 @@
         <v>317</v>
       </c>
     </row>
-    <row r="65" ht="14.5">
-      <c r="A65" t="s" s="0">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>318</v>
       </c>
-      <c r="B65" t="s" s="0">
+      <c r="B65" t="s">
         <v>319</v>
       </c>
       <c r="C65" s="6" t="s">
@@ -3861,11 +4043,11 @@
         <v>321</v>
       </c>
     </row>
-    <row r="66" ht="14.5">
-      <c r="A66" t="s" s="0">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>322</v>
       </c>
-      <c r="B66" t="s" s="0">
+      <c r="B66" t="s">
         <v>323</v>
       </c>
       <c r="C66" s="6" t="s">
@@ -3875,11 +4057,11 @@
         <v>325</v>
       </c>
     </row>
-    <row r="67" ht="14.5">
-      <c r="A67" t="s" s="0">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>326</v>
       </c>
-      <c r="B67" t="s" s="0">
+      <c r="B67" t="s">
         <v>327</v>
       </c>
       <c r="C67" s="6" t="s">
@@ -3889,11 +4071,11 @@
         <v>329</v>
       </c>
     </row>
-    <row r="68" ht="14.5">
-      <c r="A68" t="s" s="0">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>330</v>
       </c>
-      <c r="B68" t="s" s="0">
+      <c r="B68" t="s">
         <v>331</v>
       </c>
       <c r="C68" s="6" t="s">
@@ -3903,11 +4085,11 @@
         <v>333</v>
       </c>
     </row>
-    <row r="69" ht="14.5">
-      <c r="A69" t="s" s="0">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>334</v>
       </c>
-      <c r="B69" t="s" s="0">
+      <c r="B69" t="s">
         <v>335</v>
       </c>
       <c r="C69" s="6" t="s">
@@ -3917,11 +4099,11 @@
         <v>337</v>
       </c>
     </row>
-    <row r="70" ht="14.5">
-      <c r="A70" t="s" s="0">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>338</v>
       </c>
-      <c r="B70" t="s" s="0">
+      <c r="B70" t="s">
         <v>339</v>
       </c>
       <c r="C70" s="6" t="s">
@@ -3931,11 +4113,11 @@
         <v>341</v>
       </c>
     </row>
-    <row r="71" ht="14.5">
-      <c r="A71" t="s" s="0">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>342</v>
       </c>
-      <c r="B71" t="s" s="0">
+      <c r="B71" t="s">
         <v>343</v>
       </c>
       <c r="C71" s="6" t="s">
@@ -3945,11 +4127,11 @@
         <v>345</v>
       </c>
     </row>
-    <row r="72" ht="14.5">
-      <c r="A72" t="s" s="0">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>346</v>
       </c>
-      <c r="B72" t="s" s="0">
+      <c r="B72" t="s">
         <v>347</v>
       </c>
       <c r="C72" s="6" t="s">
@@ -3959,11 +4141,11 @@
         <v>349</v>
       </c>
     </row>
-    <row r="73" ht="14.5">
-      <c r="A73" t="s" s="0">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>350</v>
       </c>
-      <c r="B73" t="s" s="0">
+      <c r="B73" t="s">
         <v>351</v>
       </c>
       <c r="C73" s="6" t="s">
@@ -3973,11 +4155,11 @@
         <v>353</v>
       </c>
     </row>
-    <row r="74" ht="14.5">
-      <c r="A74" t="s" s="0">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>354</v>
       </c>
-      <c r="B74" t="s" s="0">
+      <c r="B74" t="s">
         <v>355</v>
       </c>
       <c r="C74" s="6" t="s">
@@ -3987,11 +4169,11 @@
         <v>357</v>
       </c>
     </row>
-    <row r="75" ht="14.5">
-      <c r="A75" t="s" s="0">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>358</v>
       </c>
-      <c r="B75" t="s" s="0">
+      <c r="B75" t="s">
         <v>359</v>
       </c>
       <c r="C75" s="6" t="s">
@@ -4001,11 +4183,11 @@
         <v>361</v>
       </c>
     </row>
-    <row r="76" ht="14.5">
-      <c r="A76" t="s" s="0">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>362</v>
       </c>
-      <c r="B76" t="s" s="0">
+      <c r="B76" t="s">
         <v>363</v>
       </c>
       <c r="C76" s="6" t="s">
@@ -4015,11 +4197,11 @@
         <v>365</v>
       </c>
     </row>
-    <row r="77" ht="14.5">
-      <c r="A77" t="s" s="0">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>366</v>
       </c>
-      <c r="B77" t="s" s="0">
+      <c r="B77" t="s">
         <v>367</v>
       </c>
       <c r="C77" s="6" t="s">
@@ -4029,11 +4211,11 @@
         <v>369</v>
       </c>
     </row>
-    <row r="78" ht="14.5">
-      <c r="A78" t="s" s="0">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>370</v>
       </c>
-      <c r="B78" t="s" s="0">
+      <c r="B78" t="s">
         <v>371</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -4043,11 +4225,11 @@
         <v>373</v>
       </c>
     </row>
-    <row r="79" ht="14.5">
-      <c r="A79" t="s" s="0">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>374</v>
       </c>
-      <c r="B79" t="s" s="0">
+      <c r="B79" t="s">
         <v>375</v>
       </c>
       <c r="C79" s="6" t="s">
@@ -4057,11 +4239,11 @@
         <v>377</v>
       </c>
     </row>
-    <row r="80" ht="14.5">
-      <c r="A80" t="s" s="0">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>378</v>
       </c>
-      <c r="B80" t="s" s="0">
+      <c r="B80" t="s">
         <v>379</v>
       </c>
       <c r="C80" s="6" t="s">
@@ -4071,11 +4253,11 @@
         <v>381</v>
       </c>
     </row>
-    <row r="81" ht="14.5">
-      <c r="A81" t="s" s="0">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>382</v>
       </c>
-      <c r="B81" t="s" s="0">
+      <c r="B81" t="s">
         <v>383</v>
       </c>
       <c r="C81" s="6" t="s">
@@ -4085,11 +4267,11 @@
         <v>385</v>
       </c>
     </row>
-    <row r="82" ht="14.5">
-      <c r="A82" t="s" s="0">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>386</v>
       </c>
-      <c r="B82" t="s" s="0">
+      <c r="B82" t="s">
         <v>387</v>
       </c>
       <c r="C82" s="6" t="s">
@@ -4099,11 +4281,11 @@
         <v>389</v>
       </c>
     </row>
-    <row r="83" ht="14.5">
-      <c r="A83" t="s" s="0">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
         <v>390</v>
       </c>
-      <c r="B83" t="s" s="0">
+      <c r="B83" t="s">
         <v>391</v>
       </c>
       <c r="C83" s="6" t="s">
@@ -4113,11 +4295,11 @@
         <v>393</v>
       </c>
     </row>
-    <row r="84" ht="14.5">
-      <c r="A84" t="s" s="0">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
         <v>394</v>
       </c>
-      <c r="B84" t="s" s="0">
+      <c r="B84" t="s">
         <v>395</v>
       </c>
       <c r="C84" s="6" t="s">
@@ -4127,11 +4309,11 @@
         <v>397</v>
       </c>
     </row>
-    <row r="85" ht="14.5">
-      <c r="A85" t="s" s="0">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
         <v>398</v>
       </c>
-      <c r="B85" t="s" s="0">
+      <c r="B85" t="s">
         <v>399</v>
       </c>
       <c r="C85" s="6" t="s">
@@ -4141,11 +4323,11 @@
         <v>401</v>
       </c>
     </row>
-    <row r="86" ht="14.5">
-      <c r="A86" t="s" s="0">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
         <v>402</v>
       </c>
-      <c r="B86" t="s" s="0">
+      <c r="B86" t="s">
         <v>403</v>
       </c>
       <c r="C86" s="6" t="s">
@@ -4155,11 +4337,11 @@
         <v>405</v>
       </c>
     </row>
-    <row r="87" ht="14.5">
-      <c r="A87" t="s" s="0">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
         <v>406</v>
       </c>
-      <c r="B87" t="s" s="0">
+      <c r="B87" t="s">
         <v>407</v>
       </c>
       <c r="C87" s="6" t="s">
@@ -4169,11 +4351,11 @@
         <v>409</v>
       </c>
     </row>
-    <row r="88" ht="14.5">
-      <c r="A88" t="s" s="0">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>410</v>
       </c>
-      <c r="B88" t="s" s="0">
+      <c r="B88" t="s">
         <v>411</v>
       </c>
       <c r="C88" s="6" t="s">
@@ -4183,11 +4365,11 @@
         <v>413</v>
       </c>
     </row>
-    <row r="89" ht="14.5">
-      <c r="A89" t="s" s="0">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>414</v>
       </c>
-      <c r="B89" t="s" s="0">
+      <c r="B89" t="s">
         <v>415</v>
       </c>
       <c r="C89" s="6" t="s">
@@ -4197,11 +4379,11 @@
         <v>417</v>
       </c>
     </row>
-    <row r="90" ht="14.5">
-      <c r="A90" t="s" s="0">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>418</v>
       </c>
-      <c r="B90" t="s" s="0">
+      <c r="B90" t="s">
         <v>419</v>
       </c>
       <c r="C90" s="6" t="s">
@@ -4211,11 +4393,11 @@
         <v>421</v>
       </c>
     </row>
-    <row r="91" ht="14.5">
-      <c r="A91" t="s" s="0">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
         <v>422</v>
       </c>
-      <c r="B91" t="s" s="0">
+      <c r="B91" t="s">
         <v>423</v>
       </c>
       <c r="C91" s="6" t="s">
@@ -4225,11 +4407,11 @@
         <v>425</v>
       </c>
     </row>
-    <row r="92" ht="14.5">
-      <c r="A92" t="s" s="0">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>426</v>
       </c>
-      <c r="B92" t="s" s="0">
+      <c r="B92" t="s">
         <v>427</v>
       </c>
       <c r="C92" s="6" t="s">
@@ -4239,11 +4421,11 @@
         <v>429</v>
       </c>
     </row>
-    <row r="93" ht="14.5">
-      <c r="A93" t="s" s="0">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
         <v>430</v>
       </c>
-      <c r="B93" t="s" s="0">
+      <c r="B93" t="s">
         <v>431</v>
       </c>
       <c r="C93" s="6" t="s">
@@ -4253,11 +4435,11 @@
         <v>433</v>
       </c>
     </row>
-    <row r="94" ht="14.5">
-      <c r="A94" t="s" s="0">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>434</v>
       </c>
-      <c r="B94" t="s" s="0">
+      <c r="B94" t="s">
         <v>435</v>
       </c>
       <c r="C94" s="6" t="s">
@@ -4267,11 +4449,11 @@
         <v>437</v>
       </c>
     </row>
-    <row r="95" ht="14.5">
-      <c r="A95" t="s" s="0">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>438</v>
       </c>
-      <c r="B95" t="s" s="0">
+      <c r="B95" t="s">
         <v>439</v>
       </c>
       <c r="C95" s="6" t="s">
@@ -4281,11 +4463,11 @@
         <v>441</v>
       </c>
     </row>
-    <row r="96" ht="14.5">
-      <c r="A96" t="s" s="0">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
         <v>442</v>
       </c>
-      <c r="B96" t="s" s="0">
+      <c r="B96" t="s">
         <v>443</v>
       </c>
       <c r="C96" s="6" t="s">
@@ -4295,11 +4477,11 @@
         <v>445</v>
       </c>
     </row>
-    <row r="97" ht="14.5">
-      <c r="A97" t="s" s="0">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
         <v>446</v>
       </c>
-      <c r="B97" t="s" s="0">
+      <c r="B97" t="s">
         <v>447</v>
       </c>
       <c r="C97" s="6" t="s">
@@ -4309,11 +4491,11 @@
         <v>449</v>
       </c>
     </row>
-    <row r="98" ht="14.5">
-      <c r="A98" t="s" s="0">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
         <v>450</v>
       </c>
-      <c r="B98" t="s" s="0">
+      <c r="B98" t="s">
         <v>451</v>
       </c>
       <c r="C98" s="6" t="s">
@@ -4323,11 +4505,11 @@
         <v>453</v>
       </c>
     </row>
-    <row r="99" ht="14.5">
-      <c r="A99" t="s" s="0">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
         <v>454</v>
       </c>
-      <c r="B99" t="s" s="0">
+      <c r="B99" t="s">
         <v>455</v>
       </c>
       <c r="C99" s="6" t="s">
@@ -4337,11 +4519,11 @@
         <v>457</v>
       </c>
     </row>
-    <row r="100" ht="14.5">
-      <c r="A100" t="s" s="0">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
         <v>458</v>
       </c>
-      <c r="B100" t="s" s="0">
+      <c r="B100" t="s">
         <v>459</v>
       </c>
       <c r="C100" s="6" t="s">
@@ -4351,11 +4533,11 @@
         <v>461</v>
       </c>
     </row>
-    <row r="101" ht="14.5">
-      <c r="A101" t="s" s="0">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>462</v>
       </c>
-      <c r="B101" t="s" s="0">
+      <c r="B101" t="s">
         <v>463</v>
       </c>
       <c r="C101" s="6" t="s">
@@ -4365,11 +4547,11 @@
         <v>465</v>
       </c>
     </row>
-    <row r="102" ht="14.5">
-      <c r="A102" t="s" s="0">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
         <v>466</v>
       </c>
-      <c r="B102" t="s" s="0">
+      <c r="B102" t="s">
         <v>467</v>
       </c>
       <c r="C102" s="6" t="s">
@@ -4379,11 +4561,11 @@
         <v>469</v>
       </c>
     </row>
-    <row r="103" ht="14.5">
-      <c r="A103" t="s" s="0">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
         <v>470</v>
       </c>
-      <c r="B103" t="s" s="0">
+      <c r="B103" t="s">
         <v>471</v>
       </c>
       <c r="C103" s="6" t="s">
@@ -4393,11 +4575,11 @@
         <v>473</v>
       </c>
     </row>
-    <row r="104" ht="14.5">
-      <c r="A104" t="s" s="0">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
         <v>474</v>
       </c>
-      <c r="B104" t="s" s="0">
+      <c r="B104" t="s">
         <v>475</v>
       </c>
       <c r="C104" s="6" t="s">
@@ -4407,11 +4589,11 @@
         <v>477</v>
       </c>
     </row>
-    <row r="105" ht="14.5">
-      <c r="A105" t="s" s="0">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
         <v>478</v>
       </c>
-      <c r="B105" t="s" s="0">
+      <c r="B105" t="s">
         <v>479</v>
       </c>
       <c r="C105" s="6" t="s">
@@ -4421,11 +4603,11 @@
         <v>481</v>
       </c>
     </row>
-    <row r="106" ht="14.5">
-      <c r="A106" t="s" s="0">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
         <v>482</v>
       </c>
-      <c r="B106" t="s" s="0">
+      <c r="B106" t="s">
         <v>483</v>
       </c>
       <c r="C106" s="6" t="s">
@@ -4435,11 +4617,11 @@
         <v>485</v>
       </c>
     </row>
-    <row r="107" ht="14.5">
-      <c r="A107" t="s" s="0">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
         <v>486</v>
       </c>
-      <c r="B107" t="s" s="0">
+      <c r="B107" t="s">
         <v>487</v>
       </c>
       <c r="C107" s="6" t="s">
@@ -4449,11 +4631,11 @@
         <v>489</v>
       </c>
     </row>
-    <row r="108" ht="14.5">
-      <c r="A108" t="s" s="0">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
         <v>490</v>
       </c>
-      <c r="B108" t="s" s="0">
+      <c r="B108" t="s">
         <v>491</v>
       </c>
       <c r="C108" s="6" t="s">
@@ -4463,11 +4645,11 @@
         <v>493</v>
       </c>
     </row>
-    <row r="109" ht="14.5">
-      <c r="A109" t="s" s="0">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
         <v>494</v>
       </c>
-      <c r="B109" t="s" s="0">
+      <c r="B109" t="s">
         <v>495</v>
       </c>
       <c r="C109" s="6" t="s">
@@ -4477,11 +4659,11 @@
         <v>497</v>
       </c>
     </row>
-    <row r="110" ht="14.5">
-      <c r="A110" t="s" s="0">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
         <v>498</v>
       </c>
-      <c r="B110" t="s" s="0">
+      <c r="B110" t="s">
         <v>499</v>
       </c>
       <c r="C110" s="6" t="s">
@@ -4491,11 +4673,11 @@
         <v>501</v>
       </c>
     </row>
-    <row r="111" ht="14.5">
-      <c r="A111" t="s" s="0">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
         <v>502</v>
       </c>
-      <c r="B111" t="s" s="0">
+      <c r="B111" t="s">
         <v>503</v>
       </c>
       <c r="C111" s="6" t="s">
@@ -4505,11 +4687,11 @@
         <v>505</v>
       </c>
     </row>
-    <row r="112" ht="14.5">
-      <c r="A112" t="s" s="0">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
         <v>506</v>
       </c>
-      <c r="B112" t="s" s="0">
+      <c r="B112" t="s">
         <v>507</v>
       </c>
       <c r="C112" s="6" t="s">
@@ -4519,11 +4701,11 @@
         <v>509</v>
       </c>
     </row>
-    <row r="113" ht="14.5">
-      <c r="A113" t="s" s="0">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
         <v>510</v>
       </c>
-      <c r="B113" t="s" s="0">
+      <c r="B113" t="s">
         <v>511</v>
       </c>
       <c r="C113" s="6" t="s">
@@ -4533,11 +4715,11 @@
         <v>513</v>
       </c>
     </row>
-    <row r="114" ht="14.5">
-      <c r="A114" t="s" s="0">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
         <v>514</v>
       </c>
-      <c r="B114" t="s" s="0">
+      <c r="B114" t="s">
         <v>515</v>
       </c>
       <c r="C114" s="6" t="s">
@@ -4547,11 +4729,11 @@
         <v>517</v>
       </c>
     </row>
-    <row r="115" ht="14.5">
-      <c r="A115" t="s" s="0">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
         <v>518</v>
       </c>
-      <c r="B115" t="s" s="0">
+      <c r="B115" t="s">
         <v>519</v>
       </c>
       <c r="C115" s="6" t="s">
@@ -4561,11 +4743,11 @@
         <v>521</v>
       </c>
     </row>
-    <row r="116" ht="14.5">
-      <c r="A116" t="s" s="0">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
         <v>522</v>
       </c>
-      <c r="B116" t="s" s="0">
+      <c r="B116" t="s">
         <v>523</v>
       </c>
       <c r="C116" s="6" t="s">
@@ -4575,11 +4757,11 @@
         <v>525</v>
       </c>
     </row>
-    <row r="117" ht="14.5">
-      <c r="A117" t="s" s="0">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
         <v>526</v>
       </c>
-      <c r="B117" t="s" s="0">
+      <c r="B117" t="s">
         <v>527</v>
       </c>
       <c r="C117" s="6" t="s">
@@ -4589,11 +4771,11 @@
         <v>529</v>
       </c>
     </row>
-    <row r="118" ht="14.5">
-      <c r="A118" t="s" s="0">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
         <v>530</v>
       </c>
-      <c r="B118" t="s" s="0">
+      <c r="B118" t="s">
         <v>531</v>
       </c>
       <c r="C118" s="6" t="s">
@@ -4603,11 +4785,11 @@
         <v>533</v>
       </c>
     </row>
-    <row r="119" ht="14.5">
-      <c r="A119" t="s" s="0">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
         <v>534</v>
       </c>
-      <c r="B119" t="s" s="0">
+      <c r="B119" t="s">
         <v>535</v>
       </c>
       <c r="C119" s="6" t="s">
@@ -4617,11 +4799,11 @@
         <v>537</v>
       </c>
     </row>
-    <row r="120" ht="14.5">
-      <c r="A120" t="s" s="0">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
         <v>538</v>
       </c>
-      <c r="B120" t="s" s="0">
+      <c r="B120" t="s">
         <v>539</v>
       </c>
       <c r="C120" s="6" t="s">
@@ -4631,11 +4813,11 @@
         <v>541</v>
       </c>
     </row>
-    <row r="121" ht="14.5">
-      <c r="A121" t="s" s="0">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
         <v>542</v>
       </c>
-      <c r="B121" t="s" s="0">
+      <c r="B121" t="s">
         <v>543</v>
       </c>
       <c r="C121" s="6" t="s">
@@ -4645,11 +4827,11 @@
         <v>545</v>
       </c>
     </row>
-    <row r="122" ht="14.5">
-      <c r="A122" t="s" s="0">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
         <v>546</v>
       </c>
-      <c r="B122" t="s" s="0">
+      <c r="B122" t="s">
         <v>547</v>
       </c>
       <c r="C122" s="6" t="s">
@@ -4659,11 +4841,11 @@
         <v>549</v>
       </c>
     </row>
-    <row r="123" ht="14.5">
-      <c r="A123" t="s" s="0">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
         <v>550</v>
       </c>
-      <c r="B123" t="s" s="0">
+      <c r="B123" t="s">
         <v>551</v>
       </c>
       <c r="C123" s="6" t="s">
@@ -4673,11 +4855,11 @@
         <v>553</v>
       </c>
     </row>
-    <row r="124" ht="14.5">
-      <c r="A124" t="s" s="0">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
         <v>554</v>
       </c>
-      <c r="B124" t="s" s="0">
+      <c r="B124" t="s">
         <v>555</v>
       </c>
       <c r="C124" s="6" t="s">
@@ -4687,11 +4869,11 @@
         <v>557</v>
       </c>
     </row>
-    <row r="125" ht="14.5">
-      <c r="A125" t="s" s="0">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
         <v>558</v>
       </c>
-      <c r="B125" t="s" s="0">
+      <c r="B125" t="s">
         <v>559</v>
       </c>
       <c r="C125" s="6" t="s">
@@ -4701,11 +4883,11 @@
         <v>561</v>
       </c>
     </row>
-    <row r="126" ht="14.5">
-      <c r="A126" t="s" s="0">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
         <v>562</v>
       </c>
-      <c r="B126" t="s" s="0">
+      <c r="B126" t="s">
         <v>563</v>
       </c>
       <c r="C126" s="6" t="s">
@@ -4715,11 +4897,11 @@
         <v>565</v>
       </c>
     </row>
-    <row r="127" ht="14.5">
-      <c r="A127" t="s" s="0">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
         <v>566</v>
       </c>
-      <c r="B127" t="s" s="0">
+      <c r="B127" t="s">
         <v>567</v>
       </c>
       <c r="C127" s="6" t="s">
@@ -4729,11 +4911,11 @@
         <v>569</v>
       </c>
     </row>
-    <row r="128" ht="14.5">
-      <c r="A128" t="s" s="0">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
         <v>570</v>
       </c>
-      <c r="B128" t="s" s="0">
+      <c r="B128" t="s">
         <v>571</v>
       </c>
       <c r="C128" s="6" t="s">
@@ -4743,11 +4925,11 @@
         <v>573</v>
       </c>
     </row>
-    <row r="129" ht="14.5">
-      <c r="A129" t="s" s="0">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
         <v>574</v>
       </c>
-      <c r="B129" t="s" s="0">
+      <c r="B129" t="s">
         <v>575</v>
       </c>
       <c r="C129" s="6" t="s">
@@ -4757,11 +4939,11 @@
         <v>577</v>
       </c>
     </row>
-    <row r="130" ht="14.5">
-      <c r="A130" t="s" s="0">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
         <v>578</v>
       </c>
-      <c r="B130" t="s" s="0">
+      <c r="B130" t="s">
         <v>579</v>
       </c>
       <c r="C130" s="6" t="s">
@@ -4771,11 +4953,11 @@
         <v>581</v>
       </c>
     </row>
-    <row r="131" ht="14.5">
-      <c r="A131" t="s" s="0">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
         <v>582</v>
       </c>
-      <c r="B131" t="s" s="0">
+      <c r="B131" t="s">
         <v>583</v>
       </c>
       <c r="C131" s="6" t="s">
@@ -4785,11 +4967,11 @@
         <v>585</v>
       </c>
     </row>
-    <row r="132" ht="14.5">
-      <c r="A132" t="s" s="0">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
         <v>586</v>
       </c>
-      <c r="B132" t="s" s="0">
+      <c r="B132" t="s">
         <v>587</v>
       </c>
       <c r="C132" s="6" t="s">
@@ -4799,11 +4981,11 @@
         <v>589</v>
       </c>
     </row>
-    <row r="133" ht="14.5">
-      <c r="A133" t="s" s="0">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
         <v>590</v>
       </c>
-      <c r="B133" t="s" s="0">
+      <c r="B133" t="s">
         <v>591</v>
       </c>
       <c r="C133" s="6" t="s">
@@ -4813,11 +4995,11 @@
         <v>593</v>
       </c>
     </row>
-    <row r="134" ht="14.5">
-      <c r="A134" t="s" s="0">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
         <v>594</v>
       </c>
-      <c r="B134" t="s" s="0">
+      <c r="B134" t="s">
         <v>595</v>
       </c>
       <c r="C134" s="6" t="s">
@@ -4827,11 +5009,11 @@
         <v>597</v>
       </c>
     </row>
-    <row r="135" ht="14.5">
-      <c r="A135" t="s" s="0">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
         <v>598</v>
       </c>
-      <c r="B135" t="s" s="0">
+      <c r="B135" t="s">
         <v>599</v>
       </c>
       <c r="C135" s="6" t="s">
@@ -4841,11 +5023,11 @@
         <v>601</v>
       </c>
     </row>
-    <row r="136" ht="14.5">
-      <c r="A136" t="s" s="0">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
         <v>602</v>
       </c>
-      <c r="B136" t="s" s="0">
+      <c r="B136" t="s">
         <v>603</v>
       </c>
       <c r="C136" s="6" t="s">
@@ -4855,11 +5037,11 @@
         <v>605</v>
       </c>
     </row>
-    <row r="137" ht="14.5">
-      <c r="A137" t="s" s="0">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
         <v>606</v>
       </c>
-      <c r="B137" t="s" s="0">
+      <c r="B137" t="s">
         <v>607</v>
       </c>
       <c r="C137" s="6" t="s">
@@ -4869,11 +5051,11 @@
         <v>609</v>
       </c>
     </row>
-    <row r="138" ht="14.5">
-      <c r="A138" t="s" s="0">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
         <v>610</v>
       </c>
-      <c r="B138" t="s" s="0">
+      <c r="B138" t="s">
         <v>611</v>
       </c>
       <c r="C138" s="6" t="s">
@@ -4883,11 +5065,11 @@
         <v>613</v>
       </c>
     </row>
-    <row r="139" ht="14.5">
-      <c r="A139" t="s" s="0">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
         <v>614</v>
       </c>
-      <c r="B139" t="s" s="0">
+      <c r="B139" t="s">
         <v>615</v>
       </c>
       <c r="C139" s="6" t="s">
@@ -4897,11 +5079,11 @@
         <v>617</v>
       </c>
     </row>
-    <row r="140" ht="14.5">
-      <c r="A140" t="s" s="0">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
         <v>618</v>
       </c>
-      <c r="B140" t="s" s="0">
+      <c r="B140" t="s">
         <v>619</v>
       </c>
       <c r="C140" s="6" t="s">
@@ -4911,11 +5093,11 @@
         <v>621</v>
       </c>
     </row>
-    <row r="141" ht="14.5">
-      <c r="A141" t="s" s="0">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
         <v>622</v>
       </c>
-      <c r="B141" t="s" s="0">
+      <c r="B141" t="s">
         <v>623</v>
       </c>
       <c r="C141" s="6" t="s">
@@ -4925,11 +5107,11 @@
         <v>625</v>
       </c>
     </row>
-    <row r="142" ht="14.5">
-      <c r="A142" t="s" s="0">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
         <v>626</v>
       </c>
-      <c r="B142" t="s" s="0">
+      <c r="B142" t="s">
         <v>627</v>
       </c>
       <c r="C142" s="6" t="s">
@@ -4939,11 +5121,11 @@
         <v>629</v>
       </c>
     </row>
-    <row r="143" ht="14.5">
-      <c r="A143" t="s" s="0">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
         <v>630</v>
       </c>
-      <c r="B143" t="s" s="0">
+      <c r="B143" t="s">
         <v>631</v>
       </c>
       <c r="C143" s="6" t="s">
@@ -4953,11 +5135,11 @@
         <v>633</v>
       </c>
     </row>
-    <row r="144" ht="14.5">
-      <c r="A144" t="s" s="0">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
         <v>634</v>
       </c>
-      <c r="B144" t="s" s="0">
+      <c r="B144" t="s">
         <v>635</v>
       </c>
       <c r="C144" s="6" t="s">
@@ -4967,11 +5149,11 @@
         <v>637</v>
       </c>
     </row>
-    <row r="145" ht="14.5">
-      <c r="A145" t="s" s="0">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
         <v>638</v>
       </c>
-      <c r="B145" t="s" s="0">
+      <c r="B145" t="s">
         <v>639</v>
       </c>
       <c r="C145" s="6" t="s">
@@ -4981,11 +5163,11 @@
         <v>641</v>
       </c>
     </row>
-    <row r="146" ht="14.5">
-      <c r="A146" t="s" s="0">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
         <v>642</v>
       </c>
-      <c r="B146" t="s" s="0">
+      <c r="B146" t="s">
         <v>643</v>
       </c>
       <c r="C146" s="6" t="s">
@@ -4995,11 +5177,11 @@
         <v>645</v>
       </c>
     </row>
-    <row r="147" ht="14.5">
-      <c r="A147" t="s" s="0">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
         <v>646</v>
       </c>
-      <c r="B147" t="s" s="0">
+      <c r="B147" t="s">
         <v>647</v>
       </c>
       <c r="C147" s="6" t="s">
@@ -5009,11 +5191,11 @@
         <v>649</v>
       </c>
     </row>
-    <row r="148" ht="14.5">
-      <c r="A148" t="s" s="0">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
         <v>650</v>
       </c>
-      <c r="B148" t="s" s="0">
+      <c r="B148" t="s">
         <v>651</v>
       </c>
       <c r="C148" s="6" t="s">
@@ -5023,11 +5205,11 @@
         <v>653</v>
       </c>
     </row>
-    <row r="149" ht="14.5">
-      <c r="A149" t="s" s="0">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
         <v>654</v>
       </c>
-      <c r="B149" t="s" s="0">
+      <c r="B149" t="s">
         <v>655</v>
       </c>
       <c r="C149" s="6" t="s">
@@ -5037,11 +5219,11 @@
         <v>657</v>
       </c>
     </row>
-    <row r="150" ht="14.5">
-      <c r="A150" t="s" s="0">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
         <v>658</v>
       </c>
-      <c r="B150" t="s" s="0">
+      <c r="B150" t="s">
         <v>659</v>
       </c>
       <c r="C150" s="6" t="s">
@@ -5051,11 +5233,11 @@
         <v>661</v>
       </c>
     </row>
-    <row r="151" ht="14.5">
-      <c r="A151" t="s" s="0">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
         <v>662</v>
       </c>
-      <c r="B151" t="s" s="0">
+      <c r="B151" t="s">
         <v>663</v>
       </c>
       <c r="C151" s="6" t="s">
@@ -5065,11 +5247,11 @@
         <v>665</v>
       </c>
     </row>
-    <row r="152" ht="14.5">
-      <c r="A152" t="s" s="0">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
         <v>666</v>
       </c>
-      <c r="B152" t="s" s="0">
+      <c r="B152" t="s">
         <v>667</v>
       </c>
       <c r="C152" s="6" t="s">
@@ -5079,8 +5261,8 @@
         <v>669</v>
       </c>
     </row>
-    <row r="153" ht="14.5">
-      <c r="B153" t="s" s="0">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B153" t="s">
         <v>670</v>
       </c>
       <c r="C153" s="6" t="s">
@@ -5090,8 +5272,8 @@
         <v>672</v>
       </c>
     </row>
-    <row r="154" ht="14.5">
-      <c r="B154" t="s" s="0">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B154" t="s">
         <v>673</v>
       </c>
       <c r="C154" s="6" t="s">
@@ -5101,8 +5283,8 @@
         <v>675</v>
       </c>
     </row>
-    <row r="155" ht="14.5">
-      <c r="B155" t="s" s="0">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B155" t="s">
         <v>676</v>
       </c>
       <c r="C155" s="6" t="s">
@@ -5112,8 +5294,8 @@
         <v>678</v>
       </c>
     </row>
-    <row r="156" ht="14.5">
-      <c r="B156" t="s" s="0">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B156" t="s">
         <v>679</v>
       </c>
       <c r="C156" s="6" t="s">
@@ -5123,8 +5305,8 @@
         <v>681</v>
       </c>
     </row>
-    <row r="157" ht="14.5">
-      <c r="B157" t="s" s="0">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B157" t="s">
         <v>682</v>
       </c>
       <c r="C157" s="6" t="s">
@@ -5134,8 +5316,8 @@
         <v>684</v>
       </c>
     </row>
-    <row r="158" ht="14.5">
-      <c r="B158" t="s" s="0">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B158" t="s">
         <v>685</v>
       </c>
       <c r="C158" s="6" t="s">
@@ -5145,7 +5327,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="159" ht="14.5">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C159" s="6" t="s">
         <v>688</v>
       </c>
@@ -5153,7 +5335,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="160" ht="14.5">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C160" s="6" t="s">
         <v>690</v>
       </c>
@@ -5161,7 +5343,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="161" ht="14.5">
+    <row r="161" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C161" s="6" t="s">
         <v>692</v>
       </c>
@@ -5169,7 +5351,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="162" ht="14.5">
+    <row r="162" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C162" s="6" t="s">
         <v>694</v>
       </c>
@@ -5177,7 +5359,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="163" ht="14.5">
+    <row r="163" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C163" s="6" t="s">
         <v>696</v>
       </c>
@@ -5185,7 +5367,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="164" ht="14.5">
+    <row r="164" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C164" s="6" t="s">
         <v>698</v>
       </c>
@@ -5193,7 +5375,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="165" ht="14.5">
+    <row r="165" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C165" s="6" t="s">
         <v>700</v>
       </c>
@@ -5201,7 +5383,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="166" ht="14.5">
+    <row r="166" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C166" s="6" t="s">
         <v>702</v>
       </c>
@@ -5209,7 +5391,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="167" ht="14.5">
+    <row r="167" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C167" s="6" t="s">
         <v>704</v>
       </c>
@@ -5217,7 +5399,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="168" ht="14.5">
+    <row r="168" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C168" s="6" t="s">
         <v>706</v>
       </c>
@@ -5225,7 +5407,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="169" ht="14.5">
+    <row r="169" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C169" s="6" t="s">
         <v>708</v>
       </c>
@@ -5233,7 +5415,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="170" ht="14.5">
+    <row r="170" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C170" s="6" t="s">
         <v>710</v>
       </c>
@@ -5241,162 +5423,163 @@
         <v>711</v>
       </c>
     </row>
-    <row r="171" ht="14.5">
+    <row r="171" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D171" s="5" t="s">
         <v>712</v>
       </c>
     </row>
-    <row r="172" ht="14.5">
+    <row r="172" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D172" s="5" t="s">
         <v>713</v>
       </c>
     </row>
-    <row r="173" ht="14.5">
+    <row r="173" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D173" s="5" t="s">
         <v>714</v>
       </c>
     </row>
-    <row r="174" ht="14.5">
+    <row r="174" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D174" s="5" t="s">
         <v>715</v>
       </c>
     </row>
-    <row r="175" ht="14.5">
+    <row r="175" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D175" s="5" t="s">
         <v>716</v>
       </c>
     </row>
-    <row r="176" ht="14.5">
+    <row r="176" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D176" s="5" t="s">
         <v>717</v>
       </c>
     </row>
-    <row r="177" ht="14.5">
+    <row r="177" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D177" s="5" t="s">
         <v>718</v>
       </c>
     </row>
-    <row r="178" ht="14.5">
+    <row r="178" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D178" s="5" t="s">
         <v>719</v>
       </c>
     </row>
-    <row r="179" ht="14.5">
+    <row r="179" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D179" s="5" t="s">
         <v>720</v>
       </c>
     </row>
-    <row r="180" ht="14.5">
+    <row r="180" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D180" s="5" t="s">
         <v>721</v>
       </c>
     </row>
-    <row r="181" ht="14.5">
+    <row r="181" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D181" s="5" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="182" ht="14.5">
+    <row r="182" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D182" s="5" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="183" ht="14.5">
+    <row r="183" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D183" s="5" t="s">
         <v>724</v>
       </c>
     </row>
-    <row r="184" ht="14.5">
+    <row r="184" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D184" s="5" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="185" ht="14.5">
+    <row r="185" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D185" s="5" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="186" ht="14.5">
+    <row r="186" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D186" s="5" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="187" ht="14.5">
+    <row r="187" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D187" s="5" t="s">
         <v>728</v>
       </c>
     </row>
-    <row r="188" ht="14.5">
+    <row r="188" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D188" s="5" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="189" ht="14.5">
+    <row r="189" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D189" s="5" t="s">
         <v>730</v>
       </c>
     </row>
-    <row r="190" ht="14.5">
+    <row r="190" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D190" s="5" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="191" ht="14.5">
+    <row r="191" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D191" s="5" t="s">
         <v>732</v>
       </c>
     </row>
-    <row r="192" ht="14.5">
+    <row r="192" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D192" s="5" t="s">
         <v>733</v>
       </c>
     </row>
-    <row r="193" ht="14.5">
+    <row r="193" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D193" s="5" t="s">
         <v>734</v>
       </c>
     </row>
-    <row r="194" ht="14.5">
+    <row r="194" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D194" s="5" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="195" ht="14.5">
+    <row r="195" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D195" s="5" t="s">
         <v>736</v>
       </c>
     </row>
-    <row r="196" ht="14.5">
+    <row r="196" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D196" s="5" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="197" ht="14.5">
+    <row r="197" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D197" s="5" t="s">
         <v>738</v>
       </c>
     </row>
-    <row r="198" ht="14.5">
+    <row r="198" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D198" s="5" t="s">
         <v>739</v>
       </c>
     </row>
-    <row r="199" ht="14.5">
+    <row r="199" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D199" s="5" t="s">
         <v>740</v>
       </c>
     </row>
-    <row r="200" ht="14.5">
+    <row r="200" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D200" s="5" t="s">
         <v>741</v>
       </c>
     </row>
-    <row r="201" ht="14.5">
+    <row r="201" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D201" s="5" t="s">
         <v>742</v>
       </c>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated testng.xml and samples.xlsx files
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -1,27 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tools\workspace\testing\animalBiome_Automation\src\test\resources\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13980" windowHeight="3090" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13980" windowHeight="3090"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
     <sheet name="PET_NAME" sheetId="2" r:id="rId2"/>
     <sheet name="ADD_PET" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:G8"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="791">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -2342,18 +2338,65 @@
     <t>Nexra</t>
   </si>
   <si>
-    <t>Rabbit36</t>
-  </si>
-  <si>
-    <t>Sheep32</t>
+    <t>VHKTDY</t>
+  </si>
+  <si>
+    <t>NXMGXU</t>
+  </si>
+  <si>
+    <t>FHPENF</t>
+  </si>
+  <si>
+    <t>KMVFMV</t>
+  </si>
+  <si>
+    <t>FMMDPH</t>
+  </si>
+  <si>
+    <t>VTPC7K</t>
+  </si>
+  <si>
+    <t>RXY4RX</t>
+  </si>
+  <si>
+    <t>U9ANVP</t>
+  </si>
+  <si>
+    <t>NMVMC7</t>
+  </si>
+  <si>
+    <t>YTJTEP</t>
+  </si>
+  <si>
+    <t>ADKXJK</t>
+  </si>
+  <si>
+    <t>7KMMDF</t>
+  </si>
+  <si>
+    <t>7PEXET</t>
+  </si>
+  <si>
+    <t>CAYMTM</t>
+  </si>
+  <si>
+    <t>4YJTMR</t>
+  </si>
+  <si>
+    <t>RKRYJR</t>
+  </si>
+  <si>
+    <t>NJ4YMD</t>
+  </si>
+  <si>
+    <t>NR7KMT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2365,6 +2408,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2387,12 +2437,18 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2402,18 +2458,26 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2"/>
     <cellStyle name="Normal 3" xfId="1"/>
-    <cellStyle name="Normal 2" xfId="2"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -2422,10 +2486,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -2557,7 +2621,6 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2581,11 +2644,10 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -2594,13 +2656,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cmpd="sng" algn="ctr">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2676,7 +2738,6 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2696,34 +2757,35 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J81"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K81"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="17.81641"/>
-    <col min="2" max="2" customWidth="true" style="1" width="15.0"/>
-    <col min="3" max="3" customWidth="true" style="1" width="15.36328"/>
-    <col min="4" max="4" customWidth="true" style="1" width="17.45313"/>
-    <col min="5" max="5" customWidth="true" style="1" width="16.63281"/>
-    <col min="6" max="6" customWidth="true" style="1" width="18.0"/>
-    <col min="7" max="7" customWidth="true" style="1" width="17.26953"/>
-    <col min="8" max="8" customWidth="true" style="1" width="18.17969"/>
-    <col min="9" max="9" customWidth="true" style="1" width="18.36328"/>
-    <col min="10" max="10" customWidth="true" style="1" width="17.45313"/>
-    <col min="11" max="11" customWidth="true" style="1" width="17.36328"/>
-    <col min="12" max="16384" style="1" width="8.726563"/>
+    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2755,7 +2817,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2772,7 +2834,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -2789,7 +2851,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2806,7 +2868,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>25</v>
       </c>
@@ -2823,7 +2885,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
@@ -2840,7 +2902,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
@@ -2857,7 +2919,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>40</v>
       </c>
@@ -2874,7 +2936,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>45</v>
       </c>
@@ -2891,7 +2953,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>50</v>
       </c>
@@ -2908,7 +2970,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>55</v>
       </c>
@@ -2925,7 +2987,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>60</v>
       </c>
@@ -2942,7 +3004,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>65</v>
       </c>
@@ -2953,7 +3015,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>68</v>
       </c>
@@ -2964,184 +3026,260 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>778</v>
+      </c>
+      <c r="D15" t="s">
+        <v>773</v>
+      </c>
       <c r="E15" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>779</v>
+      </c>
+      <c r="D16" t="s">
+        <v>774</v>
+      </c>
       <c r="E16" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>780</v>
+      </c>
+      <c r="D17" t="s">
+        <v>775</v>
+      </c>
       <c r="E17" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D18" t="s">
+        <v>776</v>
+      </c>
       <c r="E18" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D19" t="s">
+        <v>777</v>
+      </c>
       <c r="E19" s="8" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E20" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E21" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E22" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="78">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E23" s="1" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E24" s="1" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E25" s="1" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E26" s="1" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E27" s="1" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E28" s="1" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E29" s="1" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E30" s="1" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E31" s="1" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E32" s="1" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="78" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F78" s="3"/>
     </row>
-    <row r="81">
+    <row r="81" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F81" s="3"/>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="26.90625"/>
-    <col min="2" max="2" customWidth="true" width="29.45313"/>
-    <col min="3" max="3" customWidth="true" width="35.63281"/>
-    <col min="4" max="4" customWidth="true" width="30.90625"/>
-    <col min="5" max="5" customWidth="true" width="32.72656"/>
-    <col min="6" max="6" customWidth="true" width="32.17969"/>
-    <col min="7" max="7" customWidth="true" width="33.63281"/>
-    <col min="8" max="8" customWidth="true" width="31.26953"/>
+    <col min="1" max="1" width="26.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" customWidth="1"/>
+    <col min="4" max="4" width="30.90625" customWidth="1"/>
+    <col min="5" max="5" width="32.7265625" customWidth="1"/>
+    <col min="6" max="6" width="32.1796875" customWidth="1"/>
+    <col min="7" max="7" width="33.6328125" customWidth="1"/>
+    <col min="8" max="8" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>79</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>80</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>81</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>82</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>83</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>84</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>85</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>87</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>87</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>87</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>87</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>87</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>87</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>87</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>87</v>
       </c>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H201"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.08984"/>
-    <col min="2" max="2" customWidth="true" width="17.54297"/>
-    <col min="3" max="3" customWidth="true" width="17.36328"/>
-    <col min="4" max="5" customWidth="true" width="17.26953"/>
-    <col min="6" max="6" customWidth="true" width="17.17969"/>
-    <col min="7" max="7" customWidth="true" width="15.36328"/>
-    <col min="8" max="8" customWidth="true" width="17.17969"/>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="4" max="5" width="17.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>93</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>94</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>96</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>97</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -3151,11 +3289,11 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>100</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>101</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -3165,11 +3303,11 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>104</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>105</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -3179,11 +3317,11 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>108</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>109</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -3193,11 +3331,11 @@
         <v>111</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>112</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>113</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -3207,11 +3345,11 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>116</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s">
         <v>117</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -3221,11 +3359,11 @@
         <v>119</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>120</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="B8" t="s">
         <v>121</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -3235,11 +3373,11 @@
         <v>123</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>124</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="B9" t="s">
         <v>125</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -3249,11 +3387,11 @@
         <v>127</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>128</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="B10" t="s">
         <v>129</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -3263,11 +3401,11 @@
         <v>131</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>132</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="B11" t="s">
         <v>133</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -3277,11 +3415,11 @@
         <v>135</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>136</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="B12" t="s">
         <v>137</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -3291,11 +3429,11 @@
         <v>139</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="s" s="0">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>140</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="B13" t="s">
         <v>141</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -3305,11 +3443,11 @@
         <v>143</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="s" s="0">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>144</v>
       </c>
-      <c r="B14" t="s" s="0">
+      <c r="B14" t="s">
         <v>145</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -3319,11 +3457,11 @@
         <v>147</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="s" s="0">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>148</v>
       </c>
-      <c r="B15" t="s" s="0">
+      <c r="B15" t="s">
         <v>149</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -3333,11 +3471,11 @@
         <v>151</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>152</v>
       </c>
-      <c r="B16" t="s" s="0">
+      <c r="B16" t="s">
         <v>153</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -3347,11 +3485,11 @@
         <v>155</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="s" s="0">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>156</v>
       </c>
-      <c r="B17" t="s" s="0">
+      <c r="B17" t="s">
         <v>157</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -3361,11 +3499,11 @@
         <v>159</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>160</v>
       </c>
-      <c r="B18" t="s" s="0">
+      <c r="B18" t="s">
         <v>161</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -3375,11 +3513,11 @@
         <v>163</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>164</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="B19" t="s">
         <v>165</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -3389,11 +3527,11 @@
         <v>167</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="s" s="0">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>168</v>
       </c>
-      <c r="B20" t="s" s="0">
+      <c r="B20" t="s">
         <v>169</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -3403,11 +3541,11 @@
         <v>171</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="s" s="0">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>172</v>
       </c>
-      <c r="B21" t="s" s="0">
+      <c r="B21" t="s">
         <v>173</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -3417,11 +3555,11 @@
         <v>175</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="s" s="0">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>176</v>
       </c>
-      <c r="B22" t="s" s="0">
+      <c r="B22" t="s">
         <v>177</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -3431,11 +3569,11 @@
         <v>179</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="s" s="0">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>180</v>
       </c>
-      <c r="B23" t="s" s="0">
+      <c r="B23" t="s">
         <v>181</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -3445,11 +3583,11 @@
         <v>183</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="s" s="0">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>184</v>
       </c>
-      <c r="B24" t="s" s="0">
+      <c r="B24" t="s">
         <v>185</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -3459,11 +3597,11 @@
         <v>187</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="s" s="0">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>188</v>
       </c>
-      <c r="B25" t="s" s="0">
+      <c r="B25" t="s">
         <v>189</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -3473,11 +3611,11 @@
         <v>191</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="s" s="0">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>192</v>
       </c>
-      <c r="B26" t="s" s="0">
+      <c r="B26" t="s">
         <v>193</v>
       </c>
       <c r="C26" s="6" t="s">
@@ -3487,11 +3625,11 @@
         <v>195</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="s" s="0">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>196</v>
       </c>
-      <c r="B27" t="s" s="0">
+      <c r="B27" t="s">
         <v>197</v>
       </c>
       <c r="C27" s="6" t="s">
@@ -3501,11 +3639,11 @@
         <v>199</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="s" s="0">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>200</v>
       </c>
-      <c r="B28" t="s" s="0">
+      <c r="B28" t="s">
         <v>201</v>
       </c>
       <c r="C28" s="6" t="s">
@@ -3515,11 +3653,11 @@
         <v>203</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="s" s="0">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>204</v>
       </c>
-      <c r="B29" t="s" s="0">
+      <c r="B29" t="s">
         <v>205</v>
       </c>
       <c r="C29" s="6" t="s">
@@ -3529,11 +3667,11 @@
         <v>207</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="s" s="0">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>208</v>
       </c>
-      <c r="B30" t="s" s="0">
+      <c r="B30" t="s">
         <v>209</v>
       </c>
       <c r="C30" s="6" t="s">
@@ -3543,11 +3681,11 @@
         <v>211</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="s" s="0">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>212</v>
       </c>
-      <c r="B31" t="s" s="0">
+      <c r="B31" t="s">
         <v>213</v>
       </c>
       <c r="C31" s="6" t="s">
@@ -3557,11 +3695,11 @@
         <v>215</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="s" s="0">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>216</v>
       </c>
-      <c r="B32" t="s" s="0">
+      <c r="B32" t="s">
         <v>217</v>
       </c>
       <c r="C32" s="6" t="s">
@@ -3571,11 +3709,11 @@
         <v>219</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="s" s="0">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>220</v>
       </c>
-      <c r="B33" t="s" s="0">
+      <c r="B33" t="s">
         <v>221</v>
       </c>
       <c r="C33" s="6" t="s">
@@ -3585,11 +3723,11 @@
         <v>223</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="s" s="0">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>224</v>
       </c>
-      <c r="B34" t="s" s="0">
+      <c r="B34" t="s">
         <v>225</v>
       </c>
       <c r="C34" s="6" t="s">
@@ -3599,11 +3737,11 @@
         <v>227</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="s" s="0">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>228</v>
       </c>
-      <c r="B35" t="s" s="0">
+      <c r="B35" t="s">
         <v>229</v>
       </c>
       <c r="C35" s="6" t="s">
@@ -3613,11 +3751,11 @@
         <v>231</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="s" s="0">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>232</v>
       </c>
-      <c r="B36" t="s" s="0">
+      <c r="B36" t="s">
         <v>233</v>
       </c>
       <c r="C36" s="6" t="s">
@@ -3627,11 +3765,11 @@
         <v>235</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="s" s="0">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>236</v>
       </c>
-      <c r="B37" t="s" s="0">
+      <c r="B37" t="s">
         <v>237</v>
       </c>
       <c r="C37" s="6" t="s">
@@ -3641,11 +3779,11 @@
         <v>239</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="s" s="0">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>240</v>
       </c>
-      <c r="B38" t="s" s="0">
+      <c r="B38" t="s">
         <v>241</v>
       </c>
       <c r="C38" s="6" t="s">
@@ -3655,11 +3793,11 @@
         <v>243</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="s" s="0">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>244</v>
       </c>
-      <c r="B39" t="s" s="0">
+      <c r="B39" t="s">
         <v>245</v>
       </c>
       <c r="C39" s="6" t="s">
@@ -3669,11 +3807,11 @@
         <v>247</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="s" s="0">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>248</v>
       </c>
-      <c r="B40" t="s" s="0">
+      <c r="B40" t="s">
         <v>249</v>
       </c>
       <c r="C40" s="6" t="s">
@@ -3683,11 +3821,11 @@
         <v>251</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="s" s="0">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>252</v>
       </c>
-      <c r="B41" t="s" s="0">
+      <c r="B41" t="s">
         <v>253</v>
       </c>
       <c r="C41" s="6" t="s">
@@ -3697,11 +3835,11 @@
         <v>255</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="s" s="0">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>256</v>
       </c>
-      <c r="B42" t="s" s="0">
+      <c r="B42" t="s">
         <v>257</v>
       </c>
       <c r="C42" s="6" t="s">
@@ -3711,11 +3849,11 @@
         <v>259</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="s" s="0">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>260</v>
       </c>
-      <c r="B43" t="s" s="0">
+      <c r="B43" t="s">
         <v>261</v>
       </c>
       <c r="C43" s="6" t="s">
@@ -3725,11 +3863,11 @@
         <v>263</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="s" s="0">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>264</v>
       </c>
-      <c r="B44" t="s" s="0">
+      <c r="B44" t="s">
         <v>265</v>
       </c>
       <c r="C44" s="6" t="s">
@@ -3739,11 +3877,11 @@
         <v>267</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="s" s="0">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>268</v>
       </c>
-      <c r="B45" t="s" s="0">
+      <c r="B45" t="s">
         <v>269</v>
       </c>
       <c r="C45" s="6" t="s">
@@ -3753,11 +3891,11 @@
         <v>271</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="s" s="0">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>272</v>
       </c>
-      <c r="B46" t="s" s="0">
+      <c r="B46" t="s">
         <v>273</v>
       </c>
       <c r="C46" s="6" t="s">
@@ -3767,11 +3905,11 @@
         <v>275</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="s" s="0">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>276</v>
       </c>
-      <c r="B47" t="s" s="0">
+      <c r="B47" t="s">
         <v>277</v>
       </c>
       <c r="C47" s="6" t="s">
@@ -3781,11 +3919,11 @@
         <v>279</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="s" s="0">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>280</v>
       </c>
-      <c r="B48" t="s" s="0">
+      <c r="B48" t="s">
         <v>281</v>
       </c>
       <c r="C48" s="6" t="s">
@@ -3795,11 +3933,11 @@
         <v>283</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="s" s="0">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>284</v>
       </c>
-      <c r="B49" t="s" s="0">
+      <c r="B49" t="s">
         <v>285</v>
       </c>
       <c r="C49" s="6" t="s">
@@ -3809,11 +3947,11 @@
         <v>287</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="s" s="0">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>288</v>
       </c>
-      <c r="B50" t="s" s="0">
+      <c r="B50" t="s">
         <v>289</v>
       </c>
       <c r="C50" s="6" t="s">
@@ -3823,11 +3961,11 @@
         <v>291</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="s" s="0">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>292</v>
       </c>
-      <c r="B51" t="s" s="0">
+      <c r="B51" t="s">
         <v>293</v>
       </c>
       <c r="C51" s="6" t="s">
@@ -3837,11 +3975,11 @@
         <v>295</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="s" s="0">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>296</v>
       </c>
-      <c r="B52" t="s" s="0">
+      <c r="B52" t="s">
         <v>297</v>
       </c>
       <c r="C52" s="6" t="s">
@@ -3851,11 +3989,11 @@
         <v>299</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="s" s="0">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>300</v>
       </c>
-      <c r="B53" t="s" s="0">
+      <c r="B53" t="s">
         <v>301</v>
       </c>
       <c r="C53" s="6" t="s">
@@ -3865,11 +4003,11 @@
         <v>303</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="s" s="0">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
         <v>304</v>
       </c>
-      <c r="B54" t="s" s="0">
+      <c r="B54" t="s">
         <v>305</v>
       </c>
       <c r="C54" s="6" t="s">
@@ -3879,11 +4017,11 @@
         <v>307</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="s" s="0">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>308</v>
       </c>
-      <c r="B55" t="s" s="0">
+      <c r="B55" t="s">
         <v>309</v>
       </c>
       <c r="C55" s="6" t="s">
@@ -3893,11 +4031,11 @@
         <v>311</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="s" s="0">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>312</v>
       </c>
-      <c r="B56" t="s" s="0">
+      <c r="B56" t="s">
         <v>313</v>
       </c>
       <c r="C56" s="6" t="s">
@@ -3907,11 +4045,11 @@
         <v>315</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="s" s="0">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>316</v>
       </c>
-      <c r="B57" t="s" s="0">
+      <c r="B57" t="s">
         <v>317</v>
       </c>
       <c r="C57" s="6" t="s">
@@ -3921,11 +4059,11 @@
         <v>319</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="s" s="0">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>320</v>
       </c>
-      <c r="B58" t="s" s="0">
+      <c r="B58" t="s">
         <v>321</v>
       </c>
       <c r="C58" s="6" t="s">
@@ -3935,11 +4073,11 @@
         <v>323</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="s" s="0">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>324</v>
       </c>
-      <c r="B59" t="s" s="0">
+      <c r="B59" t="s">
         <v>325</v>
       </c>
       <c r="C59" s="6" t="s">
@@ -3949,11 +4087,11 @@
         <v>327</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="s" s="0">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>328</v>
       </c>
-      <c r="B60" t="s" s="0">
+      <c r="B60" t="s">
         <v>329</v>
       </c>
       <c r="C60" s="6" t="s">
@@ -3963,11 +4101,11 @@
         <v>331</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="s" s="0">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>332</v>
       </c>
-      <c r="B61" t="s" s="0">
+      <c r="B61" t="s">
         <v>333</v>
       </c>
       <c r="C61" s="6" t="s">
@@ -3977,11 +4115,11 @@
         <v>335</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="s" s="0">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>336</v>
       </c>
-      <c r="B62" t="s" s="0">
+      <c r="B62" t="s">
         <v>337</v>
       </c>
       <c r="C62" s="6" t="s">
@@ -3991,11 +4129,11 @@
         <v>339</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="s" s="0">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>340</v>
       </c>
-      <c r="B63" t="s" s="0">
+      <c r="B63" t="s">
         <v>341</v>
       </c>
       <c r="C63" s="6" t="s">
@@ -4005,11 +4143,11 @@
         <v>343</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="s" s="0">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>344</v>
       </c>
-      <c r="B64" t="s" s="0">
+      <c r="B64" t="s">
         <v>345</v>
       </c>
       <c r="C64" s="6" t="s">
@@ -4019,11 +4157,11 @@
         <v>347</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="s" s="0">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>348</v>
       </c>
-      <c r="B65" t="s" s="0">
+      <c r="B65" t="s">
         <v>349</v>
       </c>
       <c r="C65" s="6" t="s">
@@ -4033,11 +4171,11 @@
         <v>351</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="s" s="0">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>352</v>
       </c>
-      <c r="B66" t="s" s="0">
+      <c r="B66" t="s">
         <v>353</v>
       </c>
       <c r="C66" s="6" t="s">
@@ -4047,11 +4185,11 @@
         <v>355</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="s" s="0">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>356</v>
       </c>
-      <c r="B67" t="s" s="0">
+      <c r="B67" t="s">
         <v>357</v>
       </c>
       <c r="C67" s="6" t="s">
@@ -4061,11 +4199,11 @@
         <v>359</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="s" s="0">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>360</v>
       </c>
-      <c r="B68" t="s" s="0">
+      <c r="B68" t="s">
         <v>361</v>
       </c>
       <c r="C68" s="6" t="s">
@@ -4075,11 +4213,11 @@
         <v>363</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="s" s="0">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>364</v>
       </c>
-      <c r="B69" t="s" s="0">
+      <c r="B69" t="s">
         <v>365</v>
       </c>
       <c r="C69" s="6" t="s">
@@ -4089,11 +4227,11 @@
         <v>367</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="s" s="0">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>368</v>
       </c>
-      <c r="B70" t="s" s="0">
+      <c r="B70" t="s">
         <v>369</v>
       </c>
       <c r="C70" s="6" t="s">
@@ -4103,11 +4241,11 @@
         <v>371</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="s" s="0">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>372</v>
       </c>
-      <c r="B71" t="s" s="0">
+      <c r="B71" t="s">
         <v>373</v>
       </c>
       <c r="C71" s="6" t="s">
@@ -4117,11 +4255,11 @@
         <v>375</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="s" s="0">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>376</v>
       </c>
-      <c r="B72" t="s" s="0">
+      <c r="B72" t="s">
         <v>377</v>
       </c>
       <c r="C72" s="6" t="s">
@@ -4131,11 +4269,11 @@
         <v>379</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="s" s="0">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>380</v>
       </c>
-      <c r="B73" t="s" s="0">
+      <c r="B73" t="s">
         <v>381</v>
       </c>
       <c r="C73" s="6" t="s">
@@ -4145,11 +4283,11 @@
         <v>383</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="s" s="0">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>384</v>
       </c>
-      <c r="B74" t="s" s="0">
+      <c r="B74" t="s">
         <v>385</v>
       </c>
       <c r="C74" s="6" t="s">
@@ -4159,11 +4297,11 @@
         <v>387</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="s" s="0">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>388</v>
       </c>
-      <c r="B75" t="s" s="0">
+      <c r="B75" t="s">
         <v>389</v>
       </c>
       <c r="C75" s="6" t="s">
@@ -4173,11 +4311,11 @@
         <v>391</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="s" s="0">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>392</v>
       </c>
-      <c r="B76" t="s" s="0">
+      <c r="B76" t="s">
         <v>393</v>
       </c>
       <c r="C76" s="6" t="s">
@@ -4187,11 +4325,11 @@
         <v>395</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="s" s="0">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>396</v>
       </c>
-      <c r="B77" t="s" s="0">
+      <c r="B77" t="s">
         <v>397</v>
       </c>
       <c r="C77" s="6" t="s">
@@ -4201,11 +4339,11 @@
         <v>399</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="s" s="0">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>400</v>
       </c>
-      <c r="B78" t="s" s="0">
+      <c r="B78" t="s">
         <v>401</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -4215,11 +4353,11 @@
         <v>403</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="s" s="0">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>404</v>
       </c>
-      <c r="B79" t="s" s="0">
+      <c r="B79" t="s">
         <v>405</v>
       </c>
       <c r="C79" s="6" t="s">
@@ -4229,11 +4367,11 @@
         <v>407</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="s" s="0">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>408</v>
       </c>
-      <c r="B80" t="s" s="0">
+      <c r="B80" t="s">
         <v>409</v>
       </c>
       <c r="C80" s="6" t="s">
@@ -4243,11 +4381,11 @@
         <v>411</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="s" s="0">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>412</v>
       </c>
-      <c r="B81" t="s" s="0">
+      <c r="B81" t="s">
         <v>413</v>
       </c>
       <c r="C81" s="6" t="s">
@@ -4257,11 +4395,11 @@
         <v>415</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="s" s="0">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>416</v>
       </c>
-      <c r="B82" t="s" s="0">
+      <c r="B82" t="s">
         <v>417</v>
       </c>
       <c r="C82" s="6" t="s">
@@ -4271,11 +4409,11 @@
         <v>419</v>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="s" s="0">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
         <v>420</v>
       </c>
-      <c r="B83" t="s" s="0">
+      <c r="B83" t="s">
         <v>421</v>
       </c>
       <c r="C83" s="6" t="s">
@@ -4285,11 +4423,11 @@
         <v>423</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="s" s="0">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
         <v>424</v>
       </c>
-      <c r="B84" t="s" s="0">
+      <c r="B84" t="s">
         <v>425</v>
       </c>
       <c r="C84" s="6" t="s">
@@ -4299,11 +4437,11 @@
         <v>427</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="s" s="0">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
         <v>428</v>
       </c>
-      <c r="B85" t="s" s="0">
+      <c r="B85" t="s">
         <v>429</v>
       </c>
       <c r="C85" s="6" t="s">
@@ -4313,11 +4451,11 @@
         <v>431</v>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="s" s="0">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
         <v>432</v>
       </c>
-      <c r="B86" t="s" s="0">
+      <c r="B86" t="s">
         <v>433</v>
       </c>
       <c r="C86" s="6" t="s">
@@ -4327,11 +4465,11 @@
         <v>435</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="s" s="0">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
         <v>436</v>
       </c>
-      <c r="B87" t="s" s="0">
+      <c r="B87" t="s">
         <v>437</v>
       </c>
       <c r="C87" s="6" t="s">
@@ -4341,11 +4479,11 @@
         <v>439</v>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="s" s="0">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>440</v>
       </c>
-      <c r="B88" t="s" s="0">
+      <c r="B88" t="s">
         <v>441</v>
       </c>
       <c r="C88" s="6" t="s">
@@ -4355,11 +4493,11 @@
         <v>443</v>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="s" s="0">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>444</v>
       </c>
-      <c r="B89" t="s" s="0">
+      <c r="B89" t="s">
         <v>445</v>
       </c>
       <c r="C89" s="6" t="s">
@@ -4369,11 +4507,11 @@
         <v>447</v>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" t="s" s="0">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>448</v>
       </c>
-      <c r="B90" t="s" s="0">
+      <c r="B90" t="s">
         <v>449</v>
       </c>
       <c r="C90" s="6" t="s">
@@ -4383,11 +4521,11 @@
         <v>451</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="s" s="0">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
         <v>452</v>
       </c>
-      <c r="B91" t="s" s="0">
+      <c r="B91" t="s">
         <v>453</v>
       </c>
       <c r="C91" s="6" t="s">
@@ -4397,11 +4535,11 @@
         <v>455</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" t="s" s="0">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>456</v>
       </c>
-      <c r="B92" t="s" s="0">
+      <c r="B92" t="s">
         <v>457</v>
       </c>
       <c r="C92" s="6" t="s">
@@ -4411,11 +4549,11 @@
         <v>459</v>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" t="s" s="0">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
         <v>460</v>
       </c>
-      <c r="B93" t="s" s="0">
+      <c r="B93" t="s">
         <v>461</v>
       </c>
       <c r="C93" s="6" t="s">
@@ -4425,11 +4563,11 @@
         <v>463</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="s" s="0">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>464</v>
       </c>
-      <c r="B94" t="s" s="0">
+      <c r="B94" t="s">
         <v>465</v>
       </c>
       <c r="C94" s="6" t="s">
@@ -4439,11 +4577,11 @@
         <v>467</v>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" t="s" s="0">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>468</v>
       </c>
-      <c r="B95" t="s" s="0">
+      <c r="B95" t="s">
         <v>469</v>
       </c>
       <c r="C95" s="6" t="s">
@@ -4453,11 +4591,11 @@
         <v>471</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" t="s" s="0">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
         <v>472</v>
       </c>
-      <c r="B96" t="s" s="0">
+      <c r="B96" t="s">
         <v>473</v>
       </c>
       <c r="C96" s="6" t="s">
@@ -4467,11 +4605,11 @@
         <v>475</v>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" t="s" s="0">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
         <v>476</v>
       </c>
-      <c r="B97" t="s" s="0">
+      <c r="B97" t="s">
         <v>477</v>
       </c>
       <c r="C97" s="6" t="s">
@@ -4481,11 +4619,11 @@
         <v>479</v>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" t="s" s="0">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
         <v>480</v>
       </c>
-      <c r="B98" t="s" s="0">
+      <c r="B98" t="s">
         <v>481</v>
       </c>
       <c r="C98" s="6" t="s">
@@ -4495,11 +4633,11 @@
         <v>483</v>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" t="s" s="0">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
         <v>484</v>
       </c>
-      <c r="B99" t="s" s="0">
+      <c r="B99" t="s">
         <v>485</v>
       </c>
       <c r="C99" s="6" t="s">
@@ -4509,11 +4647,11 @@
         <v>487</v>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" t="s" s="0">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
         <v>488</v>
       </c>
-      <c r="B100" t="s" s="0">
+      <c r="B100" t="s">
         <v>489</v>
       </c>
       <c r="C100" s="6" t="s">
@@ -4523,11 +4661,11 @@
         <v>491</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" t="s" s="0">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>492</v>
       </c>
-      <c r="B101" t="s" s="0">
+      <c r="B101" t="s">
         <v>493</v>
       </c>
       <c r="C101" s="6" t="s">
@@ -4537,11 +4675,11 @@
         <v>495</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" t="s" s="0">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
         <v>496</v>
       </c>
-      <c r="B102" t="s" s="0">
+      <c r="B102" t="s">
         <v>497</v>
       </c>
       <c r="C102" s="6" t="s">
@@ -4551,11 +4689,11 @@
         <v>499</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" t="s" s="0">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
         <v>500</v>
       </c>
-      <c r="B103" t="s" s="0">
+      <c r="B103" t="s">
         <v>501</v>
       </c>
       <c r="C103" s="6" t="s">
@@ -4565,11 +4703,11 @@
         <v>503</v>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" t="s" s="0">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
         <v>504</v>
       </c>
-      <c r="B104" t="s" s="0">
+      <c r="B104" t="s">
         <v>505</v>
       </c>
       <c r="C104" s="6" t="s">
@@ -4579,11 +4717,11 @@
         <v>507</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" t="s" s="0">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
         <v>508</v>
       </c>
-      <c r="B105" t="s" s="0">
+      <c r="B105" t="s">
         <v>509</v>
       </c>
       <c r="C105" s="6" t="s">
@@ -4593,11 +4731,11 @@
         <v>511</v>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" t="s" s="0">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
         <v>512</v>
       </c>
-      <c r="B106" t="s" s="0">
+      <c r="B106" t="s">
         <v>513</v>
       </c>
       <c r="C106" s="6" t="s">
@@ -4607,11 +4745,11 @@
         <v>515</v>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" t="s" s="0">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
         <v>516</v>
       </c>
-      <c r="B107" t="s" s="0">
+      <c r="B107" t="s">
         <v>517</v>
       </c>
       <c r="C107" s="6" t="s">
@@ -4621,11 +4759,11 @@
         <v>519</v>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" t="s" s="0">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
         <v>520</v>
       </c>
-      <c r="B108" t="s" s="0">
+      <c r="B108" t="s">
         <v>521</v>
       </c>
       <c r="C108" s="6" t="s">
@@ -4635,11 +4773,11 @@
         <v>523</v>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" t="s" s="0">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
         <v>524</v>
       </c>
-      <c r="B109" t="s" s="0">
+      <c r="B109" t="s">
         <v>525</v>
       </c>
       <c r="C109" s="6" t="s">
@@ -4649,11 +4787,11 @@
         <v>527</v>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" t="s" s="0">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
         <v>528</v>
       </c>
-      <c r="B110" t="s" s="0">
+      <c r="B110" t="s">
         <v>529</v>
       </c>
       <c r="C110" s="6" t="s">
@@ -4663,11 +4801,11 @@
         <v>531</v>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" t="s" s="0">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
         <v>532</v>
       </c>
-      <c r="B111" t="s" s="0">
+      <c r="B111" t="s">
         <v>533</v>
       </c>
       <c r="C111" s="6" t="s">
@@ -4677,11 +4815,11 @@
         <v>535</v>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" t="s" s="0">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
         <v>536</v>
       </c>
-      <c r="B112" t="s" s="0">
+      <c r="B112" t="s">
         <v>537</v>
       </c>
       <c r="C112" s="6" t="s">
@@ -4691,11 +4829,11 @@
         <v>539</v>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" t="s" s="0">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
         <v>540</v>
       </c>
-      <c r="B113" t="s" s="0">
+      <c r="B113" t="s">
         <v>541</v>
       </c>
       <c r="C113" s="6" t="s">
@@ -4705,11 +4843,11 @@
         <v>543</v>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" t="s" s="0">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
         <v>544</v>
       </c>
-      <c r="B114" t="s" s="0">
+      <c r="B114" t="s">
         <v>545</v>
       </c>
       <c r="C114" s="6" t="s">
@@ -4719,11 +4857,11 @@
         <v>547</v>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" t="s" s="0">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
         <v>548</v>
       </c>
-      <c r="B115" t="s" s="0">
+      <c r="B115" t="s">
         <v>549</v>
       </c>
       <c r="C115" s="6" t="s">
@@ -4733,11 +4871,11 @@
         <v>551</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" t="s" s="0">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
         <v>552</v>
       </c>
-      <c r="B116" t="s" s="0">
+      <c r="B116" t="s">
         <v>553</v>
       </c>
       <c r="C116" s="6" t="s">
@@ -4747,11 +4885,11 @@
         <v>555</v>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" t="s" s="0">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
         <v>556</v>
       </c>
-      <c r="B117" t="s" s="0">
+      <c r="B117" t="s">
         <v>557</v>
       </c>
       <c r="C117" s="6" t="s">
@@ -4761,11 +4899,11 @@
         <v>559</v>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" t="s" s="0">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
         <v>560</v>
       </c>
-      <c r="B118" t="s" s="0">
+      <c r="B118" t="s">
         <v>561</v>
       </c>
       <c r="C118" s="6" t="s">
@@ -4775,11 +4913,11 @@
         <v>563</v>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" t="s" s="0">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
         <v>564</v>
       </c>
-      <c r="B119" t="s" s="0">
+      <c r="B119" t="s">
         <v>565</v>
       </c>
       <c r="C119" s="6" t="s">
@@ -4789,11 +4927,11 @@
         <v>567</v>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" t="s" s="0">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
         <v>568</v>
       </c>
-      <c r="B120" t="s" s="0">
+      <c r="B120" t="s">
         <v>569</v>
       </c>
       <c r="C120" s="6" t="s">
@@ -4803,11 +4941,11 @@
         <v>571</v>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" t="s" s="0">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
         <v>572</v>
       </c>
-      <c r="B121" t="s" s="0">
+      <c r="B121" t="s">
         <v>573</v>
       </c>
       <c r="C121" s="6" t="s">
@@ -4817,11 +4955,11 @@
         <v>575</v>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" t="s" s="0">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
         <v>576</v>
       </c>
-      <c r="B122" t="s" s="0">
+      <c r="B122" t="s">
         <v>577</v>
       </c>
       <c r="C122" s="6" t="s">
@@ -4831,11 +4969,11 @@
         <v>579</v>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" t="s" s="0">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
         <v>580</v>
       </c>
-      <c r="B123" t="s" s="0">
+      <c r="B123" t="s">
         <v>581</v>
       </c>
       <c r="C123" s="6" t="s">
@@ -4845,11 +4983,11 @@
         <v>583</v>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" t="s" s="0">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
         <v>584</v>
       </c>
-      <c r="B124" t="s" s="0">
+      <c r="B124" t="s">
         <v>585</v>
       </c>
       <c r="C124" s="6" t="s">
@@ -4859,11 +4997,11 @@
         <v>587</v>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" t="s" s="0">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
         <v>588</v>
       </c>
-      <c r="B125" t="s" s="0">
+      <c r="B125" t="s">
         <v>589</v>
       </c>
       <c r="C125" s="6" t="s">
@@ -4873,11 +5011,11 @@
         <v>591</v>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" t="s" s="0">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
         <v>592</v>
       </c>
-      <c r="B126" t="s" s="0">
+      <c r="B126" t="s">
         <v>593</v>
       </c>
       <c r="C126" s="6" t="s">
@@ -4887,11 +5025,11 @@
         <v>595</v>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" t="s" s="0">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
         <v>596</v>
       </c>
-      <c r="B127" t="s" s="0">
+      <c r="B127" t="s">
         <v>597</v>
       </c>
       <c r="C127" s="6" t="s">
@@ -4901,11 +5039,11 @@
         <v>599</v>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" t="s" s="0">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
         <v>600</v>
       </c>
-      <c r="B128" t="s" s="0">
+      <c r="B128" t="s">
         <v>601</v>
       </c>
       <c r="C128" s="6" t="s">
@@ -4915,11 +5053,11 @@
         <v>603</v>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" t="s" s="0">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
         <v>604</v>
       </c>
-      <c r="B129" t="s" s="0">
+      <c r="B129" t="s">
         <v>605</v>
       </c>
       <c r="C129" s="6" t="s">
@@ -4929,11 +5067,11 @@
         <v>607</v>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" t="s" s="0">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
         <v>608</v>
       </c>
-      <c r="B130" t="s" s="0">
+      <c r="B130" t="s">
         <v>609</v>
       </c>
       <c r="C130" s="6" t="s">
@@ -4943,11 +5081,11 @@
         <v>611</v>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" t="s" s="0">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
         <v>612</v>
       </c>
-      <c r="B131" t="s" s="0">
+      <c r="B131" t="s">
         <v>613</v>
       </c>
       <c r="C131" s="6" t="s">
@@ -4957,11 +5095,11 @@
         <v>615</v>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" t="s" s="0">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
         <v>616</v>
       </c>
-      <c r="B132" t="s" s="0">
+      <c r="B132" t="s">
         <v>617</v>
       </c>
       <c r="C132" s="6" t="s">
@@ -4971,11 +5109,11 @@
         <v>619</v>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" t="s" s="0">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
         <v>620</v>
       </c>
-      <c r="B133" t="s" s="0">
+      <c r="B133" t="s">
         <v>621</v>
       </c>
       <c r="C133" s="6" t="s">
@@ -4985,11 +5123,11 @@
         <v>623</v>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" t="s" s="0">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
         <v>624</v>
       </c>
-      <c r="B134" t="s" s="0">
+      <c r="B134" t="s">
         <v>625</v>
       </c>
       <c r="C134" s="6" t="s">
@@ -4999,11 +5137,11 @@
         <v>627</v>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" t="s" s="0">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
         <v>628</v>
       </c>
-      <c r="B135" t="s" s="0">
+      <c r="B135" t="s">
         <v>629</v>
       </c>
       <c r="C135" s="6" t="s">
@@ -5013,11 +5151,11 @@
         <v>631</v>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" t="s" s="0">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
         <v>632</v>
       </c>
-      <c r="B136" t="s" s="0">
+      <c r="B136" t="s">
         <v>633</v>
       </c>
       <c r="C136" s="6" t="s">
@@ -5027,11 +5165,11 @@
         <v>635</v>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" t="s" s="0">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
         <v>636</v>
       </c>
-      <c r="B137" t="s" s="0">
+      <c r="B137" t="s">
         <v>637</v>
       </c>
       <c r="C137" s="6" t="s">
@@ -5041,11 +5179,11 @@
         <v>639</v>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" t="s" s="0">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
         <v>640</v>
       </c>
-      <c r="B138" t="s" s="0">
+      <c r="B138" t="s">
         <v>641</v>
       </c>
       <c r="C138" s="6" t="s">
@@ -5055,11 +5193,11 @@
         <v>643</v>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" t="s" s="0">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
         <v>644</v>
       </c>
-      <c r="B139" t="s" s="0">
+      <c r="B139" t="s">
         <v>645</v>
       </c>
       <c r="C139" s="6" t="s">
@@ -5069,11 +5207,11 @@
         <v>647</v>
       </c>
     </row>
-    <row r="140">
-      <c r="A140" t="s" s="0">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
         <v>648</v>
       </c>
-      <c r="B140" t="s" s="0">
+      <c r="B140" t="s">
         <v>649</v>
       </c>
       <c r="C140" s="6" t="s">
@@ -5083,11 +5221,11 @@
         <v>651</v>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" t="s" s="0">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
         <v>652</v>
       </c>
-      <c r="B141" t="s" s="0">
+      <c r="B141" t="s">
         <v>653</v>
       </c>
       <c r="C141" s="6" t="s">
@@ -5097,11 +5235,11 @@
         <v>655</v>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" t="s" s="0">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
         <v>656</v>
       </c>
-      <c r="B142" t="s" s="0">
+      <c r="B142" t="s">
         <v>657</v>
       </c>
       <c r="C142" s="6" t="s">
@@ -5111,11 +5249,11 @@
         <v>659</v>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" t="s" s="0">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
         <v>660</v>
       </c>
-      <c r="B143" t="s" s="0">
+      <c r="B143" t="s">
         <v>661</v>
       </c>
       <c r="C143" s="6" t="s">
@@ -5125,11 +5263,11 @@
         <v>663</v>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" t="s" s="0">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
         <v>664</v>
       </c>
-      <c r="B144" t="s" s="0">
+      <c r="B144" t="s">
         <v>665</v>
       </c>
       <c r="C144" s="6" t="s">
@@ -5139,11 +5277,11 @@
         <v>667</v>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" t="s" s="0">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
         <v>668</v>
       </c>
-      <c r="B145" t="s" s="0">
+      <c r="B145" t="s">
         <v>669</v>
       </c>
       <c r="C145" s="6" t="s">
@@ -5153,11 +5291,11 @@
         <v>671</v>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" t="s" s="0">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
         <v>672</v>
       </c>
-      <c r="B146" t="s" s="0">
+      <c r="B146" t="s">
         <v>673</v>
       </c>
       <c r="C146" s="6" t="s">
@@ -5167,11 +5305,11 @@
         <v>675</v>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" t="s" s="0">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
         <v>676</v>
       </c>
-      <c r="B147" t="s" s="0">
+      <c r="B147" t="s">
         <v>677</v>
       </c>
       <c r="C147" s="6" t="s">
@@ -5181,11 +5319,11 @@
         <v>679</v>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" t="s" s="0">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
         <v>680</v>
       </c>
-      <c r="B148" t="s" s="0">
+      <c r="B148" t="s">
         <v>681</v>
       </c>
       <c r="C148" s="6" t="s">
@@ -5195,11 +5333,11 @@
         <v>683</v>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" t="s" s="0">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
         <v>684</v>
       </c>
-      <c r="B149" t="s" s="0">
+      <c r="B149" t="s">
         <v>685</v>
       </c>
       <c r="C149" s="6" t="s">
@@ -5209,11 +5347,11 @@
         <v>687</v>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" t="s" s="0">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
         <v>688</v>
       </c>
-      <c r="B150" t="s" s="0">
+      <c r="B150" t="s">
         <v>689</v>
       </c>
       <c r="C150" s="6" t="s">
@@ -5223,11 +5361,11 @@
         <v>691</v>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" t="s" s="0">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
         <v>692</v>
       </c>
-      <c r="B151" t="s" s="0">
+      <c r="B151" t="s">
         <v>693</v>
       </c>
       <c r="C151" s="6" t="s">
@@ -5237,11 +5375,11 @@
         <v>695</v>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" t="s" s="0">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
         <v>696</v>
       </c>
-      <c r="B152" t="s" s="0">
+      <c r="B152" t="s">
         <v>697</v>
       </c>
       <c r="C152" s="6" t="s">
@@ -5251,8 +5389,8 @@
         <v>699</v>
       </c>
     </row>
-    <row r="153">
-      <c r="B153" t="s" s="0">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B153" t="s">
         <v>700</v>
       </c>
       <c r="C153" s="6" t="s">
@@ -5262,8 +5400,8 @@
         <v>702</v>
       </c>
     </row>
-    <row r="154">
-      <c r="B154" t="s" s="0">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B154" t="s">
         <v>703</v>
       </c>
       <c r="C154" s="6" t="s">
@@ -5273,8 +5411,8 @@
         <v>705</v>
       </c>
     </row>
-    <row r="155">
-      <c r="B155" t="s" s="0">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B155" t="s">
         <v>706</v>
       </c>
       <c r="C155" s="6" t="s">
@@ -5284,8 +5422,8 @@
         <v>708</v>
       </c>
     </row>
-    <row r="156">
-      <c r="B156" t="s" s="0">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B156" t="s">
         <v>709</v>
       </c>
       <c r="C156" s="6" t="s">
@@ -5295,8 +5433,8 @@
         <v>711</v>
       </c>
     </row>
-    <row r="157">
-      <c r="B157" t="s" s="0">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B157" t="s">
         <v>712</v>
       </c>
       <c r="C157" s="6" t="s">
@@ -5306,8 +5444,8 @@
         <v>714</v>
       </c>
     </row>
-    <row r="158">
-      <c r="B158" t="s" s="0">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B158" t="s">
         <v>715</v>
       </c>
       <c r="C158" s="6" t="s">
@@ -5317,7 +5455,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="159">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C159" s="6" t="s">
         <v>718</v>
       </c>
@@ -5325,7 +5463,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="160">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C160" s="6" t="s">
         <v>720</v>
       </c>
@@ -5333,7 +5471,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="161">
+    <row r="161" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C161" s="6" t="s">
         <v>722</v>
       </c>
@@ -5341,7 +5479,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="162">
+    <row r="162" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C162" s="6" t="s">
         <v>724</v>
       </c>
@@ -5349,7 +5487,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="163">
+    <row r="163" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C163" s="6" t="s">
         <v>726</v>
       </c>
@@ -5357,7 +5495,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="164">
+    <row r="164" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C164" s="6" t="s">
         <v>728</v>
       </c>
@@ -5365,7 +5503,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="165">
+    <row r="165" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C165" s="6" t="s">
         <v>730</v>
       </c>
@@ -5373,7 +5511,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="166">
+    <row r="166" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C166" s="6" t="s">
         <v>732</v>
       </c>
@@ -5381,7 +5519,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="167">
+    <row r="167" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C167" s="6" t="s">
         <v>734</v>
       </c>
@@ -5389,7 +5527,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="168">
+    <row r="168" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C168" s="6" t="s">
         <v>736</v>
       </c>
@@ -5397,7 +5535,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="169">
+    <row r="169" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C169" s="6" t="s">
         <v>738</v>
       </c>
@@ -5405,7 +5543,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="170">
+    <row r="170" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C170" s="6" t="s">
         <v>740</v>
       </c>
@@ -5413,162 +5551,163 @@
         <v>741</v>
       </c>
     </row>
-    <row r="171">
+    <row r="171" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D171" s="5" t="s">
         <v>742</v>
       </c>
     </row>
-    <row r="172">
+    <row r="172" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D172" s="5" t="s">
         <v>743</v>
       </c>
     </row>
-    <row r="173">
+    <row r="173" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D173" s="5" t="s">
         <v>744</v>
       </c>
     </row>
-    <row r="174">
+    <row r="174" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D174" s="5" t="s">
         <v>745</v>
       </c>
     </row>
-    <row r="175">
+    <row r="175" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D175" s="5" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="176">
+    <row r="176" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D176" s="5" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="177">
+    <row r="177" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D177" s="5" t="s">
         <v>748</v>
       </c>
     </row>
-    <row r="178">
+    <row r="178" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D178" s="5" t="s">
         <v>749</v>
       </c>
     </row>
-    <row r="179">
+    <row r="179" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D179" s="5" t="s">
         <v>750</v>
       </c>
     </row>
-    <row r="180">
+    <row r="180" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D180" s="5" t="s">
         <v>751</v>
       </c>
     </row>
-    <row r="181">
+    <row r="181" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D181" s="5" t="s">
         <v>752</v>
       </c>
     </row>
-    <row r="182">
+    <row r="182" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D182" s="5" t="s">
         <v>753</v>
       </c>
     </row>
-    <row r="183">
+    <row r="183" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D183" s="5" t="s">
         <v>754</v>
       </c>
     </row>
-    <row r="184">
+    <row r="184" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D184" s="5" t="s">
         <v>755</v>
       </c>
     </row>
-    <row r="185">
+    <row r="185" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D185" s="5" t="s">
         <v>756</v>
       </c>
     </row>
-    <row r="186">
+    <row r="186" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D186" s="5" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="187">
+    <row r="187" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D187" s="5" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="188">
+    <row r="188" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D188" s="5" t="s">
         <v>759</v>
       </c>
     </row>
-    <row r="189">
+    <row r="189" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D189" s="5" t="s">
         <v>760</v>
       </c>
     </row>
-    <row r="190">
+    <row r="190" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D190" s="5" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="191">
+    <row r="191" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D191" s="5" t="s">
         <v>762</v>
       </c>
     </row>
-    <row r="192">
+    <row r="192" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D192" s="5" t="s">
         <v>763</v>
       </c>
     </row>
-    <row r="193">
+    <row r="193" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D193" s="5" t="s">
         <v>764</v>
       </c>
     </row>
-    <row r="194">
+    <row r="194" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D194" s="5" t="s">
         <v>765</v>
       </c>
     </row>
-    <row r="195">
+    <row r="195" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D195" s="5" t="s">
         <v>766</v>
       </c>
     </row>
-    <row r="196">
+    <row r="196" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D196" s="5" t="s">
         <v>767</v>
       </c>
     </row>
-    <row r="197">
+    <row r="197" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D197" s="5" t="s">
         <v>768</v>
       </c>
     </row>
-    <row r="198">
+    <row r="198" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D198" s="5" t="s">
         <v>769</v>
       </c>
     </row>
-    <row r="199">
+    <row r="199" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D199" s="5" t="s">
         <v>770</v>
       </c>
     </row>
-    <row r="200">
+    <row r="200" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D200" s="5" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="201">
+    <row r="201" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D201" s="5" t="s">
         <v>772</v>
       </c>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated the samples.xlsx file.
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -1,27 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tools\workspace\testing\animalBiome_Automation\src\test\resources\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14430" windowHeight="4320" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14430" windowHeight="4410" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
     <sheet name="PET_NAME" sheetId="2" r:id="rId2"/>
     <sheet name="ADD_PET" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:D13"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="886">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -2613,13 +2609,79 @@
   </si>
   <si>
     <t>Nexra</t>
+  </si>
+  <si>
+    <t>YNEAH4</t>
+  </si>
+  <si>
+    <t>P9D9TK</t>
+  </si>
+  <si>
+    <t>6KKKAD</t>
+  </si>
+  <si>
+    <t>PRUGRF</t>
+  </si>
+  <si>
+    <t>XMFPAV</t>
+  </si>
+  <si>
+    <t>CEVRRK</t>
+  </si>
+  <si>
+    <t>AXAPUP</t>
+  </si>
+  <si>
+    <t>K3JFMG</t>
+  </si>
+  <si>
+    <t>MMPTKX</t>
+  </si>
+  <si>
+    <t>T9EM4A</t>
+  </si>
+  <si>
+    <t>UG4AFF</t>
+  </si>
+  <si>
+    <t>EH6RXK</t>
+  </si>
+  <si>
+    <t>NDGPTY</t>
+  </si>
+  <si>
+    <t>JHERTN</t>
+  </si>
+  <si>
+    <t>7TETRT</t>
+  </si>
+  <si>
+    <t>7E6AKG</t>
+  </si>
+  <si>
+    <t>UE4CNR</t>
+  </si>
+  <si>
+    <t>PRR4EX</t>
+  </si>
+  <si>
+    <t>6ACVX7</t>
+  </si>
+  <si>
+    <t>FKHX4J</t>
+  </si>
+  <si>
+    <t>HVTUHY</t>
+  </si>
+  <si>
+    <t>MUEMAA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2631,6 +2693,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2653,12 +2722,18 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2668,16 +2743,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2"/>
     <cellStyle name="Normal 3" xfId="1"/>
-    <cellStyle name="Normal 2" xfId="2"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -2686,10 +2769,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -2821,7 +2904,6 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2845,11 +2927,10 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -2858,13 +2939,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cmpd="sng" algn="ctr">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2940,7 +3021,6 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2960,33 +3040,35 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K81"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.81641" style="1" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.36328" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.45313" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.63281" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
     <col min="6" max="6" width="18" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.26953" style="1" customWidth="1"/>
-    <col min="8" max="8" width="18.17969" style="1" customWidth="1"/>
-    <col min="9" max="9" width="18.36328" style="1" customWidth="1"/>
-    <col min="10" max="10" width="17.45313" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.726563" style="1"/>
+    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.5">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3018,7 +3100,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" ht="15.5">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -3035,7 +3117,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" ht="15.5">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -3052,7 +3134,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" ht="15.5">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3069,7 +3151,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" ht="15.5">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>25</v>
       </c>
@@ -3086,7 +3168,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" ht="15.5">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
@@ -3103,7 +3185,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" ht="15.5">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
@@ -3120,7 +3202,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" ht="15.5">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>40</v>
       </c>
@@ -3137,7 +3219,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" ht="15.5">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>45</v>
       </c>
@@ -3154,7 +3236,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" ht="15.5">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>50</v>
       </c>
@@ -3171,7 +3253,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" ht="15.5">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>55</v>
       </c>
@@ -3188,7 +3270,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" ht="15.5">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>60</v>
       </c>
@@ -3205,7 +3287,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" ht="15.5">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>65</v>
       </c>
@@ -3222,7 +3304,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="14" ht="15.5">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>70</v>
       </c>
@@ -3239,7 +3321,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" ht="15.5">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>75</v>
       </c>
@@ -3256,7 +3338,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" ht="15.5">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>80</v>
       </c>
@@ -3273,7 +3355,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="17" ht="15.5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>85</v>
       </c>
@@ -3290,7 +3372,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="18" ht="15.5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>90</v>
       </c>
@@ -3307,7 +3389,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="19" ht="15.5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>95</v>
       </c>
@@ -3324,7 +3406,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="20" ht="15.5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>100</v>
       </c>
@@ -3341,7 +3423,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="21" ht="15.5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>105</v>
       </c>
@@ -3358,7 +3440,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" ht="15.5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>110</v>
       </c>
@@ -3375,7 +3457,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="23" ht="15.5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>115</v>
       </c>
@@ -3392,7 +3474,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="24" ht="15.5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>120</v>
       </c>
@@ -3406,7 +3488,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="25" ht="15.5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>124</v>
       </c>
@@ -3417,7 +3499,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="26" ht="15.5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>127</v>
       </c>
@@ -3428,7 +3510,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="27" ht="15.5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>130</v>
       </c>
@@ -3439,7 +3521,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="28" ht="15.5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>133</v>
       </c>
@@ -3450,7 +3532,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="29" ht="15.5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>136</v>
       </c>
@@ -3461,7 +3543,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="30" ht="15.5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>139</v>
       </c>
@@ -3472,7 +3554,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="31" ht="15.5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>142</v>
       </c>
@@ -3483,7 +3565,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="32" ht="15.5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>145</v>
       </c>
@@ -3494,7 +3576,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="33" ht="15.5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>148</v>
       </c>
@@ -3505,127 +3587,215 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" ht="15.5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>880</v>
+      </c>
+      <c r="D34" t="s">
+        <v>874</v>
+      </c>
       <c r="E34" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="35" ht="15.5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>881</v>
+      </c>
+      <c r="D35" t="s">
+        <v>875</v>
+      </c>
       <c r="E35" s="2" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="36" ht="15.5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>882</v>
+      </c>
+      <c r="D36" t="s">
+        <v>876</v>
+      </c>
       <c r="E36" s="2" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="37" ht="15.5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>883</v>
+      </c>
+      <c r="D37" t="s">
+        <v>877</v>
+      </c>
       <c r="E37" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="38" ht="15.5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="D38" t="s">
+        <v>878</v>
+      </c>
       <c r="E38" s="2" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="39" ht="15.5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
+        <v>885</v>
+      </c>
+      <c r="D39" t="s">
+        <v>879</v>
+      </c>
       <c r="E39" s="2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="40" ht="15.5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E40" s="2" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="41" ht="15.5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E41" s="2" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="42" ht="15.5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E42" s="2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="43" ht="15.5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E43" s="2" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="44" ht="15.5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E44" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="45" ht="15.5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E45" s="1" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="46" ht="15.5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E46" s="1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="47" ht="15.5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E47" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="48" ht="15.5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E48" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="49" ht="15.5">
+    <row r="49" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E49" s="1" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="50" ht="15.5">
+    <row r="50" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E50" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="51" ht="15.5">
+    <row r="51" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E51" s="1" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="52" ht="15.5">
+    <row r="52" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E52" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="78" ht="15.5">
+    <row r="53" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E53" s="1" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="54" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E54" s="1" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E55" s="1" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="56" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E56" s="1" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="57" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E57" s="1" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="58" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E58" s="1" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="59" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E59" s="1" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="60" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E60" s="1" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="61" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E61" s="1" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="62" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E62" s="1" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="78" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F78" s="3"/>
     </row>
-    <row r="81" ht="15.5">
+    <row r="81" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F81" s="3"/>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.90625" customWidth="1"/>
-    <col min="2" max="2" width="29.45313" customWidth="1"/>
-    <col min="3" max="3" width="35.63281" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" customWidth="1"/>
     <col min="4" max="4" width="30.90625" customWidth="1"/>
-    <col min="5" max="5" width="32.72656" customWidth="1"/>
-    <col min="6" max="6" width="32.17969" customWidth="1"/>
-    <col min="7" max="7" width="33.63281" customWidth="1"/>
-    <col min="8" max="8" width="31.26953" customWidth="1"/>
+    <col min="5" max="5" width="32.7265625" customWidth="1"/>
+    <col min="6" max="6" width="32.1796875" customWidth="1"/>
+    <col min="7" max="7" width="33.6328125" customWidth="1"/>
+    <col min="8" max="8" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>170</v>
       </c>
@@ -3651,7 +3821,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>178</v>
       </c>
@@ -3661,9 +3831,8 @@
       <c r="C2" t="s">
         <v>178</v>
       </c>
-      <c r="D2"/>
-    </row>
-    <row r="3">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>178</v>
       </c>
@@ -3677,7 +3846,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>178</v>
       </c>
@@ -3686,24 +3855,26 @@
       </c>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H201"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.08984" customWidth="1"/>
-    <col min="2" max="2" width="17.54297" customWidth="1"/>
-    <col min="3" max="3" width="17.36328" customWidth="1"/>
-    <col min="4" max="5" width="17.26953" customWidth="1"/>
-    <col min="6" max="6" width="17.17969" customWidth="1"/>
-    <col min="7" max="7" width="15.36328" customWidth="1"/>
-    <col min="8" max="8" width="17.17969" customWidth="1"/>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="4" max="5" width="17.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.5">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>179</v>
       </c>
@@ -3729,7 +3900,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="2" ht="14.5">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>187</v>
       </c>
@@ -3743,7 +3914,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="3" ht="14.5">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>191</v>
       </c>
@@ -3757,7 +3928,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="4" ht="14.5">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>195</v>
       </c>
@@ -3771,7 +3942,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="5" ht="14.5">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>199</v>
       </c>
@@ -3785,7 +3956,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="6" ht="14.5">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>203</v>
       </c>
@@ -3799,7 +3970,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="7" ht="14.5">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>207</v>
       </c>
@@ -3813,7 +3984,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="8" ht="14.5">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>211</v>
       </c>
@@ -3827,7 +3998,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="9" ht="14.5">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>215</v>
       </c>
@@ -3841,7 +4012,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="10" ht="14.5">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>219</v>
       </c>
@@ -3855,7 +4026,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="11" ht="14.5">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>223</v>
       </c>
@@ -3869,7 +4040,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="12" ht="14.5">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>227</v>
       </c>
@@ -3883,7 +4054,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="13" ht="14.5">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>231</v>
       </c>
@@ -3897,7 +4068,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="14" ht="14.5">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>235</v>
       </c>
@@ -3911,7 +4082,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="15" ht="14.5">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>239</v>
       </c>
@@ -3925,7 +4096,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="16" ht="14.5">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>243</v>
       </c>
@@ -3939,7 +4110,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="17" ht="14.5">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>247</v>
       </c>
@@ -3953,7 +4124,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="18" ht="14.5">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>251</v>
       </c>
@@ -3967,7 +4138,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="19" ht="14.5">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>255</v>
       </c>
@@ -3981,7 +4152,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="20" ht="14.5">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>259</v>
       </c>
@@ -3995,7 +4166,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="21" ht="14.5">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>263</v>
       </c>
@@ -4009,7 +4180,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="22" ht="14.5">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>267</v>
       </c>
@@ -4023,7 +4194,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="23" ht="14.5">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>271</v>
       </c>
@@ -4037,7 +4208,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="24" ht="14.5">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>275</v>
       </c>
@@ -4051,7 +4222,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="25" ht="14.5">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>279</v>
       </c>
@@ -4065,7 +4236,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="26" ht="14.5">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>283</v>
       </c>
@@ -4079,7 +4250,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="27" ht="14.5">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>287</v>
       </c>
@@ -4093,7 +4264,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="28" ht="14.5">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>291</v>
       </c>
@@ -4107,7 +4278,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="29" ht="14.5">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>295</v>
       </c>
@@ -4121,7 +4292,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="30" ht="14.5">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>299</v>
       </c>
@@ -4135,7 +4306,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="31" ht="14.5">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>303</v>
       </c>
@@ -4149,7 +4320,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="32" ht="14.5">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>307</v>
       </c>
@@ -4163,7 +4334,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="33" ht="14.5">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>311</v>
       </c>
@@ -4177,7 +4348,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="34" ht="14.5">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>315</v>
       </c>
@@ -4191,7 +4362,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="35" ht="14.5">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>319</v>
       </c>
@@ -4205,7 +4376,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="36" ht="14.5">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>323</v>
       </c>
@@ -4219,7 +4390,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="37" ht="14.5">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>327</v>
       </c>
@@ -4233,7 +4404,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="38" ht="14.5">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>331</v>
       </c>
@@ -4247,7 +4418,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="39" ht="14.5">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>335</v>
       </c>
@@ -4261,7 +4432,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="40" ht="14.5">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>339</v>
       </c>
@@ -4275,7 +4446,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="41" ht="14.5">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>343</v>
       </c>
@@ -4289,7 +4460,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="42" ht="14.5">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>347</v>
       </c>
@@ -4303,7 +4474,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="43" ht="14.5">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>351</v>
       </c>
@@ -4317,7 +4488,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="44" ht="14.5">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>355</v>
       </c>
@@ -4331,7 +4502,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="45" ht="14.5">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>359</v>
       </c>
@@ -4345,7 +4516,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="46" ht="14.5">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>363</v>
       </c>
@@ -4359,7 +4530,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="47" ht="14.5">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>367</v>
       </c>
@@ -4373,7 +4544,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="48" ht="14.5">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>371</v>
       </c>
@@ -4387,7 +4558,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="49" ht="14.5">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>375</v>
       </c>
@@ -4401,7 +4572,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="50" ht="14.5">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>379</v>
       </c>
@@ -4415,7 +4586,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="51" ht="14.5">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>383</v>
       </c>
@@ -4429,7 +4600,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="52" ht="14.5">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>387</v>
       </c>
@@ -4443,7 +4614,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="53" ht="14.5">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>391</v>
       </c>
@@ -4457,7 +4628,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="54" ht="14.5">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>395</v>
       </c>
@@ -4471,7 +4642,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="55" ht="14.5">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>399</v>
       </c>
@@ -4485,7 +4656,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="56" ht="14.5">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>403</v>
       </c>
@@ -4499,7 +4670,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="57" ht="14.5">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>407</v>
       </c>
@@ -4513,7 +4684,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="58" ht="14.5">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>411</v>
       </c>
@@ -4527,7 +4698,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="59" ht="14.5">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>415</v>
       </c>
@@ -4541,7 +4712,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="60" ht="14.5">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>419</v>
       </c>
@@ -4555,7 +4726,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="61" ht="14.5">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>423</v>
       </c>
@@ -4569,7 +4740,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="62" ht="14.5">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>427</v>
       </c>
@@ -4583,7 +4754,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="63" ht="14.5">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>431</v>
       </c>
@@ -4597,7 +4768,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="64" ht="14.5">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>435</v>
       </c>
@@ -4611,7 +4782,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="65" ht="14.5">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>439</v>
       </c>
@@ -4625,7 +4796,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="66" ht="14.5">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>443</v>
       </c>
@@ -4639,7 +4810,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="67" ht="14.5">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>447</v>
       </c>
@@ -4653,7 +4824,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="68" ht="14.5">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>451</v>
       </c>
@@ -4667,7 +4838,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="69" ht="14.5">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>455</v>
       </c>
@@ -4681,7 +4852,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="70" ht="14.5">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>459</v>
       </c>
@@ -4695,7 +4866,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="71" ht="14.5">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>463</v>
       </c>
@@ -4709,7 +4880,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="72" ht="14.5">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>467</v>
       </c>
@@ -4723,7 +4894,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="73" ht="14.5">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>471</v>
       </c>
@@ -4737,7 +4908,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="74" ht="14.5">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>475</v>
       </c>
@@ -4751,7 +4922,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="75" ht="14.5">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>479</v>
       </c>
@@ -4765,7 +4936,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="76" ht="14.5">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>483</v>
       </c>
@@ -4779,7 +4950,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="77" ht="14.5">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>487</v>
       </c>
@@ -4793,7 +4964,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="78" ht="14.5">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>491</v>
       </c>
@@ -4807,7 +4978,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="79" ht="14.5">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>495</v>
       </c>
@@ -4821,7 +4992,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="80" ht="14.5">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>499</v>
       </c>
@@ -4835,7 +5006,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="81" ht="14.5">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>503</v>
       </c>
@@ -4849,7 +5020,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="82" ht="14.5">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>507</v>
       </c>
@@ -4863,7 +5034,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="83" ht="14.5">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>511</v>
       </c>
@@ -4877,7 +5048,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="84" ht="14.5">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>515</v>
       </c>
@@ -4891,7 +5062,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="85" ht="14.5">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>519</v>
       </c>
@@ -4905,7 +5076,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="86" ht="14.5">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>523</v>
       </c>
@@ -4919,7 +5090,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="87" ht="14.5">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>527</v>
       </c>
@@ -4933,7 +5104,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="88" ht="14.5">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>531</v>
       </c>
@@ -4947,7 +5118,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="89" ht="14.5">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>535</v>
       </c>
@@ -4961,7 +5132,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="90" ht="14.5">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>539</v>
       </c>
@@ -4975,7 +5146,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="91" ht="14.5">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>543</v>
       </c>
@@ -4989,7 +5160,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="92" ht="14.5">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>547</v>
       </c>
@@ -5003,7 +5174,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="93" ht="14.5">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>551</v>
       </c>
@@ -5017,7 +5188,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="94" ht="14.5">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>555</v>
       </c>
@@ -5031,7 +5202,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="95" ht="14.5">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>559</v>
       </c>
@@ -5045,7 +5216,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="96" ht="14.5">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>563</v>
       </c>
@@ -5059,7 +5230,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="97" ht="14.5">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>567</v>
       </c>
@@ -5073,7 +5244,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="98" ht="14.5">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>571</v>
       </c>
@@ -5087,7 +5258,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="99" ht="14.5">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>575</v>
       </c>
@@ -5101,7 +5272,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="100" ht="14.5">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>579</v>
       </c>
@@ -5115,7 +5286,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="101" ht="14.5">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>583</v>
       </c>
@@ -5129,7 +5300,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="102" ht="14.5">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>587</v>
       </c>
@@ -5143,7 +5314,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="103" ht="14.5">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>591</v>
       </c>
@@ -5157,7 +5328,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="104" ht="14.5">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>595</v>
       </c>
@@ -5171,7 +5342,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="105" ht="14.5">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>599</v>
       </c>
@@ -5185,7 +5356,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="106" ht="14.5">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>603</v>
       </c>
@@ -5199,7 +5370,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="107" ht="14.5">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>607</v>
       </c>
@@ -5213,7 +5384,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="108" ht="14.5">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>611</v>
       </c>
@@ -5227,7 +5398,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="109" ht="14.5">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>615</v>
       </c>
@@ -5241,7 +5412,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="110" ht="14.5">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>619</v>
       </c>
@@ -5255,7 +5426,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="111" ht="14.5">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>623</v>
       </c>
@@ -5269,7 +5440,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="112" ht="14.5">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>627</v>
       </c>
@@ -5283,7 +5454,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="113" ht="14.5">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>631</v>
       </c>
@@ -5297,7 +5468,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="114" ht="14.5">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>635</v>
       </c>
@@ -5311,7 +5482,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="115" ht="14.5">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>639</v>
       </c>
@@ -5325,7 +5496,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="116" ht="14.5">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>643</v>
       </c>
@@ -5339,7 +5510,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="117" ht="14.5">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>647</v>
       </c>
@@ -5353,7 +5524,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="118" ht="14.5">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>651</v>
       </c>
@@ -5367,7 +5538,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="119" ht="14.5">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>655</v>
       </c>
@@ -5381,7 +5552,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="120" ht="14.5">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>659</v>
       </c>
@@ -5395,7 +5566,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="121" ht="14.5">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>663</v>
       </c>
@@ -5409,7 +5580,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="122" ht="14.5">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>667</v>
       </c>
@@ -5423,7 +5594,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="123" ht="14.5">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>671</v>
       </c>
@@ -5437,7 +5608,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="124" ht="14.5">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>675</v>
       </c>
@@ -5451,7 +5622,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="125" ht="14.5">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>679</v>
       </c>
@@ -5465,7 +5636,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="126" ht="14.5">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>683</v>
       </c>
@@ -5479,7 +5650,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="127" ht="14.5">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>687</v>
       </c>
@@ -5493,7 +5664,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="128" ht="14.5">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>691</v>
       </c>
@@ -5507,7 +5678,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="129" ht="14.5">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>695</v>
       </c>
@@ -5521,7 +5692,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="130" ht="14.5">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>699</v>
       </c>
@@ -5535,7 +5706,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="131" ht="14.5">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>703</v>
       </c>
@@ -5549,7 +5720,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="132" ht="14.5">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>707</v>
       </c>
@@ -5563,7 +5734,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="133" ht="14.5">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>711</v>
       </c>
@@ -5577,7 +5748,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="134" ht="14.5">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>715</v>
       </c>
@@ -5591,7 +5762,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="135" ht="14.5">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>719</v>
       </c>
@@ -5605,7 +5776,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="136" ht="14.5">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>723</v>
       </c>
@@ -5619,7 +5790,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="137" ht="14.5">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>727</v>
       </c>
@@ -5633,7 +5804,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="138" ht="14.5">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>731</v>
       </c>
@@ -5647,7 +5818,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="139" ht="14.5">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>735</v>
       </c>
@@ -5661,7 +5832,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="140" ht="14.5">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>739</v>
       </c>
@@ -5675,7 +5846,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="141" ht="14.5">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>743</v>
       </c>
@@ -5689,7 +5860,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="142" ht="14.5">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>747</v>
       </c>
@@ -5703,7 +5874,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="143" ht="14.5">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>751</v>
       </c>
@@ -5717,7 +5888,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="144" ht="14.5">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>755</v>
       </c>
@@ -5731,7 +5902,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="145" ht="14.5">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>759</v>
       </c>
@@ -5745,7 +5916,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="146" ht="14.5">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>763</v>
       </c>
@@ -5759,7 +5930,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="147" ht="14.5">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>767</v>
       </c>
@@ -5773,7 +5944,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="148" ht="14.5">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>771</v>
       </c>
@@ -5787,7 +5958,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="149" ht="14.5">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>775</v>
       </c>
@@ -5801,7 +5972,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="150" ht="14.5">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>779</v>
       </c>
@@ -5815,7 +5986,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="151" ht="14.5">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>783</v>
       </c>
@@ -5829,7 +6000,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="152" ht="14.5">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>787</v>
       </c>
@@ -5843,7 +6014,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="153" ht="14.5">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B153" t="s">
         <v>791</v>
       </c>
@@ -5854,7 +6025,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="154" ht="14.5">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B154" t="s">
         <v>794</v>
       </c>
@@ -5865,7 +6036,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="155" ht="14.5">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B155" t="s">
         <v>797</v>
       </c>
@@ -5876,7 +6047,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="156" ht="14.5">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B156" t="s">
         <v>800</v>
       </c>
@@ -5887,7 +6058,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="157" ht="14.5">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B157" t="s">
         <v>803</v>
       </c>
@@ -5898,7 +6069,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="158" ht="14.5">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B158" t="s">
         <v>806</v>
       </c>
@@ -5909,7 +6080,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="159" ht="14.5">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C159" s="6" t="s">
         <v>809</v>
       </c>
@@ -5917,7 +6088,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="160" ht="14.5">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C160" s="6" t="s">
         <v>811</v>
       </c>
@@ -5925,7 +6096,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="161" ht="14.5">
+    <row r="161" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C161" s="6" t="s">
         <v>813</v>
       </c>
@@ -5933,7 +6104,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="162" ht="14.5">
+    <row r="162" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C162" s="6" t="s">
         <v>815</v>
       </c>
@@ -5941,7 +6112,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="163" ht="14.5">
+    <row r="163" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C163" s="6" t="s">
         <v>817</v>
       </c>
@@ -5949,7 +6120,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="164" ht="14.5">
+    <row r="164" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C164" s="6" t="s">
         <v>819</v>
       </c>
@@ -5957,7 +6128,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="165" ht="14.5">
+    <row r="165" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C165" s="6" t="s">
         <v>821</v>
       </c>
@@ -5965,7 +6136,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="166" ht="14.5">
+    <row r="166" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C166" s="6" t="s">
         <v>823</v>
       </c>
@@ -5973,7 +6144,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="167" ht="14.5">
+    <row r="167" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C167" s="6" t="s">
         <v>825</v>
       </c>
@@ -5981,7 +6152,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="168" ht="14.5">
+    <row r="168" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C168" s="6" t="s">
         <v>827</v>
       </c>
@@ -5989,7 +6160,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="169" ht="14.5">
+    <row r="169" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C169" s="6" t="s">
         <v>829</v>
       </c>
@@ -5997,7 +6168,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="170" ht="14.5">
+    <row r="170" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C170" s="6" t="s">
         <v>831</v>
       </c>
@@ -6005,162 +6176,163 @@
         <v>832</v>
       </c>
     </row>
-    <row r="171" ht="14.5">
+    <row r="171" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D171" s="5" t="s">
         <v>833</v>
       </c>
     </row>
-    <row r="172" ht="14.5">
+    <row r="172" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D172" s="5" t="s">
         <v>834</v>
       </c>
     </row>
-    <row r="173" ht="14.5">
+    <row r="173" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D173" s="5" t="s">
         <v>835</v>
       </c>
     </row>
-    <row r="174" ht="14.5">
+    <row r="174" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D174" s="5" t="s">
         <v>836</v>
       </c>
     </row>
-    <row r="175" ht="14.5">
+    <row r="175" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D175" s="5" t="s">
         <v>837</v>
       </c>
     </row>
-    <row r="176" ht="14.5">
+    <row r="176" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D176" s="5" t="s">
         <v>838</v>
       </c>
     </row>
-    <row r="177" ht="14.5">
+    <row r="177" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D177" s="5" t="s">
         <v>839</v>
       </c>
     </row>
-    <row r="178" ht="14.5">
+    <row r="178" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D178" s="5" t="s">
         <v>840</v>
       </c>
     </row>
-    <row r="179" ht="14.5">
+    <row r="179" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D179" s="5" t="s">
         <v>841</v>
       </c>
     </row>
-    <row r="180" ht="14.5">
+    <row r="180" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D180" s="5" t="s">
         <v>842</v>
       </c>
     </row>
-    <row r="181" ht="14.5">
+    <row r="181" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D181" s="5" t="s">
         <v>843</v>
       </c>
     </row>
-    <row r="182" ht="14.5">
+    <row r="182" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D182" s="5" t="s">
         <v>844</v>
       </c>
     </row>
-    <row r="183" ht="14.5">
+    <row r="183" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D183" s="5" t="s">
         <v>845</v>
       </c>
     </row>
-    <row r="184" ht="14.5">
+    <row r="184" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D184" s="5" t="s">
         <v>846</v>
       </c>
     </row>
-    <row r="185" ht="14.5">
+    <row r="185" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D185" s="5" t="s">
         <v>847</v>
       </c>
     </row>
-    <row r="186" ht="14.5">
+    <row r="186" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D186" s="5" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="187" ht="14.5">
+    <row r="187" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D187" s="5" t="s">
         <v>849</v>
       </c>
     </row>
-    <row r="188" ht="14.5">
+    <row r="188" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D188" s="5" t="s">
         <v>850</v>
       </c>
     </row>
-    <row r="189" ht="14.5">
+    <row r="189" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D189" s="5" t="s">
         <v>851</v>
       </c>
     </row>
-    <row r="190" ht="14.5">
+    <row r="190" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D190" s="5" t="s">
         <v>852</v>
       </c>
     </row>
-    <row r="191" ht="14.5">
+    <row r="191" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D191" s="5" t="s">
         <v>853</v>
       </c>
     </row>
-    <row r="192" ht="14.5">
+    <row r="192" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D192" s="5" t="s">
         <v>854</v>
       </c>
     </row>
-    <row r="193" ht="14.5">
+    <row r="193" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D193" s="5" t="s">
         <v>855</v>
       </c>
     </row>
-    <row r="194" ht="14.5">
+    <row r="194" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D194" s="5" t="s">
         <v>856</v>
       </c>
     </row>
-    <row r="195" ht="14.5">
+    <row r="195" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D195" s="5" t="s">
         <v>857</v>
       </c>
     </row>
-    <row r="196" ht="14.5">
+    <row r="196" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D196" s="5" t="s">
         <v>858</v>
       </c>
     </row>
-    <row r="197" ht="14.5">
+    <row r="197" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D197" s="5" t="s">
         <v>859</v>
       </c>
     </row>
-    <row r="198" ht="14.5">
+    <row r="198" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D198" s="5" t="s">
         <v>860</v>
       </c>
     </row>
-    <row r="199" ht="14.5">
+    <row r="199" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D199" s="5" t="s">
         <v>861</v>
       </c>
     </row>
-    <row r="200" ht="14.5">
+    <row r="200" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D200" s="5" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="201" ht="14.5">
+    <row r="201" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D201" s="5" t="s">
         <v>863</v>
       </c>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated email report template
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -1,27 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tools\workspace\testing\animalBiome_Automation\src\test\resources\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14430" windowHeight="4110" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14430" windowHeight="3390"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
     <sheet name="PET_NAME" sheetId="2" r:id="rId2"/>
     <sheet name="ADD_PET" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A10:G18"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="820">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -2420,66 +2416,74 @@
     <t>Nexra</t>
   </si>
   <si>
-    <t>Charlie114</t>
-  </si>
-  <si>
-    <t>Milo83</t>
-  </si>
-  <si>
-    <t>Taffy81</t>
-  </si>
-  <si>
-    <t>Cutie68</t>
-  </si>
-  <si>
-    <t>Cinder68</t>
-  </si>
-  <si>
-    <t>pony60</t>
-  </si>
-  <si>
-    <t>fury57</t>
-  </si>
-  <si>
-    <t>Rabbit58</t>
-  </si>
-  <si>
-    <t>Sheep47</t>
-  </si>
-  <si>
-    <t>Charlie115</t>
-  </si>
-  <si>
-    <t>Milo84</t>
-  </si>
-  <si>
-    <t>Taffy82</t>
-  </si>
-  <si>
-    <t>Cutie69</t>
-  </si>
-  <si>
-    <t>Cinder69</t>
-  </si>
-  <si>
-    <t>pony61</t>
-  </si>
-  <si>
-    <t>fury58</t>
-  </si>
-  <si>
-    <t>Rabbit59</t>
-  </si>
-  <si>
-    <t>Sheep48</t>
+    <t>ATVGRK</t>
+  </si>
+  <si>
+    <t>AMYGYD</t>
+  </si>
+  <si>
+    <t>EXVDDD</t>
+  </si>
+  <si>
+    <t>CTCP4P</t>
+  </si>
+  <si>
+    <t>AUNGFE</t>
+  </si>
+  <si>
+    <t>PM9DRK</t>
+  </si>
+  <si>
+    <t>HVMT9H</t>
+  </si>
+  <si>
+    <t>9AKFMJ</t>
+  </si>
+  <si>
+    <t>JKNFGJ</t>
+  </si>
+  <si>
+    <t>XHPJDV</t>
+  </si>
+  <si>
+    <t>U7KEKR</t>
+  </si>
+  <si>
+    <t>HV7FNT</t>
+  </si>
+  <si>
+    <t>VYF9NN</t>
+  </si>
+  <si>
+    <t>UN9CKJ</t>
+  </si>
+  <si>
+    <t>KUMPNY</t>
+  </si>
+  <si>
+    <t>RPXM9Y</t>
+  </si>
+  <si>
+    <t>H6U4FG</t>
+  </si>
+  <si>
+    <t>MR7NGM</t>
+  </si>
+  <si>
+    <t>A7NM49</t>
+  </si>
+  <si>
+    <t>79XDNU</t>
+  </si>
+  <si>
+    <t>9MRN7E</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2491,6 +2495,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2513,12 +2524,18 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2528,38 +2545,46 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2"/>
     <cellStyle name="Normal 3" xfId="1"/>
-    <cellStyle name="Normal 2" xfId="2"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -2568,10 +2593,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -2703,7 +2728,6 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2727,11 +2751,10 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -2740,13 +2763,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cmpd="sng" algn="ctr">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2822,7 +2845,6 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2842,34 +2864,35 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J81"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K81"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="17.81641"/>
-    <col min="2" max="2" customWidth="true" style="1" width="15.0"/>
-    <col min="3" max="3" customWidth="true" style="1" width="15.36328"/>
-    <col min="4" max="4" customWidth="true" style="1" width="17.45313"/>
-    <col min="5" max="5" customWidth="true" style="1" width="16.63281"/>
-    <col min="6" max="6" customWidth="true" style="1" width="18.0"/>
-    <col min="7" max="7" customWidth="true" style="1" width="17.26953"/>
-    <col min="8" max="8" customWidth="true" style="1" width="18.17969"/>
-    <col min="9" max="9" customWidth="true" style="1" width="18.36328"/>
-    <col min="10" max="10" customWidth="true" style="1" width="17.45313"/>
-    <col min="11" max="11" customWidth="true" style="1" width="17.36328"/>
-    <col min="12" max="16384" style="1" width="8.726563"/>
+    <col min="1" max="1" width="17.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.36328125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2901,7 +2924,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2918,7 +2941,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -2935,7 +2958,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2952,7 +2975,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>25</v>
       </c>
@@ -2969,7 +2992,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
@@ -2986,7 +3009,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
@@ -3003,7 +3026,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>40</v>
       </c>
@@ -3020,7 +3043,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>45</v>
       </c>
@@ -3037,7 +3060,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>50</v>
       </c>
@@ -3054,7 +3077,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>55</v>
       </c>
@@ -3071,7 +3094,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>60</v>
       </c>
@@ -3088,7 +3111,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>65</v>
       </c>
@@ -3105,7 +3128,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="18" t="s">
         <v>70</v>
       </c>
@@ -3122,7 +3145,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="20" t="s">
         <v>75</v>
       </c>
@@ -3139,7 +3162,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>80</v>
       </c>
@@ -3156,7 +3179,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>85</v>
       </c>
@@ -3173,7 +3196,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>90</v>
       </c>
@@ -3190,7 +3213,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>95</v>
       </c>
@@ -3207,7 +3230,10 @@
         <v>99</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>809</v>
+      </c>
       <c r="B20" s="1" t="s">
         <v>100</v>
       </c>
@@ -3218,166 +3244,239 @@
         <v>102</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>810</v>
+      </c>
+      <c r="D21" t="s">
+        <v>815</v>
+      </c>
       <c r="E21" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>811</v>
+      </c>
+      <c r="D22" t="s">
+        <v>816</v>
+      </c>
       <c r="E22" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="78">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>812</v>
+      </c>
+      <c r="D23" t="s">
+        <v>817</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>813</v>
+      </c>
+      <c r="D24" t="s">
+        <v>818</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>814</v>
+      </c>
+      <c r="D25" t="s">
+        <v>819</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E26" s="1" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E27" s="1" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E28" s="1" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E29" s="1" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E30" s="1" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E31" s="1" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E32" s="1" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="78" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F78" s="3"/>
     </row>
-    <row r="81">
+    <row r="81" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F81" s="3"/>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="26.90625"/>
-    <col min="2" max="2" customWidth="true" width="29.45313"/>
-    <col min="3" max="3" customWidth="true" width="35.63281"/>
-    <col min="4" max="4" customWidth="true" width="30.90625"/>
-    <col min="5" max="5" customWidth="true" width="32.72656"/>
-    <col min="6" max="6" customWidth="true" width="32.17969"/>
-    <col min="7" max="7" customWidth="true" width="33.63281"/>
-    <col min="8" max="8" customWidth="true" width="31.26953"/>
+    <col min="1" max="1" width="26.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" customWidth="1"/>
+    <col min="4" max="4" width="30.90625" customWidth="1"/>
+    <col min="5" max="5" width="32.7265625" customWidth="1"/>
+    <col min="6" max="6" width="32.1796875" customWidth="1"/>
+    <col min="7" max="7" width="33.6328125" customWidth="1"/>
+    <col min="8" max="8" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>105</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>106</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>107</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>108</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>109</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>110</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>111</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>113</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>113</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>113</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>113</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>113</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>113</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>113</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="0"/>
-      <c r="D4" s="0"/>
-    </row>
-    <row r="5">
-      <c r="C5" s="0"/>
-      <c r="D5" s="0"/>
-    </row>
-    <row r="6">
-      <c r="C6" s="0"/>
-    </row>
-    <row r="7">
-      <c r="C7" s="0"/>
-    </row>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35"/>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H201"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.08984"/>
-    <col min="2" max="2" customWidth="true" width="17.54297"/>
-    <col min="3" max="3" customWidth="true" width="17.36328"/>
-    <col min="4" max="5" customWidth="true" width="17.26953"/>
-    <col min="6" max="6" customWidth="true" width="17.17969"/>
-    <col min="7" max="7" customWidth="true" width="15.36328"/>
-    <col min="8" max="8" customWidth="true" width="17.17969"/>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="4" max="5" width="17.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.5">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>115</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>116</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>117</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>118</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>119</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>120</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="2" ht="14.5">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>122</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>123</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -3387,11 +3486,11 @@
         <v>125</v>
       </c>
     </row>
-    <row r="3" ht="14.5">
-      <c r="A3" t="s" s="0">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>126</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>127</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -3401,11 +3500,11 @@
         <v>129</v>
       </c>
     </row>
-    <row r="4" ht="14.5">
-      <c r="A4" t="s" s="0">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>130</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>131</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -3415,11 +3514,11 @@
         <v>133</v>
       </c>
     </row>
-    <row r="5" ht="14.5">
-      <c r="A5" t="s" s="0">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>134</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>135</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -3429,11 +3528,11 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" ht="14.5">
-      <c r="A6" t="s" s="0">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>138</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>139</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -3443,11 +3542,11 @@
         <v>141</v>
       </c>
     </row>
-    <row r="7" ht="14.5">
-      <c r="A7" t="s" s="0">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>142</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s">
         <v>143</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -3457,11 +3556,11 @@
         <v>145</v>
       </c>
     </row>
-    <row r="8" ht="14.5">
-      <c r="A8" t="s" s="0">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>146</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="B8" t="s">
         <v>147</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -3471,11 +3570,11 @@
         <v>149</v>
       </c>
     </row>
-    <row r="9" ht="14.5">
-      <c r="A9" t="s" s="0">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>150</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="B9" t="s">
         <v>151</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -3485,11 +3584,11 @@
         <v>153</v>
       </c>
     </row>
-    <row r="10" ht="14.5">
-      <c r="A10" t="s" s="0">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>154</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="B10" t="s">
         <v>155</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -3499,11 +3598,11 @@
         <v>157</v>
       </c>
     </row>
-    <row r="11" ht="14.5">
-      <c r="A11" t="s" s="0">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>158</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="B11" t="s">
         <v>159</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -3513,11 +3612,11 @@
         <v>161</v>
       </c>
     </row>
-    <row r="12" ht="14.5">
-      <c r="A12" t="s" s="0">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>162</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="B12" t="s">
         <v>163</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -3527,11 +3626,11 @@
         <v>165</v>
       </c>
     </row>
-    <row r="13" ht="14.5">
-      <c r="A13" t="s" s="0">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>166</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="B13" t="s">
         <v>167</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -3541,11 +3640,11 @@
         <v>169</v>
       </c>
     </row>
-    <row r="14" ht="14.5">
-      <c r="A14" t="s" s="0">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>170</v>
       </c>
-      <c r="B14" t="s" s="0">
+      <c r="B14" t="s">
         <v>171</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -3555,11 +3654,11 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" ht="14.5">
-      <c r="A15" t="s" s="0">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>174</v>
       </c>
-      <c r="B15" t="s" s="0">
+      <c r="B15" t="s">
         <v>175</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -3569,11 +3668,11 @@
         <v>177</v>
       </c>
     </row>
-    <row r="16" ht="14.5">
-      <c r="A16" t="s" s="0">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>178</v>
       </c>
-      <c r="B16" t="s" s="0">
+      <c r="B16" t="s">
         <v>179</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -3583,11 +3682,11 @@
         <v>181</v>
       </c>
     </row>
-    <row r="17" ht="14.5">
-      <c r="A17" t="s" s="0">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>182</v>
       </c>
-      <c r="B17" t="s" s="0">
+      <c r="B17" t="s">
         <v>183</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -3597,11 +3696,11 @@
         <v>185</v>
       </c>
     </row>
-    <row r="18" ht="14.5">
-      <c r="A18" t="s" s="0">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>186</v>
       </c>
-      <c r="B18" t="s" s="0">
+      <c r="B18" t="s">
         <v>187</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -3611,11 +3710,11 @@
         <v>189</v>
       </c>
     </row>
-    <row r="19" ht="14.5">
-      <c r="A19" t="s" s="0">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>190</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="B19" t="s">
         <v>191</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -3625,11 +3724,11 @@
         <v>193</v>
       </c>
     </row>
-    <row r="20" ht="14.5">
-      <c r="A20" t="s" s="0">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>194</v>
       </c>
-      <c r="B20" t="s" s="0">
+      <c r="B20" t="s">
         <v>195</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -3639,11 +3738,11 @@
         <v>197</v>
       </c>
     </row>
-    <row r="21" ht="14.5">
-      <c r="A21" t="s" s="0">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>198</v>
       </c>
-      <c r="B21" t="s" s="0">
+      <c r="B21" t="s">
         <v>199</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -3653,11 +3752,11 @@
         <v>201</v>
       </c>
     </row>
-    <row r="22" ht="14.5">
-      <c r="A22" t="s" s="0">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>202</v>
       </c>
-      <c r="B22" t="s" s="0">
+      <c r="B22" t="s">
         <v>203</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -3667,11 +3766,11 @@
         <v>205</v>
       </c>
     </row>
-    <row r="23" ht="14.5">
-      <c r="A23" t="s" s="0">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>206</v>
       </c>
-      <c r="B23" t="s" s="0">
+      <c r="B23" t="s">
         <v>207</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -3681,11 +3780,11 @@
         <v>209</v>
       </c>
     </row>
-    <row r="24" ht="14.5">
-      <c r="A24" t="s" s="0">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>210</v>
       </c>
-      <c r="B24" t="s" s="0">
+      <c r="B24" t="s">
         <v>211</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -3695,11 +3794,11 @@
         <v>213</v>
       </c>
     </row>
-    <row r="25" ht="14.5">
-      <c r="A25" t="s" s="0">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>214</v>
       </c>
-      <c r="B25" t="s" s="0">
+      <c r="B25" t="s">
         <v>215</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -3709,11 +3808,11 @@
         <v>217</v>
       </c>
     </row>
-    <row r="26" ht="14.5">
-      <c r="A26" t="s" s="0">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>218</v>
       </c>
-      <c r="B26" t="s" s="0">
+      <c r="B26" t="s">
         <v>219</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -3723,11 +3822,11 @@
         <v>221</v>
       </c>
     </row>
-    <row r="27" ht="14.5">
-      <c r="A27" t="s" s="0">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>222</v>
       </c>
-      <c r="B27" t="s" s="0">
+      <c r="B27" t="s">
         <v>223</v>
       </c>
       <c r="C27" s="2" t="s">
@@ -3737,11 +3836,11 @@
         <v>225</v>
       </c>
     </row>
-    <row r="28" ht="14.5">
-      <c r="A28" t="s" s="0">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>226</v>
       </c>
-      <c r="B28" t="s" s="0">
+      <c r="B28" t="s">
         <v>227</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -3751,11 +3850,11 @@
         <v>229</v>
       </c>
     </row>
-    <row r="29" ht="14.5">
-      <c r="A29" t="s" s="0">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>230</v>
       </c>
-      <c r="B29" t="s" s="0">
+      <c r="B29" t="s">
         <v>231</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -3765,11 +3864,11 @@
         <v>233</v>
       </c>
     </row>
-    <row r="30" ht="14.5">
-      <c r="A30" t="s" s="0">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>234</v>
       </c>
-      <c r="B30" t="s" s="0">
+      <c r="B30" t="s">
         <v>235</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -3779,11 +3878,11 @@
         <v>237</v>
       </c>
     </row>
-    <row r="31" ht="14.5">
-      <c r="A31" t="s" s="0">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>238</v>
       </c>
-      <c r="B31" t="s" s="0">
+      <c r="B31" t="s">
         <v>239</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -3793,11 +3892,11 @@
         <v>241</v>
       </c>
     </row>
-    <row r="32" ht="14.5">
-      <c r="A32" t="s" s="0">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>242</v>
       </c>
-      <c r="B32" t="s" s="0">
+      <c r="B32" t="s">
         <v>243</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -3807,11 +3906,11 @@
         <v>245</v>
       </c>
     </row>
-    <row r="33" ht="14.5">
-      <c r="A33" t="s" s="0">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>246</v>
       </c>
-      <c r="B33" t="s" s="0">
+      <c r="B33" t="s">
         <v>247</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -3821,11 +3920,11 @@
         <v>249</v>
       </c>
     </row>
-    <row r="34" ht="14.5">
-      <c r="A34" t="s" s="0">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>250</v>
       </c>
-      <c r="B34" t="s" s="0">
+      <c r="B34" t="s">
         <v>251</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -3835,11 +3934,11 @@
         <v>253</v>
       </c>
     </row>
-    <row r="35" ht="14.5">
-      <c r="A35" t="s" s="0">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>254</v>
       </c>
-      <c r="B35" t="s" s="0">
+      <c r="B35" t="s">
         <v>255</v>
       </c>
       <c r="C35" s="2" t="s">
@@ -3849,11 +3948,11 @@
         <v>257</v>
       </c>
     </row>
-    <row r="36" ht="14.5">
-      <c r="A36" t="s" s="0">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>258</v>
       </c>
-      <c r="B36" t="s" s="0">
+      <c r="B36" t="s">
         <v>259</v>
       </c>
       <c r="C36" s="2" t="s">
@@ -3863,11 +3962,11 @@
         <v>261</v>
       </c>
     </row>
-    <row r="37" ht="14.5">
-      <c r="A37" t="s" s="0">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>262</v>
       </c>
-      <c r="B37" t="s" s="0">
+      <c r="B37" t="s">
         <v>263</v>
       </c>
       <c r="C37" s="2" t="s">
@@ -3877,11 +3976,11 @@
         <v>265</v>
       </c>
     </row>
-    <row r="38" ht="14.5">
-      <c r="A38" t="s" s="0">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>266</v>
       </c>
-      <c r="B38" t="s" s="0">
+      <c r="B38" t="s">
         <v>267</v>
       </c>
       <c r="C38" s="2" t="s">
@@ -3891,11 +3990,11 @@
         <v>269</v>
       </c>
     </row>
-    <row r="39" ht="14.5">
-      <c r="A39" t="s" s="0">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>270</v>
       </c>
-      <c r="B39" t="s" s="0">
+      <c r="B39" t="s">
         <v>271</v>
       </c>
       <c r="C39" s="2" t="s">
@@ -3905,11 +4004,11 @@
         <v>273</v>
       </c>
     </row>
-    <row r="40" ht="14.5">
-      <c r="A40" t="s" s="0">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>274</v>
       </c>
-      <c r="B40" t="s" s="0">
+      <c r="B40" t="s">
         <v>275</v>
       </c>
       <c r="C40" s="2" t="s">
@@ -3919,11 +4018,11 @@
         <v>277</v>
       </c>
     </row>
-    <row r="41" ht="14.5">
-      <c r="A41" t="s" s="0">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>278</v>
       </c>
-      <c r="B41" t="s" s="0">
+      <c r="B41" t="s">
         <v>279</v>
       </c>
       <c r="C41" s="2" t="s">
@@ -3933,11 +4032,11 @@
         <v>281</v>
       </c>
     </row>
-    <row r="42" ht="14.5">
-      <c r="A42" t="s" s="0">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>282</v>
       </c>
-      <c r="B42" t="s" s="0">
+      <c r="B42" t="s">
         <v>283</v>
       </c>
       <c r="C42" s="13" t="s">
@@ -3947,11 +4046,11 @@
         <v>285</v>
       </c>
     </row>
-    <row r="43" ht="14.5">
-      <c r="A43" t="s" s="0">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>286</v>
       </c>
-      <c r="B43" t="s" s="0">
+      <c r="B43" t="s">
         <v>287</v>
       </c>
       <c r="C43" s="24" t="s">
@@ -3961,11 +4060,11 @@
         <v>289</v>
       </c>
     </row>
-    <row r="44" ht="14.5">
-      <c r="A44" t="s" s="0">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>290</v>
       </c>
-      <c r="B44" t="s" s="0">
+      <c r="B44" t="s">
         <v>291</v>
       </c>
       <c r="C44" s="6" t="s">
@@ -3975,11 +4074,11 @@
         <v>293</v>
       </c>
     </row>
-    <row r="45" ht="14.5">
-      <c r="A45" t="s" s="0">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>294</v>
       </c>
-      <c r="B45" t="s" s="0">
+      <c r="B45" t="s">
         <v>295</v>
       </c>
       <c r="C45" s="6" t="s">
@@ -3989,11 +4088,11 @@
         <v>297</v>
       </c>
     </row>
-    <row r="46" ht="14.5">
-      <c r="A46" t="s" s="0">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>298</v>
       </c>
-      <c r="B46" t="s" s="0">
+      <c r="B46" t="s">
         <v>299</v>
       </c>
       <c r="C46" s="6" t="s">
@@ -4003,11 +4102,11 @@
         <v>301</v>
       </c>
     </row>
-    <row r="47" ht="14.5">
-      <c r="A47" t="s" s="0">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>302</v>
       </c>
-      <c r="B47" t="s" s="0">
+      <c r="B47" t="s">
         <v>303</v>
       </c>
       <c r="C47" s="6" t="s">
@@ -4017,11 +4116,11 @@
         <v>305</v>
       </c>
     </row>
-    <row r="48" ht="14.5">
-      <c r="A48" t="s" s="0">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>306</v>
       </c>
-      <c r="B48" t="s" s="0">
+      <c r="B48" t="s">
         <v>307</v>
       </c>
       <c r="C48" s="6" t="s">
@@ -4031,11 +4130,11 @@
         <v>309</v>
       </c>
     </row>
-    <row r="49" ht="14.5">
-      <c r="A49" t="s" s="0">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>310</v>
       </c>
-      <c r="B49" t="s" s="0">
+      <c r="B49" t="s">
         <v>311</v>
       </c>
       <c r="C49" s="6" t="s">
@@ -4045,11 +4144,11 @@
         <v>313</v>
       </c>
     </row>
-    <row r="50" ht="14.5">
-      <c r="A50" t="s" s="0">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>314</v>
       </c>
-      <c r="B50" t="s" s="0">
+      <c r="B50" t="s">
         <v>315</v>
       </c>
       <c r="C50" s="6" t="s">
@@ -4059,11 +4158,11 @@
         <v>317</v>
       </c>
     </row>
-    <row r="51" ht="14.5">
-      <c r="A51" t="s" s="0">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>318</v>
       </c>
-      <c r="B51" t="s" s="0">
+      <c r="B51" t="s">
         <v>319</v>
       </c>
       <c r="C51" s="6" t="s">
@@ -4073,11 +4172,11 @@
         <v>321</v>
       </c>
     </row>
-    <row r="52" ht="14.5">
-      <c r="A52" t="s" s="0">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>322</v>
       </c>
-      <c r="B52" t="s" s="0">
+      <c r="B52" t="s">
         <v>323</v>
       </c>
       <c r="C52" s="6" t="s">
@@ -4087,11 +4186,11 @@
         <v>325</v>
       </c>
     </row>
-    <row r="53" ht="14.5">
-      <c r="A53" t="s" s="0">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>326</v>
       </c>
-      <c r="B53" t="s" s="0">
+      <c r="B53" t="s">
         <v>327</v>
       </c>
       <c r="C53" s="6" t="s">
@@ -4101,11 +4200,11 @@
         <v>329</v>
       </c>
     </row>
-    <row r="54" ht="14.5">
-      <c r="A54" t="s" s="0">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
         <v>330</v>
       </c>
-      <c r="B54" t="s" s="0">
+      <c r="B54" t="s">
         <v>331</v>
       </c>
       <c r="C54" s="6" t="s">
@@ -4115,11 +4214,11 @@
         <v>333</v>
       </c>
     </row>
-    <row r="55" ht="14.5">
-      <c r="A55" t="s" s="0">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>334</v>
       </c>
-      <c r="B55" t="s" s="0">
+      <c r="B55" t="s">
         <v>335</v>
       </c>
       <c r="C55" s="6" t="s">
@@ -4129,11 +4228,11 @@
         <v>337</v>
       </c>
     </row>
-    <row r="56" ht="14.5">
-      <c r="A56" t="s" s="0">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>338</v>
       </c>
-      <c r="B56" t="s" s="0">
+      <c r="B56" t="s">
         <v>339</v>
       </c>
       <c r="C56" s="6" t="s">
@@ -4143,11 +4242,11 @@
         <v>341</v>
       </c>
     </row>
-    <row r="57" ht="14.5">
-      <c r="A57" t="s" s="0">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>342</v>
       </c>
-      <c r="B57" t="s" s="0">
+      <c r="B57" t="s">
         <v>343</v>
       </c>
       <c r="C57" s="6" t="s">
@@ -4157,11 +4256,11 @@
         <v>345</v>
       </c>
     </row>
-    <row r="58" ht="14.5">
-      <c r="A58" t="s" s="0">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>346</v>
       </c>
-      <c r="B58" t="s" s="0">
+      <c r="B58" t="s">
         <v>347</v>
       </c>
       <c r="C58" s="6" t="s">
@@ -4171,11 +4270,11 @@
         <v>349</v>
       </c>
     </row>
-    <row r="59" ht="14.5">
-      <c r="A59" t="s" s="0">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>350</v>
       </c>
-      <c r="B59" t="s" s="0">
+      <c r="B59" t="s">
         <v>351</v>
       </c>
       <c r="C59" s="6" t="s">
@@ -4185,11 +4284,11 @@
         <v>353</v>
       </c>
     </row>
-    <row r="60" ht="14.5">
-      <c r="A60" t="s" s="0">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>354</v>
       </c>
-      <c r="B60" t="s" s="0">
+      <c r="B60" t="s">
         <v>355</v>
       </c>
       <c r="C60" s="6" t="s">
@@ -4199,11 +4298,11 @@
         <v>357</v>
       </c>
     </row>
-    <row r="61" ht="14.5">
-      <c r="A61" t="s" s="0">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>358</v>
       </c>
-      <c r="B61" t="s" s="0">
+      <c r="B61" t="s">
         <v>359</v>
       </c>
       <c r="C61" s="6" t="s">
@@ -4213,11 +4312,11 @@
         <v>361</v>
       </c>
     </row>
-    <row r="62" ht="14.5">
-      <c r="A62" t="s" s="0">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>362</v>
       </c>
-      <c r="B62" t="s" s="0">
+      <c r="B62" t="s">
         <v>363</v>
       </c>
       <c r="C62" s="6" t="s">
@@ -4227,11 +4326,11 @@
         <v>365</v>
       </c>
     </row>
-    <row r="63" ht="14.5">
-      <c r="A63" t="s" s="0">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>366</v>
       </c>
-      <c r="B63" t="s" s="0">
+      <c r="B63" t="s">
         <v>367</v>
       </c>
       <c r="C63" s="6" t="s">
@@ -4241,11 +4340,11 @@
         <v>369</v>
       </c>
     </row>
-    <row r="64" ht="14.5">
-      <c r="A64" t="s" s="0">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>370</v>
       </c>
-      <c r="B64" t="s" s="0">
+      <c r="B64" t="s">
         <v>371</v>
       </c>
       <c r="C64" s="6" t="s">
@@ -4255,11 +4354,11 @@
         <v>373</v>
       </c>
     </row>
-    <row r="65" ht="14.5">
-      <c r="A65" t="s" s="0">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>374</v>
       </c>
-      <c r="B65" t="s" s="0">
+      <c r="B65" t="s">
         <v>375</v>
       </c>
       <c r="C65" s="6" t="s">
@@ -4269,11 +4368,11 @@
         <v>377</v>
       </c>
     </row>
-    <row r="66" ht="14.5">
-      <c r="A66" t="s" s="0">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>378</v>
       </c>
-      <c r="B66" t="s" s="0">
+      <c r="B66" t="s">
         <v>379</v>
       </c>
       <c r="C66" s="6" t="s">
@@ -4283,11 +4382,11 @@
         <v>381</v>
       </c>
     </row>
-    <row r="67" ht="14.5">
-      <c r="A67" t="s" s="0">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>382</v>
       </c>
-      <c r="B67" t="s" s="0">
+      <c r="B67" t="s">
         <v>383</v>
       </c>
       <c r="C67" s="6" t="s">
@@ -4297,11 +4396,11 @@
         <v>385</v>
       </c>
     </row>
-    <row r="68" ht="14.5">
-      <c r="A68" t="s" s="0">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>386</v>
       </c>
-      <c r="B68" t="s" s="0">
+      <c r="B68" t="s">
         <v>387</v>
       </c>
       <c r="C68" s="6" t="s">
@@ -4311,11 +4410,11 @@
         <v>389</v>
       </c>
     </row>
-    <row r="69" ht="14.5">
-      <c r="A69" t="s" s="0">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>390</v>
       </c>
-      <c r="B69" t="s" s="0">
+      <c r="B69" t="s">
         <v>391</v>
       </c>
       <c r="C69" s="6" t="s">
@@ -4325,11 +4424,11 @@
         <v>393</v>
       </c>
     </row>
-    <row r="70" ht="14.5">
-      <c r="A70" t="s" s="0">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>394</v>
       </c>
-      <c r="B70" t="s" s="0">
+      <c r="B70" t="s">
         <v>395</v>
       </c>
       <c r="C70" s="6" t="s">
@@ -4339,11 +4438,11 @@
         <v>397</v>
       </c>
     </row>
-    <row r="71" ht="14.5">
-      <c r="A71" t="s" s="0">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>398</v>
       </c>
-      <c r="B71" t="s" s="0">
+      <c r="B71" t="s">
         <v>399</v>
       </c>
       <c r="C71" s="6" t="s">
@@ -4353,11 +4452,11 @@
         <v>401</v>
       </c>
     </row>
-    <row r="72" ht="14.5">
-      <c r="A72" t="s" s="0">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>402</v>
       </c>
-      <c r="B72" t="s" s="0">
+      <c r="B72" t="s">
         <v>403</v>
       </c>
       <c r="C72" s="6" t="s">
@@ -4367,11 +4466,11 @@
         <v>405</v>
       </c>
     </row>
-    <row r="73" ht="14.5">
-      <c r="A73" t="s" s="0">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>406</v>
       </c>
-      <c r="B73" t="s" s="0">
+      <c r="B73" t="s">
         <v>407</v>
       </c>
       <c r="C73" s="6" t="s">
@@ -4381,11 +4480,11 @@
         <v>409</v>
       </c>
     </row>
-    <row r="74" ht="14.5">
-      <c r="A74" t="s" s="0">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>410</v>
       </c>
-      <c r="B74" t="s" s="0">
+      <c r="B74" t="s">
         <v>411</v>
       </c>
       <c r="C74" s="6" t="s">
@@ -4395,11 +4494,11 @@
         <v>413</v>
       </c>
     </row>
-    <row r="75" ht="14.5">
-      <c r="A75" t="s" s="0">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>414</v>
       </c>
-      <c r="B75" t="s" s="0">
+      <c r="B75" t="s">
         <v>415</v>
       </c>
       <c r="C75" s="6" t="s">
@@ -4409,11 +4508,11 @@
         <v>417</v>
       </c>
     </row>
-    <row r="76" ht="14.5">
-      <c r="A76" t="s" s="0">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>418</v>
       </c>
-      <c r="B76" t="s" s="0">
+      <c r="B76" t="s">
         <v>419</v>
       </c>
       <c r="C76" s="6" t="s">
@@ -4423,11 +4522,11 @@
         <v>421</v>
       </c>
     </row>
-    <row r="77" ht="14.5">
-      <c r="A77" t="s" s="0">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>422</v>
       </c>
-      <c r="B77" t="s" s="0">
+      <c r="B77" t="s">
         <v>423</v>
       </c>
       <c r="C77" s="6" t="s">
@@ -4437,11 +4536,11 @@
         <v>425</v>
       </c>
     </row>
-    <row r="78" ht="14.5">
-      <c r="A78" t="s" s="0">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>426</v>
       </c>
-      <c r="B78" t="s" s="0">
+      <c r="B78" t="s">
         <v>427</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -4451,11 +4550,11 @@
         <v>429</v>
       </c>
     </row>
-    <row r="79" ht="14.5">
-      <c r="A79" t="s" s="0">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>430</v>
       </c>
-      <c r="B79" t="s" s="0">
+      <c r="B79" t="s">
         <v>431</v>
       </c>
       <c r="C79" s="6" t="s">
@@ -4465,11 +4564,11 @@
         <v>433</v>
       </c>
     </row>
-    <row r="80" ht="14.5">
-      <c r="A80" t="s" s="0">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>434</v>
       </c>
-      <c r="B80" t="s" s="0">
+      <c r="B80" t="s">
         <v>435</v>
       </c>
       <c r="C80" s="6" t="s">
@@ -4479,11 +4578,11 @@
         <v>437</v>
       </c>
     </row>
-    <row r="81" ht="14.5">
-      <c r="A81" t="s" s="0">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>438</v>
       </c>
-      <c r="B81" t="s" s="0">
+      <c r="B81" t="s">
         <v>439</v>
       </c>
       <c r="C81" s="6" t="s">
@@ -4493,11 +4592,11 @@
         <v>441</v>
       </c>
     </row>
-    <row r="82" ht="14.5">
-      <c r="A82" t="s" s="0">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>442</v>
       </c>
-      <c r="B82" t="s" s="0">
+      <c r="B82" t="s">
         <v>443</v>
       </c>
       <c r="C82" s="6" t="s">
@@ -4507,11 +4606,11 @@
         <v>445</v>
       </c>
     </row>
-    <row r="83" ht="14.5">
-      <c r="A83" t="s" s="0">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
         <v>446</v>
       </c>
-      <c r="B83" t="s" s="0">
+      <c r="B83" t="s">
         <v>447</v>
       </c>
       <c r="C83" s="6" t="s">
@@ -4521,11 +4620,11 @@
         <v>449</v>
       </c>
     </row>
-    <row r="84" ht="14.5">
-      <c r="A84" t="s" s="0">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
         <v>450</v>
       </c>
-      <c r="B84" t="s" s="0">
+      <c r="B84" t="s">
         <v>451</v>
       </c>
       <c r="C84" s="6" t="s">
@@ -4535,11 +4634,11 @@
         <v>453</v>
       </c>
     </row>
-    <row r="85" ht="14.5">
-      <c r="A85" t="s" s="0">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
         <v>454</v>
       </c>
-      <c r="B85" t="s" s="0">
+      <c r="B85" t="s">
         <v>455</v>
       </c>
       <c r="C85" s="6" t="s">
@@ -4549,11 +4648,11 @@
         <v>457</v>
       </c>
     </row>
-    <row r="86" ht="14.5">
-      <c r="A86" t="s" s="0">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
         <v>458</v>
       </c>
-      <c r="B86" t="s" s="0">
+      <c r="B86" t="s">
         <v>459</v>
       </c>
       <c r="C86" s="6" t="s">
@@ -4563,11 +4662,11 @@
         <v>461</v>
       </c>
     </row>
-    <row r="87" ht="14.5">
-      <c r="A87" t="s" s="0">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
         <v>462</v>
       </c>
-      <c r="B87" t="s" s="0">
+      <c r="B87" t="s">
         <v>463</v>
       </c>
       <c r="C87" s="6" t="s">
@@ -4577,11 +4676,11 @@
         <v>465</v>
       </c>
     </row>
-    <row r="88" ht="14.5">
-      <c r="A88" t="s" s="0">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>466</v>
       </c>
-      <c r="B88" t="s" s="0">
+      <c r="B88" t="s">
         <v>467</v>
       </c>
       <c r="C88" s="6" t="s">
@@ -4591,11 +4690,11 @@
         <v>469</v>
       </c>
     </row>
-    <row r="89" ht="14.5">
-      <c r="A89" t="s" s="0">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>470</v>
       </c>
-      <c r="B89" t="s" s="0">
+      <c r="B89" t="s">
         <v>471</v>
       </c>
       <c r="C89" s="6" t="s">
@@ -4605,11 +4704,11 @@
         <v>473</v>
       </c>
     </row>
-    <row r="90" ht="14.5">
-      <c r="A90" t="s" s="0">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>474</v>
       </c>
-      <c r="B90" t="s" s="0">
+      <c r="B90" t="s">
         <v>475</v>
       </c>
       <c r="C90" s="6" t="s">
@@ -4619,11 +4718,11 @@
         <v>477</v>
       </c>
     </row>
-    <row r="91" ht="14.5">
-      <c r="A91" t="s" s="0">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
         <v>478</v>
       </c>
-      <c r="B91" t="s" s="0">
+      <c r="B91" t="s">
         <v>479</v>
       </c>
       <c r="C91" s="6" t="s">
@@ -4633,11 +4732,11 @@
         <v>481</v>
       </c>
     </row>
-    <row r="92" ht="14.5">
-      <c r="A92" t="s" s="0">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>482</v>
       </c>
-      <c r="B92" t="s" s="0">
+      <c r="B92" t="s">
         <v>483</v>
       </c>
       <c r="C92" s="6" t="s">
@@ -4647,11 +4746,11 @@
         <v>485</v>
       </c>
     </row>
-    <row r="93" ht="14.5">
-      <c r="A93" t="s" s="0">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
         <v>486</v>
       </c>
-      <c r="B93" t="s" s="0">
+      <c r="B93" t="s">
         <v>487</v>
       </c>
       <c r="C93" s="6" t="s">
@@ -4661,11 +4760,11 @@
         <v>489</v>
       </c>
     </row>
-    <row r="94" ht="14.5">
-      <c r="A94" t="s" s="0">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>490</v>
       </c>
-      <c r="B94" t="s" s="0">
+      <c r="B94" t="s">
         <v>491</v>
       </c>
       <c r="C94" s="6" t="s">
@@ -4675,11 +4774,11 @@
         <v>493</v>
       </c>
     </row>
-    <row r="95" ht="14.5">
-      <c r="A95" t="s" s="0">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>494</v>
       </c>
-      <c r="B95" t="s" s="0">
+      <c r="B95" t="s">
         <v>495</v>
       </c>
       <c r="C95" s="6" t="s">
@@ -4689,11 +4788,11 @@
         <v>497</v>
       </c>
     </row>
-    <row r="96" ht="14.5">
-      <c r="A96" t="s" s="0">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
         <v>498</v>
       </c>
-      <c r="B96" t="s" s="0">
+      <c r="B96" t="s">
         <v>499</v>
       </c>
       <c r="C96" s="6" t="s">
@@ -4703,11 +4802,11 @@
         <v>501</v>
       </c>
     </row>
-    <row r="97" ht="14.5">
-      <c r="A97" t="s" s="0">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
         <v>502</v>
       </c>
-      <c r="B97" t="s" s="0">
+      <c r="B97" t="s">
         <v>503</v>
       </c>
       <c r="C97" s="6" t="s">
@@ -4717,11 +4816,11 @@
         <v>505</v>
       </c>
     </row>
-    <row r="98" ht="14.5">
-      <c r="A98" t="s" s="0">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
         <v>506</v>
       </c>
-      <c r="B98" t="s" s="0">
+      <c r="B98" t="s">
         <v>507</v>
       </c>
       <c r="C98" s="6" t="s">
@@ -4731,11 +4830,11 @@
         <v>509</v>
       </c>
     </row>
-    <row r="99" ht="14.5">
-      <c r="A99" t="s" s="0">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
         <v>510</v>
       </c>
-      <c r="B99" t="s" s="0">
+      <c r="B99" t="s">
         <v>511</v>
       </c>
       <c r="C99" s="6" t="s">
@@ -4745,11 +4844,11 @@
         <v>513</v>
       </c>
     </row>
-    <row r="100" ht="14.5">
-      <c r="A100" t="s" s="0">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
         <v>514</v>
       </c>
-      <c r="B100" t="s" s="0">
+      <c r="B100" t="s">
         <v>515</v>
       </c>
       <c r="C100" s="6" t="s">
@@ -4759,11 +4858,11 @@
         <v>517</v>
       </c>
     </row>
-    <row r="101" ht="14.5">
-      <c r="A101" t="s" s="0">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>518</v>
       </c>
-      <c r="B101" t="s" s="0">
+      <c r="B101" t="s">
         <v>519</v>
       </c>
       <c r="C101" s="6" t="s">
@@ -4773,11 +4872,11 @@
         <v>521</v>
       </c>
     </row>
-    <row r="102" ht="14.5">
-      <c r="A102" t="s" s="0">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
         <v>522</v>
       </c>
-      <c r="B102" t="s" s="0">
+      <c r="B102" t="s">
         <v>523</v>
       </c>
       <c r="C102" s="6" t="s">
@@ -4787,11 +4886,11 @@
         <v>525</v>
       </c>
     </row>
-    <row r="103" ht="14.5">
-      <c r="A103" t="s" s="0">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
         <v>526</v>
       </c>
-      <c r="B103" t="s" s="0">
+      <c r="B103" t="s">
         <v>527</v>
       </c>
       <c r="C103" s="6" t="s">
@@ -4801,11 +4900,11 @@
         <v>529</v>
       </c>
     </row>
-    <row r="104" ht="14.5">
-      <c r="A104" t="s" s="0">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
         <v>530</v>
       </c>
-      <c r="B104" t="s" s="0">
+      <c r="B104" t="s">
         <v>531</v>
       </c>
       <c r="C104" s="6" t="s">
@@ -4815,11 +4914,11 @@
         <v>533</v>
       </c>
     </row>
-    <row r="105" ht="14.5">
-      <c r="A105" t="s" s="0">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
         <v>534</v>
       </c>
-      <c r="B105" t="s" s="0">
+      <c r="B105" t="s">
         <v>535</v>
       </c>
       <c r="C105" s="6" t="s">
@@ -4829,11 +4928,11 @@
         <v>537</v>
       </c>
     </row>
-    <row r="106" ht="14.5">
-      <c r="A106" t="s" s="0">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
         <v>538</v>
       </c>
-      <c r="B106" t="s" s="0">
+      <c r="B106" t="s">
         <v>539</v>
       </c>
       <c r="C106" s="6" t="s">
@@ -4843,11 +4942,11 @@
         <v>541</v>
       </c>
     </row>
-    <row r="107" ht="14.5">
-      <c r="A107" t="s" s="0">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
         <v>542</v>
       </c>
-      <c r="B107" t="s" s="0">
+      <c r="B107" t="s">
         <v>543</v>
       </c>
       <c r="C107" s="6" t="s">
@@ -4857,11 +4956,11 @@
         <v>545</v>
       </c>
     </row>
-    <row r="108" ht="14.5">
-      <c r="A108" t="s" s="0">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
         <v>546</v>
       </c>
-      <c r="B108" t="s" s="0">
+      <c r="B108" t="s">
         <v>547</v>
       </c>
       <c r="C108" s="6" t="s">
@@ -4871,11 +4970,11 @@
         <v>549</v>
       </c>
     </row>
-    <row r="109" ht="14.5">
-      <c r="A109" t="s" s="0">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
         <v>550</v>
       </c>
-      <c r="B109" t="s" s="0">
+      <c r="B109" t="s">
         <v>551</v>
       </c>
       <c r="C109" s="6" t="s">
@@ -4885,11 +4984,11 @@
         <v>553</v>
       </c>
     </row>
-    <row r="110" ht="14.5">
-      <c r="A110" t="s" s="0">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
         <v>554</v>
       </c>
-      <c r="B110" t="s" s="0">
+      <c r="B110" t="s">
         <v>555</v>
       </c>
       <c r="C110" s="6" t="s">
@@ -4899,11 +4998,11 @@
         <v>557</v>
       </c>
     </row>
-    <row r="111" ht="14.5">
-      <c r="A111" t="s" s="0">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
         <v>558</v>
       </c>
-      <c r="B111" t="s" s="0">
+      <c r="B111" t="s">
         <v>559</v>
       </c>
       <c r="C111" s="6" t="s">
@@ -4913,11 +5012,11 @@
         <v>561</v>
       </c>
     </row>
-    <row r="112" ht="14.5">
-      <c r="A112" t="s" s="0">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
         <v>562</v>
       </c>
-      <c r="B112" t="s" s="0">
+      <c r="B112" t="s">
         <v>563</v>
       </c>
       <c r="C112" s="6" t="s">
@@ -4927,11 +5026,11 @@
         <v>565</v>
       </c>
     </row>
-    <row r="113" ht="14.5">
-      <c r="A113" t="s" s="0">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
         <v>566</v>
       </c>
-      <c r="B113" t="s" s="0">
+      <c r="B113" t="s">
         <v>567</v>
       </c>
       <c r="C113" s="6" t="s">
@@ -4941,11 +5040,11 @@
         <v>569</v>
       </c>
     </row>
-    <row r="114" ht="14.5">
-      <c r="A114" t="s" s="0">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
         <v>570</v>
       </c>
-      <c r="B114" t="s" s="0">
+      <c r="B114" t="s">
         <v>571</v>
       </c>
       <c r="C114" s="6" t="s">
@@ -4955,11 +5054,11 @@
         <v>573</v>
       </c>
     </row>
-    <row r="115" ht="14.5">
-      <c r="A115" t="s" s="0">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
         <v>574</v>
       </c>
-      <c r="B115" t="s" s="0">
+      <c r="B115" t="s">
         <v>575</v>
       </c>
       <c r="C115" s="6" t="s">
@@ -4969,11 +5068,11 @@
         <v>577</v>
       </c>
     </row>
-    <row r="116" ht="14.5">
-      <c r="A116" t="s" s="0">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
         <v>578</v>
       </c>
-      <c r="B116" t="s" s="0">
+      <c r="B116" t="s">
         <v>579</v>
       </c>
       <c r="C116" s="6" t="s">
@@ -4983,11 +5082,11 @@
         <v>581</v>
       </c>
     </row>
-    <row r="117" ht="14.5">
-      <c r="A117" t="s" s="0">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
         <v>582</v>
       </c>
-      <c r="B117" t="s" s="0">
+      <c r="B117" t="s">
         <v>583</v>
       </c>
       <c r="C117" s="6" t="s">
@@ -4997,11 +5096,11 @@
         <v>585</v>
       </c>
     </row>
-    <row r="118" ht="14.5">
-      <c r="A118" t="s" s="0">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
         <v>586</v>
       </c>
-      <c r="B118" t="s" s="0">
+      <c r="B118" t="s">
         <v>587</v>
       </c>
       <c r="C118" s="6" t="s">
@@ -5011,11 +5110,11 @@
         <v>589</v>
       </c>
     </row>
-    <row r="119" ht="14.5">
-      <c r="A119" t="s" s="0">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
         <v>590</v>
       </c>
-      <c r="B119" t="s" s="0">
+      <c r="B119" t="s">
         <v>591</v>
       </c>
       <c r="C119" s="6" t="s">
@@ -5025,11 +5124,11 @@
         <v>593</v>
       </c>
     </row>
-    <row r="120" ht="14.5">
-      <c r="A120" t="s" s="0">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
         <v>594</v>
       </c>
-      <c r="B120" t="s" s="0">
+      <c r="B120" t="s">
         <v>595</v>
       </c>
       <c r="C120" s="6" t="s">
@@ -5039,11 +5138,11 @@
         <v>597</v>
       </c>
     </row>
-    <row r="121" ht="14.5">
-      <c r="A121" t="s" s="0">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
         <v>598</v>
       </c>
-      <c r="B121" t="s" s="0">
+      <c r="B121" t="s">
         <v>599</v>
       </c>
       <c r="C121" s="6" t="s">
@@ -5053,11 +5152,11 @@
         <v>601</v>
       </c>
     </row>
-    <row r="122" ht="14.5">
-      <c r="A122" t="s" s="0">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
         <v>602</v>
       </c>
-      <c r="B122" t="s" s="0">
+      <c r="B122" t="s">
         <v>603</v>
       </c>
       <c r="C122" s="6" t="s">
@@ -5067,11 +5166,11 @@
         <v>605</v>
       </c>
     </row>
-    <row r="123" ht="14.5">
-      <c r="A123" t="s" s="0">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
         <v>606</v>
       </c>
-      <c r="B123" t="s" s="0">
+      <c r="B123" t="s">
         <v>607</v>
       </c>
       <c r="C123" s="6" t="s">
@@ -5081,11 +5180,11 @@
         <v>609</v>
       </c>
     </row>
-    <row r="124" ht="14.5">
-      <c r="A124" t="s" s="0">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
         <v>610</v>
       </c>
-      <c r="B124" t="s" s="0">
+      <c r="B124" t="s">
         <v>611</v>
       </c>
       <c r="C124" s="6" t="s">
@@ -5095,11 +5194,11 @@
         <v>613</v>
       </c>
     </row>
-    <row r="125" ht="14.5">
-      <c r="A125" t="s" s="0">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
         <v>614</v>
       </c>
-      <c r="B125" t="s" s="0">
+      <c r="B125" t="s">
         <v>615</v>
       </c>
       <c r="C125" s="6" t="s">
@@ -5109,11 +5208,11 @@
         <v>617</v>
       </c>
     </row>
-    <row r="126" ht="14.5">
-      <c r="A126" t="s" s="0">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
         <v>618</v>
       </c>
-      <c r="B126" t="s" s="0">
+      <c r="B126" t="s">
         <v>619</v>
       </c>
       <c r="C126" s="6" t="s">
@@ -5123,11 +5222,11 @@
         <v>621</v>
       </c>
     </row>
-    <row r="127" ht="14.5">
-      <c r="A127" t="s" s="0">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
         <v>622</v>
       </c>
-      <c r="B127" t="s" s="0">
+      <c r="B127" t="s">
         <v>623</v>
       </c>
       <c r="C127" s="6" t="s">
@@ -5137,11 +5236,11 @@
         <v>625</v>
       </c>
     </row>
-    <row r="128" ht="14.5">
-      <c r="A128" t="s" s="0">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
         <v>626</v>
       </c>
-      <c r="B128" t="s" s="0">
+      <c r="B128" t="s">
         <v>627</v>
       </c>
       <c r="C128" s="6" t="s">
@@ -5151,11 +5250,11 @@
         <v>629</v>
       </c>
     </row>
-    <row r="129" ht="14.5">
-      <c r="A129" t="s" s="0">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
         <v>630</v>
       </c>
-      <c r="B129" t="s" s="0">
+      <c r="B129" t="s">
         <v>631</v>
       </c>
       <c r="C129" s="6" t="s">
@@ -5165,11 +5264,11 @@
         <v>633</v>
       </c>
     </row>
-    <row r="130" ht="14.5">
-      <c r="A130" t="s" s="0">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
         <v>634</v>
       </c>
-      <c r="B130" t="s" s="0">
+      <c r="B130" t="s">
         <v>635</v>
       </c>
       <c r="C130" s="6" t="s">
@@ -5179,11 +5278,11 @@
         <v>637</v>
       </c>
     </row>
-    <row r="131" ht="14.5">
-      <c r="A131" t="s" s="0">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
         <v>638</v>
       </c>
-      <c r="B131" t="s" s="0">
+      <c r="B131" t="s">
         <v>639</v>
       </c>
       <c r="C131" s="6" t="s">
@@ -5193,11 +5292,11 @@
         <v>641</v>
       </c>
     </row>
-    <row r="132" ht="14.5">
-      <c r="A132" t="s" s="0">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
         <v>642</v>
       </c>
-      <c r="B132" t="s" s="0">
+      <c r="B132" t="s">
         <v>643</v>
       </c>
       <c r="C132" s="6" t="s">
@@ -5207,11 +5306,11 @@
         <v>645</v>
       </c>
     </row>
-    <row r="133" ht="14.5">
-      <c r="A133" t="s" s="0">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
         <v>646</v>
       </c>
-      <c r="B133" t="s" s="0">
+      <c r="B133" t="s">
         <v>647</v>
       </c>
       <c r="C133" s="6" t="s">
@@ -5221,11 +5320,11 @@
         <v>649</v>
       </c>
     </row>
-    <row r="134" ht="14.5">
-      <c r="A134" t="s" s="0">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
         <v>650</v>
       </c>
-      <c r="B134" t="s" s="0">
+      <c r="B134" t="s">
         <v>651</v>
       </c>
       <c r="C134" s="6" t="s">
@@ -5235,11 +5334,11 @@
         <v>653</v>
       </c>
     </row>
-    <row r="135" ht="14.5">
-      <c r="A135" t="s" s="0">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
         <v>654</v>
       </c>
-      <c r="B135" t="s" s="0">
+      <c r="B135" t="s">
         <v>655</v>
       </c>
       <c r="C135" s="6" t="s">
@@ -5249,11 +5348,11 @@
         <v>657</v>
       </c>
     </row>
-    <row r="136" ht="14.5">
-      <c r="A136" t="s" s="0">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
         <v>658</v>
       </c>
-      <c r="B136" t="s" s="0">
+      <c r="B136" t="s">
         <v>659</v>
       </c>
       <c r="C136" s="6" t="s">
@@ -5263,11 +5362,11 @@
         <v>661</v>
       </c>
     </row>
-    <row r="137" ht="14.5">
-      <c r="A137" t="s" s="0">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
         <v>662</v>
       </c>
-      <c r="B137" t="s" s="0">
+      <c r="B137" t="s">
         <v>663</v>
       </c>
       <c r="C137" s="6" t="s">
@@ -5277,11 +5376,11 @@
         <v>665</v>
       </c>
     </row>
-    <row r="138" ht="14.5">
-      <c r="A138" t="s" s="0">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
         <v>666</v>
       </c>
-      <c r="B138" t="s" s="0">
+      <c r="B138" t="s">
         <v>667</v>
       </c>
       <c r="C138" s="6" t="s">
@@ -5291,11 +5390,11 @@
         <v>669</v>
       </c>
     </row>
-    <row r="139" ht="14.5">
-      <c r="A139" t="s" s="0">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
         <v>670</v>
       </c>
-      <c r="B139" t="s" s="0">
+      <c r="B139" t="s">
         <v>671</v>
       </c>
       <c r="C139" s="6" t="s">
@@ -5305,11 +5404,11 @@
         <v>673</v>
       </c>
     </row>
-    <row r="140" ht="14.5">
-      <c r="A140" t="s" s="0">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
         <v>674</v>
       </c>
-      <c r="B140" t="s" s="0">
+      <c r="B140" t="s">
         <v>675</v>
       </c>
       <c r="C140" s="6" t="s">
@@ -5319,11 +5418,11 @@
         <v>677</v>
       </c>
     </row>
-    <row r="141" ht="14.5">
-      <c r="A141" t="s" s="0">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
         <v>678</v>
       </c>
-      <c r="B141" t="s" s="0">
+      <c r="B141" t="s">
         <v>679</v>
       </c>
       <c r="C141" s="6" t="s">
@@ -5333,11 +5432,11 @@
         <v>681</v>
       </c>
     </row>
-    <row r="142" ht="14.5">
-      <c r="A142" t="s" s="0">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
         <v>682</v>
       </c>
-      <c r="B142" t="s" s="0">
+      <c r="B142" t="s">
         <v>683</v>
       </c>
       <c r="C142" s="6" t="s">
@@ -5347,11 +5446,11 @@
         <v>685</v>
       </c>
     </row>
-    <row r="143" ht="14.5">
-      <c r="A143" t="s" s="0">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
         <v>686</v>
       </c>
-      <c r="B143" t="s" s="0">
+      <c r="B143" t="s">
         <v>687</v>
       </c>
       <c r="C143" s="6" t="s">
@@ -5361,11 +5460,11 @@
         <v>689</v>
       </c>
     </row>
-    <row r="144" ht="14.5">
-      <c r="A144" t="s" s="0">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
         <v>690</v>
       </c>
-      <c r="B144" t="s" s="0">
+      <c r="B144" t="s">
         <v>691</v>
       </c>
       <c r="C144" s="6" t="s">
@@ -5375,11 +5474,11 @@
         <v>693</v>
       </c>
     </row>
-    <row r="145" ht="14.5">
-      <c r="A145" t="s" s="0">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
         <v>694</v>
       </c>
-      <c r="B145" t="s" s="0">
+      <c r="B145" t="s">
         <v>695</v>
       </c>
       <c r="C145" s="6" t="s">
@@ -5389,11 +5488,11 @@
         <v>697</v>
       </c>
     </row>
-    <row r="146" ht="14.5">
-      <c r="A146" t="s" s="0">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
         <v>698</v>
       </c>
-      <c r="B146" t="s" s="0">
+      <c r="B146" t="s">
         <v>699</v>
       </c>
       <c r="C146" s="6" t="s">
@@ -5403,11 +5502,11 @@
         <v>701</v>
       </c>
     </row>
-    <row r="147" ht="14.5">
-      <c r="A147" t="s" s="0">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
         <v>702</v>
       </c>
-      <c r="B147" t="s" s="0">
+      <c r="B147" t="s">
         <v>703</v>
       </c>
       <c r="C147" s="6" t="s">
@@ -5417,11 +5516,11 @@
         <v>705</v>
       </c>
     </row>
-    <row r="148" ht="14.5">
-      <c r="A148" t="s" s="0">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
         <v>706</v>
       </c>
-      <c r="B148" t="s" s="0">
+      <c r="B148" t="s">
         <v>707</v>
       </c>
       <c r="C148" s="6" t="s">
@@ -5431,11 +5530,11 @@
         <v>709</v>
       </c>
     </row>
-    <row r="149" ht="14.5">
-      <c r="A149" t="s" s="0">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
         <v>710</v>
       </c>
-      <c r="B149" t="s" s="0">
+      <c r="B149" t="s">
         <v>711</v>
       </c>
       <c r="C149" s="6" t="s">
@@ -5445,11 +5544,11 @@
         <v>713</v>
       </c>
     </row>
-    <row r="150" ht="14.5">
-      <c r="A150" t="s" s="0">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
         <v>714</v>
       </c>
-      <c r="B150" t="s" s="0">
+      <c r="B150" t="s">
         <v>715</v>
       </c>
       <c r="C150" s="6" t="s">
@@ -5459,11 +5558,11 @@
         <v>717</v>
       </c>
     </row>
-    <row r="151" ht="14.5">
-      <c r="A151" t="s" s="0">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
         <v>718</v>
       </c>
-      <c r="B151" t="s" s="0">
+      <c r="B151" t="s">
         <v>719</v>
       </c>
       <c r="C151" s="6" t="s">
@@ -5473,11 +5572,11 @@
         <v>721</v>
       </c>
     </row>
-    <row r="152" ht="14.5">
-      <c r="A152" t="s" s="0">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
         <v>722</v>
       </c>
-      <c r="B152" t="s" s="0">
+      <c r="B152" t="s">
         <v>723</v>
       </c>
       <c r="C152" s="6" t="s">
@@ -5487,8 +5586,8 @@
         <v>725</v>
       </c>
     </row>
-    <row r="153" ht="14.5">
-      <c r="B153" t="s" s="0">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B153" t="s">
         <v>726</v>
       </c>
       <c r="C153" s="6" t="s">
@@ -5498,8 +5597,8 @@
         <v>728</v>
       </c>
     </row>
-    <row r="154" ht="14.5">
-      <c r="B154" t="s" s="0">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B154" t="s">
         <v>729</v>
       </c>
       <c r="C154" s="6" t="s">
@@ -5509,8 +5608,8 @@
         <v>731</v>
       </c>
     </row>
-    <row r="155" ht="14.5">
-      <c r="B155" t="s" s="0">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B155" t="s">
         <v>732</v>
       </c>
       <c r="C155" s="6" t="s">
@@ -5520,8 +5619,8 @@
         <v>734</v>
       </c>
     </row>
-    <row r="156" ht="14.5">
-      <c r="B156" t="s" s="0">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B156" t="s">
         <v>735</v>
       </c>
       <c r="C156" s="6" t="s">
@@ -5531,8 +5630,8 @@
         <v>737</v>
       </c>
     </row>
-    <row r="157" ht="14.5">
-      <c r="B157" t="s" s="0">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B157" t="s">
         <v>738</v>
       </c>
       <c r="C157" s="6" t="s">
@@ -5542,8 +5641,8 @@
         <v>740</v>
       </c>
     </row>
-    <row r="158" ht="14.5">
-      <c r="B158" t="s" s="0">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B158" t="s">
         <v>741</v>
       </c>
       <c r="C158" s="6" t="s">
@@ -5553,7 +5652,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="159" ht="14.5">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C159" s="6" t="s">
         <v>744</v>
       </c>
@@ -5561,7 +5660,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="160" ht="14.5">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C160" s="6" t="s">
         <v>746</v>
       </c>
@@ -5569,7 +5668,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="161" ht="14.5">
+    <row r="161" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C161" s="6" t="s">
         <v>748</v>
       </c>
@@ -5577,7 +5676,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="162" ht="14.5">
+    <row r="162" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C162" s="6" t="s">
         <v>750</v>
       </c>
@@ -5585,7 +5684,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="163" ht="14.5">
+    <row r="163" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C163" s="6" t="s">
         <v>752</v>
       </c>
@@ -5593,7 +5692,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="164" ht="14.5">
+    <row r="164" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C164" s="6" t="s">
         <v>754</v>
       </c>
@@ -5601,7 +5700,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="165" ht="14.5">
+    <row r="165" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C165" s="6" t="s">
         <v>756</v>
       </c>
@@ -5609,7 +5708,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="166" ht="14.5">
+    <row r="166" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C166" s="6" t="s">
         <v>758</v>
       </c>
@@ -5617,7 +5716,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="167" ht="14.5">
+    <row r="167" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C167" s="6" t="s">
         <v>760</v>
       </c>
@@ -5625,7 +5724,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="168" ht="14.5">
+    <row r="168" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C168" s="6" t="s">
         <v>762</v>
       </c>
@@ -5633,7 +5732,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="169" ht="14.5">
+    <row r="169" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C169" s="6" t="s">
         <v>764</v>
       </c>
@@ -5641,7 +5740,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="170" ht="14.5">
+    <row r="170" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C170" s="6" t="s">
         <v>766</v>
       </c>
@@ -5649,162 +5748,163 @@
         <v>767</v>
       </c>
     </row>
-    <row r="171" ht="14.5">
+    <row r="171" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D171" s="5" t="s">
         <v>768</v>
       </c>
     </row>
-    <row r="172" ht="14.5">
+    <row r="172" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D172" s="5" t="s">
         <v>769</v>
       </c>
     </row>
-    <row r="173" ht="14.5">
+    <row r="173" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D173" s="5" t="s">
         <v>770</v>
       </c>
     </row>
-    <row r="174" ht="14.5">
+    <row r="174" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D174" s="5" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="175" ht="14.5">
+    <row r="175" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D175" s="5" t="s">
         <v>772</v>
       </c>
     </row>
-    <row r="176" ht="14.5">
+    <row r="176" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D176" s="5" t="s">
         <v>773</v>
       </c>
     </row>
-    <row r="177" ht="14.5">
+    <row r="177" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D177" s="5" t="s">
         <v>774</v>
       </c>
     </row>
-    <row r="178" ht="14.5">
+    <row r="178" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D178" s="5" t="s">
         <v>775</v>
       </c>
     </row>
-    <row r="179" ht="14.5">
+    <row r="179" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D179" s="5" t="s">
         <v>776</v>
       </c>
     </row>
-    <row r="180" ht="14.5">
+    <row r="180" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D180" s="5" t="s">
         <v>777</v>
       </c>
     </row>
-    <row r="181" ht="14.5">
+    <row r="181" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D181" s="5" t="s">
         <v>778</v>
       </c>
     </row>
-    <row r="182" ht="14.5">
+    <row r="182" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D182" s="5" t="s">
         <v>779</v>
       </c>
     </row>
-    <row r="183" ht="14.5">
+    <row r="183" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D183" s="5" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="184" ht="14.5">
+    <row r="184" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D184" s="5" t="s">
         <v>781</v>
       </c>
     </row>
-    <row r="185" ht="14.5">
+    <row r="185" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D185" s="5" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="186" ht="14.5">
+    <row r="186" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D186" s="5" t="s">
         <v>783</v>
       </c>
     </row>
-    <row r="187" ht="14.5">
+    <row r="187" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D187" s="5" t="s">
         <v>784</v>
       </c>
     </row>
-    <row r="188" ht="14.5">
+    <row r="188" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D188" s="5" t="s">
         <v>785</v>
       </c>
     </row>
-    <row r="189" ht="14.5">
+    <row r="189" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D189" s="5" t="s">
         <v>786</v>
       </c>
     </row>
-    <row r="190" ht="14.5">
+    <row r="190" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D190" s="5" t="s">
         <v>787</v>
       </c>
     </row>
-    <row r="191" ht="14.5">
+    <row r="191" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D191" s="5" t="s">
         <v>788</v>
       </c>
     </row>
-    <row r="192" ht="14.5">
+    <row r="192" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D192" s="5" t="s">
         <v>789</v>
       </c>
     </row>
-    <row r="193" ht="14.5">
+    <row r="193" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D193" s="5" t="s">
         <v>790</v>
       </c>
     </row>
-    <row r="194" ht="14.5">
+    <row r="194" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D194" s="5" t="s">
         <v>791</v>
       </c>
     </row>
-    <row r="195" ht="14.5">
+    <row r="195" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D195" s="5" t="s">
         <v>792</v>
       </c>
     </row>
-    <row r="196" ht="14.5">
+    <row r="196" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D196" s="5" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="197" ht="14.5">
+    <row r="197" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D197" s="5" t="s">
         <v>794</v>
       </c>
     </row>
-    <row r="198" ht="14.5">
+    <row r="198" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D198" s="5" t="s">
         <v>795</v>
       </c>
     </row>
-    <row r="199" ht="14.5">
+    <row r="199" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D199" s="5" t="s">
         <v>796</v>
       </c>
     </row>
-    <row r="200" ht="14.5">
+    <row r="200" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D200" s="5" t="s">
         <v>797</v>
       </c>
     </row>
-    <row r="201" ht="14.5">
+    <row r="201" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D201" s="5" t="s">
         <v>798</v>
       </c>
     </row>
   </sheetData>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated url and sample id's back to release instance
</commit_message>
<xml_diff>
--- a/animalBiome_Automation/src/test/resources/data/samples.xlsx
+++ b/animalBiome_Automation/src/test/resources/data/samples.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14900" windowHeight="4230"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14900" windowHeight="3510"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE_ID" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="824">
   <si>
     <t>User_Dog_Gut</t>
   </si>
@@ -2131,106 +2131,364 @@
     <t>Nexra</t>
   </si>
   <si>
-    <t>CYTTFN</t>
-  </si>
-  <si>
-    <t>9XHARY</t>
-  </si>
-  <si>
-    <t>HY3RHC</t>
-  </si>
-  <si>
-    <t>HHNANV</t>
-  </si>
-  <si>
-    <t>VN4TKK</t>
-  </si>
-  <si>
-    <t>K69JHM</t>
-  </si>
-  <si>
-    <t>6HVKNY</t>
-  </si>
-  <si>
-    <t>HYMVFR</t>
-  </si>
-  <si>
-    <t>99NNH7</t>
-  </si>
-  <si>
-    <t>PCDYG7</t>
-  </si>
-  <si>
-    <t>K6MGK6</t>
-  </si>
-  <si>
-    <t>XUFXHD</t>
-  </si>
-  <si>
-    <t>DN3XAJ</t>
-  </si>
-  <si>
-    <t>XKUFJG</t>
-  </si>
-  <si>
-    <t>NEUT43</t>
-  </si>
-  <si>
-    <t>YVPGM6</t>
-  </si>
-  <si>
-    <t>TCKRHX</t>
-  </si>
-  <si>
-    <t>TUTEDX</t>
-  </si>
-  <si>
-    <t>MRRTAU</t>
-  </si>
-  <si>
-    <t>XCMFDM</t>
-  </si>
-  <si>
-    <t>GAHXKK</t>
-  </si>
-  <si>
-    <t>YMFYJY</t>
-  </si>
-  <si>
-    <t>FM3E3M</t>
-  </si>
-  <si>
-    <t>CEGDAV</t>
-  </si>
-  <si>
-    <t>KDURKV</t>
-  </si>
-  <si>
-    <t>V6HFYF</t>
-  </si>
-  <si>
-    <t>NM9RKK</t>
-  </si>
-  <si>
-    <t>4NCKNU</t>
-  </si>
-  <si>
-    <t>YVMEVH</t>
-  </si>
-  <si>
-    <t>GFRJXR</t>
-  </si>
-  <si>
-    <t>FPTAVX</t>
-  </si>
-  <si>
-    <t>VHDU3X</t>
-  </si>
-  <si>
-    <t>HC4NVT</t>
-  </si>
-  <si>
-    <t>ANAYVD</t>
+    <t>VURYN6</t>
+  </si>
+  <si>
+    <t>RXTRR4</t>
+  </si>
+  <si>
+    <t>XPDXXY</t>
+  </si>
+  <si>
+    <t>GHYPGJ</t>
+  </si>
+  <si>
+    <t>JXAU6X</t>
+  </si>
+  <si>
+    <t>NGYEPY</t>
+  </si>
+  <si>
+    <t>H7FHE7</t>
+  </si>
+  <si>
+    <t>MCVVDP</t>
+  </si>
+  <si>
+    <t>DDEVVV</t>
+  </si>
+  <si>
+    <t>UPCAP7</t>
+  </si>
+  <si>
+    <t>KXK9RR</t>
+  </si>
+  <si>
+    <t>AFCME4</t>
+  </si>
+  <si>
+    <t>K94HVP</t>
+  </si>
+  <si>
+    <t>U6XRME</t>
+  </si>
+  <si>
+    <t>VXJTDG</t>
+  </si>
+  <si>
+    <t>KGNTFK</t>
+  </si>
+  <si>
+    <t>CVDTTF</t>
+  </si>
+  <si>
+    <t>JU4NJ4</t>
+  </si>
+  <si>
+    <t>EVYEHK</t>
+  </si>
+  <si>
+    <t>TTAPAU</t>
+  </si>
+  <si>
+    <t>PJKY9D</t>
+  </si>
+  <si>
+    <t>DPA9YR</t>
+  </si>
+  <si>
+    <t>A7KDNT</t>
+  </si>
+  <si>
+    <t>RDN9HJ</t>
+  </si>
+  <si>
+    <t>K9V7FN</t>
+  </si>
+  <si>
+    <t>HYUU6X</t>
+  </si>
+  <si>
+    <t>DA7DT6</t>
+  </si>
+  <si>
+    <t>EVCHRV</t>
+  </si>
+  <si>
+    <t>PR4MJY</t>
+  </si>
+  <si>
+    <t>TGV9F3</t>
+  </si>
+  <si>
+    <t>V4UE4R</t>
+  </si>
+  <si>
+    <t>FXVUTF</t>
+  </si>
+  <si>
+    <t>F9G9CU</t>
+  </si>
+  <si>
+    <t>UR7TCD</t>
+  </si>
+  <si>
+    <t>CK7CUM</t>
+  </si>
+  <si>
+    <t>J3E4GF</t>
+  </si>
+  <si>
+    <t>XKVXVU</t>
+  </si>
+  <si>
+    <t>PA6EAP</t>
+  </si>
+  <si>
+    <t>RXHRAY</t>
+  </si>
+  <si>
+    <t>EFPA4N</t>
+  </si>
+  <si>
+    <t>V6E7KK</t>
+  </si>
+  <si>
+    <t>VGEKD4</t>
+  </si>
+  <si>
+    <t>YNT6VK</t>
+  </si>
+  <si>
+    <t>VFVPNK</t>
+  </si>
+  <si>
+    <t>MCCUU7</t>
+  </si>
+  <si>
+    <t>4JFUKV</t>
+  </si>
+  <si>
+    <t>VKRHAM</t>
+  </si>
+  <si>
+    <t>XKVFRV</t>
+  </si>
+  <si>
+    <t>YCAGAU</t>
+  </si>
+  <si>
+    <t>NUXCM9</t>
+  </si>
+  <si>
+    <t>9VCEED</t>
+  </si>
+  <si>
+    <t>PKJVHN</t>
+  </si>
+  <si>
+    <t>GGF6XE</t>
+  </si>
+  <si>
+    <t>KPHDMM</t>
+  </si>
+  <si>
+    <t>NE7A9U</t>
+  </si>
+  <si>
+    <t>VYPVA4</t>
+  </si>
+  <si>
+    <t>KNJYVN</t>
+  </si>
+  <si>
+    <t>U7PEGT</t>
+  </si>
+  <si>
+    <t>NVMPVK</t>
+  </si>
+  <si>
+    <t>97RRYU</t>
+  </si>
+  <si>
+    <t>CJTDEY</t>
+  </si>
+  <si>
+    <t>CE7TYM</t>
+  </si>
+  <si>
+    <t>VPNHJC</t>
+  </si>
+  <si>
+    <t>VEUU7D</t>
+  </si>
+  <si>
+    <t>VDVTAM</t>
+  </si>
+  <si>
+    <t>P6KHMN</t>
+  </si>
+  <si>
+    <t>4TGRER</t>
+  </si>
+  <si>
+    <t>JCXVEA</t>
+  </si>
+  <si>
+    <t>CMNYKU</t>
+  </si>
+  <si>
+    <t>GVNKMT</t>
+  </si>
+  <si>
+    <t>UPA4DH</t>
+  </si>
+  <si>
+    <t>DAPRCM</t>
+  </si>
+  <si>
+    <t>RJPTXR</t>
+  </si>
+  <si>
+    <t>YNCD7H</t>
+  </si>
+  <si>
+    <t>MFC6VE</t>
+  </si>
+  <si>
+    <t>VN9XHX</t>
+  </si>
+  <si>
+    <t>KKACAP</t>
+  </si>
+  <si>
+    <t>7DEDR6</t>
+  </si>
+  <si>
+    <t>V7TNJA</t>
+  </si>
+  <si>
+    <t>NVUF4N</t>
+  </si>
+  <si>
+    <t>AVVTVH</t>
+  </si>
+  <si>
+    <t>CC7CJV</t>
+  </si>
+  <si>
+    <t>EKHGDH</t>
+  </si>
+  <si>
+    <t>K9AMHP</t>
+  </si>
+  <si>
+    <t>VGHRPU</t>
+  </si>
+  <si>
+    <t>9P66DK</t>
+  </si>
+  <si>
+    <t>VUTC79</t>
+  </si>
+  <si>
+    <t>ARM6FD</t>
+  </si>
+  <si>
+    <t>HUCRMU</t>
+  </si>
+  <si>
+    <t>4TAFFK</t>
+  </si>
+  <si>
+    <t>MDNDDD</t>
+  </si>
+  <si>
+    <t>MNTKDD</t>
+  </si>
+  <si>
+    <t>PPFEUA</t>
+  </si>
+  <si>
+    <t>KDFPNT</t>
+  </si>
+  <si>
+    <t>YMXH9G</t>
+  </si>
+  <si>
+    <t>AJ47UF</t>
+  </si>
+  <si>
+    <t>TRTPGH</t>
+  </si>
+  <si>
+    <t>79EMRP</t>
+  </si>
+  <si>
+    <t>E4KDRJ</t>
+  </si>
+  <si>
+    <t>RMMXNH</t>
+  </si>
+  <si>
+    <t>NMKMYE</t>
+  </si>
+  <si>
+    <t>EK6RXN</t>
+  </si>
+  <si>
+    <t>UDMX4D</t>
+  </si>
+  <si>
+    <t>M6AYJU</t>
+  </si>
+  <si>
+    <t>JUEYPV</t>
+  </si>
+  <si>
+    <t>74HEHU</t>
+  </si>
+  <si>
+    <t>F7AYTG</t>
+  </si>
+  <si>
+    <t>VMCY6V</t>
+  </si>
+  <si>
+    <t>XY6PYC</t>
+  </si>
+  <si>
+    <t>UCFHET</t>
+  </si>
+  <si>
+    <t>NVR9Y4</t>
+  </si>
+  <si>
+    <t>K6HA6M</t>
+  </si>
+  <si>
+    <t>EUERGK</t>
+  </si>
+  <si>
+    <t>VATGME</t>
+  </si>
+  <si>
+    <t>DDM4E4</t>
+  </si>
+  <si>
+    <t>KA4DJE</t>
+  </si>
+  <si>
+    <t>DD9CPH</t>
+  </si>
+  <si>
+    <t>PU7UHK</t>
+  </si>
+  <si>
+    <t>H6NMDK</t>
+  </si>
+  <si>
+    <t>6UNPVJ</t>
   </si>
 </sst>
 </file>
@@ -2661,16 +2919,16 @@
         <v>704</v>
       </c>
       <c r="B2" t="s">
-        <v>710</v>
-      </c>
-      <c r="C2" t="s">
-        <v>716</v>
+        <v>724</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>744</v>
       </c>
       <c r="D2" t="s">
-        <v>722</v>
+        <v>764</v>
       </c>
       <c r="E2" t="s">
-        <v>728</v>
+        <v>784</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -2678,16 +2936,16 @@
         <v>705</v>
       </c>
       <c r="B3" t="s">
-        <v>711</v>
-      </c>
-      <c r="C3" t="s">
-        <v>717</v>
+        <v>725</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>745</v>
       </c>
       <c r="D3" t="s">
-        <v>723</v>
+        <v>765</v>
       </c>
       <c r="E3" t="s">
-        <v>729</v>
+        <v>785</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -2695,16 +2953,16 @@
         <v>706</v>
       </c>
       <c r="B4" t="s">
-        <v>712</v>
-      </c>
-      <c r="C4" t="s">
-        <v>718</v>
+        <v>726</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>746</v>
       </c>
       <c r="D4" t="s">
-        <v>724</v>
+        <v>766</v>
       </c>
       <c r="E4" t="s">
-        <v>730</v>
+        <v>786</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -2712,16 +2970,16 @@
         <v>707</v>
       </c>
       <c r="B5" t="s">
-        <v>713</v>
-      </c>
-      <c r="C5" t="s">
-        <v>719</v>
+        <v>727</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>747</v>
       </c>
       <c r="D5" t="s">
-        <v>725</v>
+        <v>767</v>
       </c>
       <c r="E5" t="s">
-        <v>731</v>
+        <v>787</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -2729,16 +2987,16 @@
         <v>708</v>
       </c>
       <c r="B6" t="s">
-        <v>714</v>
-      </c>
-      <c r="C6" t="s">
-        <v>720</v>
+        <v>728</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>748</v>
       </c>
       <c r="D6" t="s">
-        <v>726</v>
+        <v>768</v>
       </c>
       <c r="E6" t="s">
-        <v>732</v>
+        <v>788</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -2746,53 +3004,362 @@
         <v>709</v>
       </c>
       <c r="B7" t="s">
+        <v>729</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>749</v>
+      </c>
+      <c r="D7" t="s">
+        <v>769</v>
+      </c>
+      <c r="E7" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>710</v>
+      </c>
+      <c r="B8" t="s">
+        <v>730</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="D8" t="s">
+        <v>770</v>
+      </c>
+      <c r="E8" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>711</v>
+      </c>
+      <c r="B9" t="s">
+        <v>731</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="D9" t="s">
+        <v>771</v>
+      </c>
+      <c r="E9" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>712</v>
+      </c>
+      <c r="B10" t="s">
+        <v>732</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="D10" t="s">
+        <v>772</v>
+      </c>
+      <c r="E10" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>713</v>
+      </c>
+      <c r="B11" t="s">
+        <v>733</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="D11" t="s">
+        <v>773</v>
+      </c>
+      <c r="E11" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>714</v>
+      </c>
+      <c r="B12" t="s">
+        <v>734</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>754</v>
+      </c>
+      <c r="D12" t="s">
+        <v>774</v>
+      </c>
+      <c r="E12" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>715</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B13" t="s">
+        <v>735</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>755</v>
+      </c>
+      <c r="D13" t="s">
+        <v>775</v>
+      </c>
+      <c r="E13" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>716</v>
+      </c>
+      <c r="B14" t="s">
+        <v>736</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>756</v>
+      </c>
+      <c r="D14" t="s">
+        <v>776</v>
+      </c>
+      <c r="E14" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>717</v>
+      </c>
+      <c r="B15" t="s">
+        <v>737</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="D15" t="s">
+        <v>777</v>
+      </c>
+      <c r="E15" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>718</v>
+      </c>
+      <c r="B16" t="s">
+        <v>738</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>758</v>
+      </c>
+      <c r="D16" t="s">
+        <v>778</v>
+      </c>
+      <c r="E16" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>719</v>
+      </c>
+      <c r="B17" t="s">
+        <v>739</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="D17" t="s">
+        <v>779</v>
+      </c>
+      <c r="E17" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>720</v>
+      </c>
+      <c r="B18" t="s">
+        <v>740</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="D18" t="s">
+        <v>780</v>
+      </c>
+      <c r="E18" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>721</v>
       </c>
-      <c r="D7" t="s">
-        <v>727</v>
-      </c>
-      <c r="E7" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E8" t="s">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E9" t="s">
-        <v>735</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E10" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E11" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35"/>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35"/>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35"/>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35"/>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35"/>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35"/>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35"/>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35"/>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35"/>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35"/>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35"/>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35"/>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35"/>
+      <c r="B19" t="s">
+        <v>741</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>761</v>
+      </c>
+      <c r="D19" t="s">
+        <v>781</v>
+      </c>
+      <c r="E19" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>722</v>
+      </c>
+      <c r="B20" t="s">
+        <v>742</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>762</v>
+      </c>
+      <c r="D20" t="s">
+        <v>782</v>
+      </c>
+      <c r="E20" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>723</v>
+      </c>
+      <c r="B21" t="s">
+        <v>743</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>763</v>
+      </c>
+      <c r="D21" t="s">
+        <v>783</v>
+      </c>
+      <c r="E21" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E22" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E23" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E24" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E25" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E26" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E27" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E28" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E29" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E30" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E31" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E32" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E33" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E34" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E35" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E36" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E37" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E38" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E39" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E40" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E41" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35"/>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35"/>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35"/>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35"/>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35"/>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35"/>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="F78" s="3"/>
     </row>

</xml_diff>